<commit_message>
Add Treasury sleeves from Fed H.15 yields; drop FRED/corporates
FRED refuses connections from the build environment, so the Treasury
yields now come straight from the Federal Reserve's H.15 data download
(the same series FRED republishes as DGS1/DGS5/DGS10). The full-history
daily package link is read from the H.15 page on each refresh.

UST_1Y / UST_5Y / UST_10Y: monthly total returns rebuilt from month-end
constant-maturity yields (par bond repriced one month later, plus one
month of coupon), 1962-02 to 2026-09. Checked against published annual
returns: 10-year within ~1pp in most years (Damodaran), 5-year within
1-2pp of SBBI intermediate government in 1982/1994/2008.

Corporate (Moody's Aaa) is left out for now; it is only on FRED.
Bumps the service worker cache so installed apps pick up the new data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtyJ36mjEj9LzVccKuq7PT
</commit_message>
<xml_diff>
--- a/data/processed/stats.xlsx
+++ b/data/processed/stats.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="86">
   <si>
     <t>note</t>
   </si>
@@ -89,6 +89,9 @@
     <t>Emerging_Markets_6_Portfolios_ME_BE-ME_CSV.zip</t>
   </si>
   <si>
+    <t>Federal Reserve H.15 (daily Treasury CMT)</t>
+  </si>
+  <si>
     <t>F-F_Research_Data_Factors.csv</t>
   </si>
   <si>
@@ -107,16 +110,28 @@
     <t>Emerging_Markets_6_Portfolios_ME_BE-ME.csv</t>
   </si>
   <si>
+    <t>H15_treasury_constant_maturity_daily.csv</t>
+  </si>
+  <si>
     <t>This file was created using the 202609 CRSP database.</t>
   </si>
   <si>
     <t>This file was created using the 202609 Bloomberg database. It contains</t>
   </si>
   <si>
+    <t>1962-01-02 to 2026-10-28</t>
+  </si>
+  <si>
     <t>202609</t>
   </si>
   <si>
-    <t>2026-10-30T00:48:01</t>
+    <t>20261028</t>
+  </si>
+  <si>
+    <t>2026-10-30T01:32:05</t>
+  </si>
+  <si>
+    <t>2026-10-30T01:32:06</t>
   </si>
   <si>
     <t>start</t>
@@ -188,6 +203,15 @@
     <t>Cash</t>
   </si>
   <si>
+    <t>UST_1Y</t>
+  </si>
+  <si>
+    <t>UST_5Y</t>
+  </si>
+  <si>
+    <t>UST_10Y</t>
+  </si>
+  <si>
     <t>1926-07</t>
   </si>
   <si>
@@ -198,6 +222,9 @@
   </si>
   <si>
     <t>1989-07</t>
+  </si>
+  <si>
+    <t>1962-02</t>
   </si>
   <si>
     <t>2026-09</t>
@@ -691,21 +718,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B1" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B2">
         <v>99</v>
@@ -719,7 +746,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B3">
         <v>99</v>
@@ -733,7 +760,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B4">
         <v>99</v>
@@ -747,7 +774,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B5">
         <v>99</v>
@@ -761,7 +788,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B6">
         <v>62</v>
@@ -775,7 +802,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B7">
         <v>62</v>
@@ -789,7 +816,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B8">
         <v>35</v>
@@ -803,7 +830,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B9">
         <v>35</v>
@@ -817,7 +844,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B10">
         <v>36</v>
@@ -831,7 +858,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -862,19 +889,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -918,7 +945,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -948,16 +975,16 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -965,16 +992,16 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -982,16 +1009,16 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -999,16 +1026,16 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1016,16 +1043,16 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D6" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1033,16 +1060,33 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
         <v>28</v>
       </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" t="s">
-        <v>30</v>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1052,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -1066,31 +1110,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1098,13 +1142,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D2">
         <v>1203</v>
@@ -1127,13 +1171,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>1203</v>
@@ -1156,13 +1200,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D4">
         <v>1203</v>
@@ -1185,13 +1229,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D5">
         <v>1203</v>
@@ -1214,13 +1258,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D6">
         <v>1203</v>
@@ -1243,13 +1287,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D7">
         <v>759</v>
@@ -1272,13 +1316,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>759</v>
@@ -1301,13 +1345,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D9">
         <v>435</v>
@@ -1330,13 +1374,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D10">
         <v>435</v>
@@ -1359,13 +1403,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D11">
         <v>435</v>
@@ -1388,13 +1432,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D12">
         <v>447</v>
@@ -1417,13 +1461,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D13">
         <v>447</v>
@@ -1446,13 +1490,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D14">
         <v>447</v>
@@ -1475,13 +1519,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D15">
         <v>1203</v>
@@ -1497,6 +1541,93 @@
       </c>
       <c r="I15" s="1">
         <v>-0.0005000999779984916</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16">
+        <v>776</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.04965026048338661</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.01730225600848117</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.4038664843369107</v>
+      </c>
+      <c r="H16" s="1">
+        <v>-0.02288705888851483</v>
+      </c>
+      <c r="I16" s="1">
+        <v>-0.02227681545763738</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17">
+        <v>776</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.05482375892730773</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.05310849875295689</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.2251862498175984</v>
+      </c>
+      <c r="H17" s="1">
+        <v>-0.1461807592457053</v>
+      </c>
+      <c r="I17" s="1">
+        <v>-0.1143645431823892</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18">
+        <v>776</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.05689591091979174</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.07799539053849196</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.1975971028901461</v>
+      </c>
+      <c r="H18" s="1">
+        <v>-0.2609225927601962</v>
+      </c>
+      <c r="I18" s="1">
+        <v>-0.1791690462697122</v>
       </c>
     </row>
   </sheetData>
@@ -1506,7 +1637,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -1520,31 +1651,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1552,13 +1683,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D2">
         <v>441</v>
@@ -1581,13 +1712,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>441</v>
@@ -1610,13 +1741,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D4">
         <v>441</v>
@@ -1639,13 +1770,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D5">
         <v>441</v>
@@ -1668,13 +1799,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D6">
         <v>441</v>
@@ -1697,13 +1828,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D7">
         <v>441</v>
@@ -1726,13 +1857,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>441</v>
@@ -1755,37 +1886,37 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="J10" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="J11" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D12">
         <v>441</v>
@@ -1808,13 +1939,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D13">
         <v>441</v>
@@ -1837,13 +1968,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D14">
         <v>441</v>
@@ -1866,13 +1997,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D15">
         <v>441</v>
@@ -1888,6 +2019,93 @@
       </c>
       <c r="I15" s="1">
         <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16">
+        <v>441</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.03142218742841441</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.009947156021953446</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.6009519777131356</v>
+      </c>
+      <c r="H16" s="1">
+        <v>-0.02288705888851483</v>
+      </c>
+      <c r="I16" s="1">
+        <v>-0.02227681545763738</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17">
+        <v>441</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.04105866038938299</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.04346222543718948</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.3340872508230641</v>
+      </c>
+      <c r="H17" s="1">
+        <v>-0.1461807592457053</v>
+      </c>
+      <c r="I17" s="1">
+        <v>-0.1143645431823892</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18">
+        <v>441</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.04749700885783747</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.07353552343305854</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.3033165828654143</v>
+      </c>
+      <c r="H18" s="1">
+        <v>-0.2609225927601962</v>
+      </c>
+      <c r="I18" s="1">
+        <v>-0.1791690462697122</v>
       </c>
     </row>
   </sheetData>
@@ -1897,7 +2115,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -1911,31 +2129,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1943,13 +2161,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D2">
         <v>321</v>
@@ -1972,13 +2190,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>321</v>
@@ -2001,13 +2219,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D4">
         <v>321</v>
@@ -2030,13 +2248,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D5">
         <v>321</v>
@@ -2059,13 +2277,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D6">
         <v>321</v>
@@ -2088,13 +2306,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D7">
         <v>321</v>
@@ -2117,13 +2335,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>321</v>
@@ -2146,13 +2364,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D9">
         <v>321</v>
@@ -2175,13 +2393,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D10">
         <v>321</v>
@@ -2204,13 +2422,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D11">
         <v>321</v>
@@ -2233,13 +2451,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D12">
         <v>321</v>
@@ -2262,13 +2480,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C13" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D13">
         <v>321</v>
@@ -2291,13 +2509,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D14">
         <v>321</v>
@@ -2320,13 +2538,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D15">
         <v>321</v>
@@ -2342,6 +2560,93 @@
       </c>
       <c r="I15" s="1">
         <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16">
+        <v>321</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.0221272062542095</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.008958685194048572</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.4500841368265734</v>
+      </c>
+      <c r="H16" s="1">
+        <v>-0.02288705888851505</v>
+      </c>
+      <c r="I16" s="1">
+        <v>-0.02227681545763738</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17">
+        <v>321</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.02998234075676631</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.04321707074845944</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.2677816092207557</v>
+      </c>
+      <c r="H17" s="1">
+        <v>-0.1461807592457053</v>
+      </c>
+      <c r="I17" s="1">
+        <v>-0.1143645431823892</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C18" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18">
+        <v>321</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.03598525831433008</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.07541449014476291</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.2546539766173046</v>
+      </c>
+      <c r="H18" s="1">
+        <v>-0.260922592760196</v>
+      </c>
+      <c r="I18" s="1">
+        <v>-0.1791690462697122</v>
       </c>
     </row>
   </sheetData>
@@ -2351,7 +2656,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -2365,31 +2670,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -2397,13 +2702,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D2">
         <v>120</v>
@@ -2426,13 +2731,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D3">
         <v>120</v>
@@ -2455,13 +2760,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D4">
         <v>120</v>
@@ -2484,13 +2789,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D5">
         <v>120</v>
@@ -2513,13 +2818,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D6">
         <v>120</v>
@@ -2542,13 +2847,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D7">
         <v>120</v>
@@ -2571,13 +2876,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D8">
         <v>120</v>
@@ -2600,13 +2905,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D9">
         <v>120</v>
@@ -2629,13 +2934,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D10">
         <v>120</v>
@@ -2658,13 +2963,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D11">
         <v>120</v>
@@ -2687,13 +2992,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D12">
         <v>120</v>
@@ -2716,13 +3021,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D13">
         <v>120</v>
@@ -2745,13 +3050,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D14">
         <v>120</v>
@@ -2774,13 +3079,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="D15">
         <v>120</v>
@@ -2796,6 +3101,93 @@
       </c>
       <c r="I15" s="1">
         <v>9.999999999998899E-05</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16">
+        <v>120</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.02063610788471548</v>
+      </c>
+      <c r="F16" s="1">
+        <v>0.008762179625003388</v>
+      </c>
+      <c r="G16" s="2">
+        <v>-0.06819031746378371</v>
+      </c>
+      <c r="H16" s="1">
+        <v>-0.02288705888851539</v>
+      </c>
+      <c r="I16" s="1">
+        <v>-0.02227681545763738</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17">
+        <v>120</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.01488225577470015</v>
+      </c>
+      <c r="F17" s="1">
+        <v>0.04137815442333979</v>
+      </c>
+      <c r="G17" s="2">
+        <v>-0.1294236608592681</v>
+      </c>
+      <c r="H17" s="1">
+        <v>-0.1461807592457049</v>
+      </c>
+      <c r="I17" s="1">
+        <v>-0.1143645431823892</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18">
+        <v>120</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.009522461450945707</v>
+      </c>
+      <c r="F18" s="1">
+        <v>0.07228671494409303</v>
+      </c>
+      <c r="G18" s="2">
+        <v>-0.1227193097409438</v>
+      </c>
+      <c r="H18" s="1">
+        <v>-0.2609225927601965</v>
+      </c>
+      <c r="I18" s="1">
+        <v>-0.1791690462697122</v>
       </c>
     </row>
   </sheetData>
@@ -2805,7 +3197,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -2818,59 +3210,68 @@
     <col min="9" max="10" width="20.7109375" style="2" customWidth="1"/>
     <col min="11" max="11" width="16.7109375" style="2" customWidth="1"/>
     <col min="12" max="13" width="15.7109375" style="2" customWidth="1"/>
-    <col min="14" max="15" width="12.7109375" style="2" customWidth="1"/>
+    <col min="14" max="18" width="12.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
+      <c r="A2" t="s">
         <v>45</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
-      <c r="A2" t="s">
-        <v>40</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -2914,10 +3315,19 @@
       <c r="O2" s="2">
         <v>0.008720575418330557</v>
       </c>
-    </row>
-    <row r="3" spans="1:15">
+      <c r="P2" s="2">
+        <v>-0.04506667671579052</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>-0.09296776454437576</v>
+      </c>
+      <c r="R2" s="2">
+        <v>-0.06844342659119444</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B3" s="2">
         <v>0.8084723245525287</v>
@@ -2961,10 +3371,19 @@
       <c r="O3" s="2">
         <v>-0.02824889606400737</v>
       </c>
-    </row>
-    <row r="4" spans="1:15">
+      <c r="P3" s="2">
+        <v>-0.08341305607916655</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>-0.1669728157126054</v>
+      </c>
+      <c r="R3" s="2">
+        <v>-0.1530995276764361</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B4" s="2">
         <v>0.8453565887860622</v>
@@ -3008,10 +3427,19 @@
       <c r="O4" s="2">
         <v>-0.03719089081106493</v>
       </c>
-    </row>
-    <row r="5" spans="1:15">
+      <c r="P4" s="2">
+        <v>-0.09814503936050406</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>-0.1618658671180353</v>
+      </c>
+      <c r="R4" s="2">
+        <v>-0.1286849343882467</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B5" s="2">
         <v>0.8427478229847296</v>
@@ -3055,10 +3483,19 @@
       <c r="O5" s="2">
         <v>0.03408876177247213</v>
       </c>
-    </row>
-    <row r="6" spans="1:15">
+      <c r="P5" s="2">
+        <v>-0.04266035602041702</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>-0.1331638473484328</v>
+      </c>
+      <c r="R5" s="2">
+        <v>-0.1282930343377397</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B6" s="2">
         <v>0.9722190415305743</v>
@@ -3102,10 +3539,19 @@
       <c r="O6" s="2">
         <v>0.01855625776085682</v>
       </c>
-    </row>
-    <row r="7" spans="1:15">
+      <c r="P6" s="2">
+        <v>-0.02456960704491969</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>-0.05024814655886989</v>
+      </c>
+      <c r="R6" s="2">
+        <v>-0.02164763978431109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B7" s="2">
         <v>0.853257488679916</v>
@@ -3149,10 +3595,19 @@
       <c r="O7" s="2">
         <v>-0.03372260379160047</v>
       </c>
-    </row>
-    <row r="8" spans="1:15">
+      <c r="P7" s="2">
+        <v>-0.0987636496596019</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>-0.1569293347194135</v>
+      </c>
+      <c r="R7" s="2">
+        <v>-0.1419150028229105</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" s="2">
         <v>0.8369340000236228</v>
@@ -3196,10 +3651,19 @@
       <c r="O8" s="2">
         <v>-0.03399474920195936</v>
       </c>
-    </row>
-    <row r="9" spans="1:15">
+      <c r="P8" s="2">
+        <v>-0.09187391203733189</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>-0.1688919112178923</v>
+      </c>
+      <c r="R8" s="2">
+        <v>-0.1382991339059669</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2">
         <v>0.6226168068197092</v>
@@ -3243,10 +3707,19 @@
       <c r="O9" s="2">
         <v>-0.05951069382568925</v>
       </c>
-    </row>
-    <row r="10" spans="1:15">
+      <c r="P9" s="2">
+        <v>-0.0920500071833109</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>-0.0631135836438298</v>
+      </c>
+      <c r="R9" s="2">
+        <v>-0.06846292883645531</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B10" s="2">
         <v>0.7124647204721374</v>
@@ -3290,10 +3763,19 @@
       <c r="O10" s="2">
         <v>-0.003678721405237023</v>
       </c>
-    </row>
-    <row r="11" spans="1:15">
+      <c r="P10" s="2">
+        <v>-0.07642551925864281</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>-0.1238126821986896</v>
+      </c>
+      <c r="R10" s="2">
+        <v>-0.1423558442270655</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B11" s="2">
         <v>0.7658313815373569</v>
@@ -3337,10 +3819,19 @@
       <c r="O11" s="2">
         <v>-0.02020794712335095</v>
       </c>
-    </row>
-    <row r="12" spans="1:15">
+      <c r="P11" s="2">
+        <v>-0.05876270085485161</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>-0.04906326386447808</v>
+      </c>
+      <c r="R11" s="2">
+        <v>-0.05280389386797559</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B12" s="2">
         <v>0.6018775544729295</v>
@@ -3384,10 +3875,19 @@
       <c r="O12" s="2">
         <v>-0.04736336177182777</v>
       </c>
-    </row>
-    <row r="13" spans="1:15">
+      <c r="P12" s="2">
+        <v>-0.1480923084546124</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>-0.1752914157207034</v>
+      </c>
+      <c r="R12" s="2">
+        <v>-0.1568476382277995</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2">
         <v>0.6774842229672553</v>
@@ -3431,10 +3931,19 @@
       <c r="O13" s="2">
         <v>-0.03577601559653747</v>
       </c>
-    </row>
-    <row r="14" spans="1:15">
+      <c r="P13" s="2">
+        <v>-0.09856543192274309</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>-0.132987825107985</v>
+      </c>
+      <c r="R13" s="2">
+        <v>-0.1348365253180284</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2">
         <v>0.7107951348280582</v>
@@ -3478,10 +3987,19 @@
       <c r="O14" s="2">
         <v>-0.03205137004009748</v>
       </c>
-    </row>
-    <row r="15" spans="1:15">
+      <c r="P14" s="2">
+        <v>-0.09573142285310315</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>-0.1230057814950013</v>
+      </c>
+      <c r="R14" s="2">
+        <v>-0.1128898733858209</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2">
         <v>0.008720575418330557</v>
@@ -3523,6 +4041,183 @@
         <v>-0.03205137004009748</v>
       </c>
       <c r="O15" s="2">
+        <v>1</v>
+      </c>
+      <c r="P15" s="2">
+        <v>0.7395611554326234</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>0.2022336728240978</v>
+      </c>
+      <c r="R15" s="2">
+        <v>0.1085441373330153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18">
+      <c r="A16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="2">
+        <v>-0.04506667671579052</v>
+      </c>
+      <c r="C16" s="2">
+        <v>-0.08341305607916655</v>
+      </c>
+      <c r="D16" s="2">
+        <v>-0.09814503936050406</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-0.04266035602041702</v>
+      </c>
+      <c r="F16" s="2">
+        <v>-0.02456960704491969</v>
+      </c>
+      <c r="G16" s="2">
+        <v>-0.0987636496596019</v>
+      </c>
+      <c r="H16" s="2">
+        <v>-0.09187391203733189</v>
+      </c>
+      <c r="I16" s="2">
+        <v>-0.0920500071833109</v>
+      </c>
+      <c r="J16" s="2">
+        <v>-0.07642551925864281</v>
+      </c>
+      <c r="K16" s="2">
+        <v>-0.05876270085485161</v>
+      </c>
+      <c r="L16" s="2">
+        <v>-0.1480923084546124</v>
+      </c>
+      <c r="M16" s="2">
+        <v>-0.09856543192274309</v>
+      </c>
+      <c r="N16" s="2">
+        <v>-0.09573142285310315</v>
+      </c>
+      <c r="O16" s="2">
+        <v>0.7395611554326234</v>
+      </c>
+      <c r="P16" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>0.6510818536523723</v>
+      </c>
+      <c r="R16" s="2">
+        <v>0.5104391547759107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18">
+      <c r="A17" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="2">
+        <v>-0.09296776454437576</v>
+      </c>
+      <c r="C17" s="2">
+        <v>-0.1669728157126054</v>
+      </c>
+      <c r="D17" s="2">
+        <v>-0.1618658671180353</v>
+      </c>
+      <c r="E17" s="2">
+        <v>-0.1331638473484328</v>
+      </c>
+      <c r="F17" s="2">
+        <v>-0.05024814655886989</v>
+      </c>
+      <c r="G17" s="2">
+        <v>-0.1569293347194135</v>
+      </c>
+      <c r="H17" s="2">
+        <v>-0.1688919112178923</v>
+      </c>
+      <c r="I17" s="2">
+        <v>-0.0631135836438298</v>
+      </c>
+      <c r="J17" s="2">
+        <v>-0.1238126821986896</v>
+      </c>
+      <c r="K17" s="2">
+        <v>-0.04906326386447808</v>
+      </c>
+      <c r="L17" s="2">
+        <v>-0.1752914157207034</v>
+      </c>
+      <c r="M17" s="2">
+        <v>-0.132987825107985</v>
+      </c>
+      <c r="N17" s="2">
+        <v>-0.1230057814950013</v>
+      </c>
+      <c r="O17" s="2">
+        <v>0.2022336728240978</v>
+      </c>
+      <c r="P17" s="2">
+        <v>0.6510818536523723</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>1</v>
+      </c>
+      <c r="R17" s="2">
+        <v>0.9400664376200487</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18">
+      <c r="A18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="2">
+        <v>-0.06844342659119444</v>
+      </c>
+      <c r="C18" s="2">
+        <v>-0.1530995276764361</v>
+      </c>
+      <c r="D18" s="2">
+        <v>-0.1286849343882467</v>
+      </c>
+      <c r="E18" s="2">
+        <v>-0.1282930343377397</v>
+      </c>
+      <c r="F18" s="2">
+        <v>-0.02164763978431109</v>
+      </c>
+      <c r="G18" s="2">
+        <v>-0.1419150028229105</v>
+      </c>
+      <c r="H18" s="2">
+        <v>-0.1382991339059669</v>
+      </c>
+      <c r="I18" s="2">
+        <v>-0.06846292883645531</v>
+      </c>
+      <c r="J18" s="2">
+        <v>-0.1423558442270655</v>
+      </c>
+      <c r="K18" s="2">
+        <v>-0.05280389386797559</v>
+      </c>
+      <c r="L18" s="2">
+        <v>-0.1568476382277995</v>
+      </c>
+      <c r="M18" s="2">
+        <v>-0.1348365253180284</v>
+      </c>
+      <c r="N18" s="2">
+        <v>-0.1128898733858209</v>
+      </c>
+      <c r="O18" s="2">
+        <v>0.1085441373330153</v>
+      </c>
+      <c r="P18" s="2">
+        <v>0.5104391547759107</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>0.9400664376200487</v>
+      </c>
+      <c r="R18" s="2">
         <v>1</v>
       </c>
     </row>
@@ -3533,7 +4228,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:R100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -3546,57 +4241,66 @@
     <col min="9" max="10" width="20.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="16.7109375" style="1" customWidth="1"/>
     <col min="12" max="13" width="15.7109375" style="1" customWidth="1"/>
-    <col min="14" max="15" width="12.7109375" style="1" customWidth="1"/>
+    <col min="14" max="18" width="12.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15">
+        <v>58</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2">
         <v>1927</v>
       </c>
@@ -3619,7 +4323,7 @@
         <v>0.03134078242998228</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:18">
       <c r="A3">
         <v>1928</v>
       </c>
@@ -3642,7 +4346,7 @@
         <v>0.03535597953433101</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:18">
       <c r="A4">
         <v>1929</v>
       </c>
@@ -3665,7 +4369,7 @@
         <v>0.047397677669484</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:18">
       <c r="A5">
         <v>1930</v>
       </c>
@@ -3688,7 +4392,7 @@
         <v>0.02426179995774591</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:18">
       <c r="A6">
         <v>1931</v>
       </c>
@@ -3711,7 +4415,7 @@
         <v>0.01085244021158438</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:18">
       <c r="A7">
         <v>1932</v>
       </c>
@@ -3734,7 +4438,7 @@
         <v>0.009436727769233766</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:18">
       <c r="A8">
         <v>1933</v>
       </c>
@@ -3757,7 +4461,7 @@
         <v>0.003003642310775989</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:18">
       <c r="A9">
         <v>1934</v>
       </c>
@@ -3780,7 +4484,7 @@
         <v>0.001801410644192591</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:18">
       <c r="A10">
         <v>1935</v>
       </c>
@@ -3803,7 +4507,7 @@
         <v>0.001400890340086836</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:18">
       <c r="A11">
         <v>1936</v>
       </c>
@@ -3826,7 +4530,7 @@
         <v>0.00180145069021509</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:18">
       <c r="A12">
         <v>1937</v>
       </c>
@@ -3849,7 +4553,7 @@
         <v>0.002903722791360863</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:18">
       <c r="A13">
         <v>1938</v>
       </c>
@@ -3872,7 +4576,7 @@
         <v>-0.0004001399919977278</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:18">
       <c r="A14">
         <v>1939</v>
       </c>
@@ -3895,7 +4599,7 @@
         <v>9.996999700012665E-05</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:18">
       <c r="A15">
         <v>1940</v>
       </c>
@@ -3918,7 +4622,7 @@
         <v>-0.0002000099979999614</v>
       </c>
     </row>
-    <row r="16" spans="1:15">
+    <row r="16" spans="1:18">
       <c r="A16">
         <v>1941</v>
       </c>
@@ -4309,7 +5013,7 @@
         <v>0.03154688516655124</v>
       </c>
     </row>
-    <row r="33" spans="1:15">
+    <row r="33" spans="1:18">
       <c r="A33">
         <v>1958</v>
       </c>
@@ -4332,7 +5036,7 @@
         <v>0.01530313907384762</v>
       </c>
     </row>
-    <row r="34" spans="1:15">
+    <row r="34" spans="1:18">
       <c r="A34">
         <v>1959</v>
       </c>
@@ -4355,7 +5059,7 @@
         <v>0.02969530696561828</v>
       </c>
     </row>
-    <row r="35" spans="1:15">
+    <row r="35" spans="1:18">
       <c r="A35">
         <v>1960</v>
       </c>
@@ -4378,7 +5082,7 @@
         <v>0.02671854421052489</v>
       </c>
     </row>
-    <row r="36" spans="1:15">
+    <row r="36" spans="1:18">
       <c r="A36">
         <v>1961</v>
       </c>
@@ -4401,7 +5105,7 @@
         <v>0.02120304919998262</v>
       </c>
     </row>
-    <row r="37" spans="1:15">
+    <row r="37" spans="1:18">
       <c r="A37">
         <v>1962</v>
       </c>
@@ -4424,7 +5128,7 @@
         <v>0.02733631130815972</v>
       </c>
     </row>
-    <row r="38" spans="1:15">
+    <row r="38" spans="1:18">
       <c r="A38">
         <v>1963</v>
       </c>
@@ -4446,8 +5150,17 @@
       <c r="O38" s="1">
         <v>0.03113540823864613</v>
       </c>
-    </row>
-    <row r="39" spans="1:15">
+      <c r="P38" s="1">
+        <v>0.02649591940279516</v>
+      </c>
+      <c r="Q38" s="1">
+        <v>0.01596314470176896</v>
+      </c>
+      <c r="R38" s="1">
+        <v>0.01642398815500656</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18">
       <c r="A39">
         <v>1964</v>
       </c>
@@ -4475,8 +5188,17 @@
       <c r="O39" s="1">
         <v>0.03525706968952402</v>
       </c>
-    </row>
-    <row r="40" spans="1:15">
+      <c r="P39" s="1">
+        <v>0.03770780558237052</v>
+      </c>
+      <c r="Q39" s="1">
+        <v>0.03872754652216259</v>
+      </c>
+      <c r="R39" s="1">
+        <v>0.03678913482557777</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18">
       <c r="A40">
         <v>1965</v>
       </c>
@@ -4504,8 +5226,17 @@
       <c r="O40" s="1">
         <v>0.03918636823954325</v>
       </c>
-    </row>
-    <row r="41" spans="1:15">
+      <c r="P40" s="1">
+        <v>0.03299650491109252</v>
+      </c>
+      <c r="Q40" s="1">
+        <v>0.008969981844349606</v>
+      </c>
+      <c r="R40" s="1">
+        <v>0.007672018178028539</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18">
       <c r="A41">
         <v>1966</v>
       </c>
@@ -4533,8 +5264,17 @@
       <c r="O41" s="1">
         <v>0.04750339219432975</v>
       </c>
-    </row>
-    <row r="42" spans="1:15">
+      <c r="P41" s="1">
+        <v>0.05288528831294026</v>
+      </c>
+      <c r="Q41" s="1">
+        <v>0.05579973864792831</v>
+      </c>
+      <c r="R41" s="1">
+        <v>0.05034466578234298</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18">
       <c r="A42">
         <v>1967</v>
       </c>
@@ -4562,8 +5302,17 @@
       <c r="O42" s="1">
         <v>0.04208973213020073</v>
       </c>
-    </row>
-    <row r="43" spans="1:15">
+      <c r="P42" s="1">
+        <v>0.04279475219790552</v>
+      </c>
+      <c r="Q42" s="1">
+        <v>0.008483485773714827</v>
+      </c>
+      <c r="R42" s="1">
+        <v>-0.03104652906435323</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18">
       <c r="A43">
         <v>1968</v>
       </c>
@@ -4591,8 +5340,17 @@
       <c r="O43" s="1">
         <v>0.05220876393709961</v>
       </c>
-    </row>
-    <row r="44" spans="1:15">
+      <c r="P43" s="1">
+        <v>0.05162383496393685</v>
+      </c>
+      <c r="Q43" s="1">
+        <v>0.03399151180147597</v>
+      </c>
+      <c r="R43" s="1">
+        <v>0.02197897736253074</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18">
       <c r="A44">
         <v>1969</v>
       </c>
@@ -4620,8 +5378,17 @@
       <c r="O44" s="1">
         <v>0.06569703672500227</v>
       </c>
-    </row>
-    <row r="45" spans="1:15">
+      <c r="P44" s="1">
+        <v>0.05595602558940849</v>
+      </c>
+      <c r="Q44" s="1">
+        <v>-0.008535237276688701</v>
+      </c>
+      <c r="R44" s="1">
+        <v>-0.05436642343112508</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18">
       <c r="A45">
         <v>1970</v>
       </c>
@@ -4649,8 +5416,17 @@
       <c r="O45" s="1">
         <v>0.06516705987919003</v>
       </c>
-    </row>
-    <row r="46" spans="1:15">
+      <c r="P45" s="1">
+        <v>0.1051939769271852</v>
+      </c>
+      <c r="Q45" s="1">
+        <v>0.1791787278820318</v>
+      </c>
+      <c r="R45" s="1">
+        <v>0.1830540341427311</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18">
       <c r="A46">
         <v>1971</v>
       </c>
@@ -4678,8 +5454,17 @@
       <c r="O46" s="1">
         <v>0.04385608936775598</v>
       </c>
-    </row>
-    <row r="47" spans="1:15">
+      <c r="P46" s="1">
+        <v>0.05474072938020447</v>
+      </c>
+      <c r="Q46" s="1">
+        <v>0.08232169351177943</v>
+      </c>
+      <c r="R46" s="1">
+        <v>0.1104292187312061</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18">
       <c r="A47">
         <v>1972</v>
       </c>
@@ -4707,8 +5492,17 @@
       <c r="O47" s="1">
         <v>0.03835711405871467</v>
       </c>
-    </row>
-    <row r="48" spans="1:15">
+      <c r="P47" s="1">
+        <v>0.03928793378593487</v>
+      </c>
+      <c r="Q47" s="1">
+        <v>0.02768211514310681</v>
+      </c>
+      <c r="R47" s="1">
+        <v>0.02377857491876068</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18">
       <c r="A48">
         <v>1973</v>
       </c>
@@ -4736,8 +5530,17 @@
       <c r="O48" s="1">
         <v>0.06940964906929548</v>
       </c>
-    </row>
-    <row r="49" spans="1:15">
+      <c r="P48" s="1">
+        <v>0.0592423301298568</v>
+      </c>
+      <c r="Q48" s="1">
+        <v>0.0451092556470496</v>
+      </c>
+      <c r="R48" s="1">
+        <v>0.03308110141548481</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18">
       <c r="A49">
         <v>1974</v>
       </c>
@@ -4765,8 +5568,17 @@
       <c r="O49" s="1">
         <v>0.08009299500445022</v>
       </c>
-    </row>
-    <row r="50" spans="1:15">
+      <c r="P49" s="1">
+        <v>0.08519250794841526</v>
+      </c>
+      <c r="Q49" s="1">
+        <v>0.05731689230463521</v>
+      </c>
+      <c r="R49" s="1">
+        <v>0.0406758792986166</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18">
       <c r="A50">
         <v>1975</v>
       </c>
@@ -4794,8 +5606,17 @@
       <c r="O50" s="1">
         <v>0.05798431629002376</v>
       </c>
-    </row>
-    <row r="51" spans="1:15">
+      <c r="P50" s="1">
+        <v>0.08122490760986678</v>
+      </c>
+      <c r="Q50" s="1">
+        <v>0.07369038246157067</v>
+      </c>
+      <c r="R50" s="1">
+        <v>0.05538676072433169</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18">
       <c r="A51">
         <v>1976</v>
       </c>
@@ -4823,8 +5644,17 @@
       <c r="O51" s="1">
         <v>0.05084710391799252</v>
       </c>
-    </row>
-    <row r="52" spans="1:15">
+      <c r="P51" s="1">
+        <v>0.07360447655307789</v>
+      </c>
+      <c r="Q51" s="1">
+        <v>0.1366127078135049</v>
+      </c>
+      <c r="R51" s="1">
+        <v>0.152513866627177</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18">
       <c r="A52">
         <v>1977</v>
       </c>
@@ -4852,8 +5682,17 @@
       <c r="O52" s="1">
         <v>0.05126495522821517</v>
       </c>
-    </row>
-    <row r="53" spans="1:15">
+      <c r="P52" s="1">
+        <v>0.04194278576446542</v>
+      </c>
+      <c r="Q52" s="1">
+        <v>0.01120144432326642</v>
+      </c>
+      <c r="R52" s="1">
+        <v>0.00570142500209192</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18">
       <c r="A53">
         <v>1978</v>
       </c>
@@ -4881,8 +5720,17 @@
       <c r="O53" s="1">
         <v>0.07196501341871353</v>
       </c>
-    </row>
-    <row r="54" spans="1:15">
+      <c r="P53" s="1">
+        <v>0.05251854901170483</v>
+      </c>
+      <c r="Q53" s="1">
+        <v>0.01244082494516974</v>
+      </c>
+      <c r="R53" s="1">
+        <v>-0.00693361814222615</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18">
       <c r="A54">
         <v>1979</v>
       </c>
@@ -4910,8 +5758,17 @@
       <c r="O54" s="1">
         <v>0.1038334430458425</v>
       </c>
-    </row>
-    <row r="55" spans="1:15">
+      <c r="P54" s="1">
+        <v>0.1000858443511792</v>
+      </c>
+      <c r="Q54" s="1">
+        <v>0.05411383013561677</v>
+      </c>
+      <c r="R54" s="1">
+        <v>0.01867664423220239</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18">
       <c r="A55">
         <v>1980</v>
       </c>
@@ -4939,8 +5796,17 @@
       <c r="O55" s="1">
         <v>0.1125873347536877</v>
       </c>
-    </row>
-    <row r="56" spans="1:15">
+      <c r="P55" s="1">
+        <v>0.1075620220535449</v>
+      </c>
+      <c r="Q55" s="1">
+        <v>0.02999612832269682</v>
+      </c>
+      <c r="R55" s="1">
+        <v>-0.01234512314576519</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18">
       <c r="A56">
         <v>1981</v>
       </c>
@@ -4968,8 +5834,17 @@
       <c r="O56" s="1">
         <v>0.1471747478188747</v>
       </c>
-    </row>
-    <row r="57" spans="1:15">
+      <c r="P56" s="1">
+        <v>0.1618748297900527</v>
+      </c>
+      <c r="Q56" s="1">
+        <v>0.09479057826594861</v>
+      </c>
+      <c r="R56" s="1">
+        <v>0.05317831235208814</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18">
       <c r="A57">
         <v>1982</v>
       </c>
@@ -4997,8 +5872,17 @@
       <c r="O57" s="1">
         <v>0.1053450799423241</v>
       </c>
-    </row>
-    <row r="58" spans="1:15">
+      <c r="P57" s="1">
+        <v>0.1771442379756776</v>
+      </c>
+      <c r="Q57" s="1">
+        <v>0.3090957058801094</v>
+      </c>
+      <c r="R57" s="1">
+        <v>0.3944908276934136</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18">
       <c r="A58">
         <v>1983</v>
       </c>
@@ -5026,8 +5910,17 @@
       <c r="O58" s="1">
         <v>0.087957322322191</v>
       </c>
-    </row>
-    <row r="59" spans="1:15">
+      <c r="P58" s="1">
+        <v>0.08637633459558414</v>
+      </c>
+      <c r="Q58" s="1">
+        <v>0.05298500745996915</v>
+      </c>
+      <c r="R58" s="1">
+        <v>0.02338095350910829</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18">
       <c r="A59">
         <v>1984</v>
       </c>
@@ -5055,8 +5948,17 @@
       <c r="O59" s="1">
         <v>0.09837053073148572</v>
       </c>
-    </row>
-    <row r="60" spans="1:15">
+      <c r="P59" s="1">
+        <v>0.1235984462740674</v>
+      </c>
+      <c r="Q59" s="1">
+        <v>0.149908050800257</v>
+      </c>
+      <c r="R59" s="1">
+        <v>0.148664555016591</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18">
       <c r="A60">
         <v>1985</v>
       </c>
@@ -5084,8 +5986,17 @@
       <c r="O60" s="1">
         <v>0.07720290931256968</v>
       </c>
-    </row>
-    <row r="61" spans="1:15">
+      <c r="P60" s="1">
+        <v>0.1037122591522808</v>
+      </c>
+      <c r="Q60" s="1">
+        <v>0.2208820094991095</v>
+      </c>
+      <c r="R60" s="1">
+        <v>0.2975207867461596</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18">
       <c r="A61">
         <v>1986</v>
       </c>
@@ -5113,8 +6024,17 @@
       <c r="O61" s="1">
         <v>0.06157040643142619</v>
       </c>
-    </row>
-    <row r="62" spans="1:15">
+      <c r="P61" s="1">
+        <v>0.08253125611092282</v>
+      </c>
+      <c r="Q61" s="1">
+        <v>0.149991521385427</v>
+      </c>
+      <c r="R61" s="1">
+        <v>0.2127337703791732</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18">
       <c r="A62">
         <v>1987</v>
       </c>
@@ -5142,8 +6062,17 @@
       <c r="O62" s="1">
         <v>0.0547242533511505</v>
       </c>
-    </row>
-    <row r="63" spans="1:15">
+      <c r="P62" s="1">
+        <v>0.05804708868847563</v>
+      </c>
+      <c r="Q62" s="1">
+        <v>0.01643336726600375</v>
+      </c>
+      <c r="R62" s="1">
+        <v>-0.02584594328744705</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18">
       <c r="A63">
         <v>1988</v>
       </c>
@@ -5171,8 +6100,17 @@
       <c r="O63" s="1">
         <v>0.06357536181976098</v>
       </c>
-    </row>
-    <row r="64" spans="1:15">
+      <c r="P63" s="1">
+        <v>0.06032841705049452</v>
+      </c>
+      <c r="Q63" s="1">
+        <v>0.05302374893568063</v>
+      </c>
+      <c r="R63" s="1">
+        <v>0.06913042135692216</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18">
       <c r="A64">
         <v>1989</v>
       </c>
@@ -5200,8 +6138,17 @@
       <c r="O64" s="1">
         <v>0.08375046134037034</v>
       </c>
-    </row>
-    <row r="65" spans="1:15">
+      <c r="P64" s="1">
+        <v>0.101308205218416</v>
+      </c>
+      <c r="Q64" s="1">
+        <v>0.1444321340535573</v>
+      </c>
+      <c r="R64" s="1">
+        <v>0.177924703507784</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18">
       <c r="A65">
         <v>1990</v>
       </c>
@@ -5238,8 +6185,17 @@
       <c r="O65" s="1">
         <v>0.07838118061963439</v>
       </c>
-    </row>
-    <row r="66" spans="1:15">
+      <c r="P65" s="1">
+        <v>0.09100242147911475</v>
+      </c>
+      <c r="Q65" s="1">
+        <v>0.09450938294858524</v>
+      </c>
+      <c r="R65" s="1">
+        <v>0.07706153396391113</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18">
       <c r="A66">
         <v>1991</v>
       </c>
@@ -5285,8 +6241,17 @@
       <c r="O66" s="1">
         <v>0.05598602000744579</v>
       </c>
-    </row>
-    <row r="67" spans="1:15">
+      <c r="P66" s="1">
+        <v>0.08685274878211313</v>
+      </c>
+      <c r="Q66" s="1">
+        <v>0.1565975541786297</v>
+      </c>
+      <c r="R66" s="1">
+        <v>0.1884482920288948</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18">
       <c r="A67">
         <v>1992</v>
       </c>
@@ -5332,8 +6297,17 @@
       <c r="O67" s="1">
         <v>0.03504994804571737</v>
       </c>
-    </row>
-    <row r="68" spans="1:15">
+      <c r="P67" s="1">
+        <v>0.04498275866775092</v>
+      </c>
+      <c r="Q67" s="1">
+        <v>0.058538284073544</v>
+      </c>
+      <c r="R67" s="1">
+        <v>0.07231271909294934</v>
+      </c>
+    </row>
+    <row r="68" spans="1:18">
       <c r="A68">
         <v>1993</v>
       </c>
@@ -5379,8 +6353,17 @@
       <c r="O68" s="1">
         <v>0.02897778178063759</v>
       </c>
-    </row>
-    <row r="69" spans="1:15">
+      <c r="P68" s="1">
+        <v>0.03485402406078197</v>
+      </c>
+      <c r="Q68" s="1">
+        <v>0.09047464372571379</v>
+      </c>
+      <c r="R68" s="1">
+        <v>0.1293172684390369</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18">
       <c r="A69">
         <v>1994</v>
       </c>
@@ -5426,8 +6409,17 @@
       <c r="O69" s="1">
         <v>0.03908056138318683</v>
       </c>
-    </row>
-    <row r="70" spans="1:15">
+      <c r="P69" s="1">
+        <v>0.02004932216529909</v>
+      </c>
+      <c r="Q69" s="1">
+        <v>-0.04248263935540941</v>
+      </c>
+      <c r="R69" s="1">
+        <v>-0.07113709769976606</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18">
       <c r="A70">
         <v>1995</v>
       </c>
@@ -5473,8 +6465,17 @@
       <c r="O70" s="1">
         <v>0.05598649105330922</v>
       </c>
-    </row>
-    <row r="71" spans="1:15">
+      <c r="P70" s="1">
+        <v>0.08112274640782968</v>
+      </c>
+      <c r="Q70" s="1">
+        <v>0.1798037366119227</v>
+      </c>
+      <c r="R70" s="1">
+        <v>0.2543007391909076</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18">
       <c r="A71">
         <v>1996</v>
       </c>
@@ -5520,8 +6521,17 @@
       <c r="O71" s="1">
         <v>0.05199928578383561</v>
       </c>
-    </row>
-    <row r="72" spans="1:15">
+      <c r="P71" s="1">
+        <v>0.05342858311109766</v>
+      </c>
+      <c r="Q71" s="1">
+        <v>0.0263013390062603</v>
+      </c>
+      <c r="R71" s="1">
+        <v>0.0003716294744005033</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18">
       <c r="A72">
         <v>1997</v>
       </c>
@@ -5567,8 +6577,17 @@
       <c r="O72" s="1">
         <v>0.05252282460020363</v>
       </c>
-    </row>
-    <row r="73" spans="1:15">
+      <c r="P72" s="1">
+        <v>0.05773672602391122</v>
+      </c>
+      <c r="Q72" s="1">
+        <v>0.08635774012010766</v>
+      </c>
+      <c r="R72" s="1">
+        <v>0.119324061307428</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18">
       <c r="A73">
         <v>1998</v>
       </c>
@@ -5614,8 +6633,17 @@
       <c r="O73" s="1">
         <v>0.04854677372756999</v>
       </c>
-    </row>
-    <row r="74" spans="1:15">
+      <c r="P73" s="1">
+        <v>0.06134421488876618</v>
+      </c>
+      <c r="Q73" s="1">
+        <v>0.105931558725012</v>
+      </c>
+      <c r="R73" s="1">
+        <v>0.1457777663984334</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18">
       <c r="A74">
         <v>1999</v>
       </c>
@@ -5661,8 +6689,17 @@
       <c r="O74" s="1">
         <v>0.04687748765610511</v>
       </c>
-    </row>
-    <row r="75" spans="1:15">
+      <c r="P74" s="1">
+        <v>0.03803771776468001</v>
+      </c>
+      <c r="Q74" s="1">
+        <v>-0.02195072677628562</v>
+      </c>
+      <c r="R74" s="1">
+        <v>-0.07747570052046415</v>
+      </c>
+    </row>
+    <row r="75" spans="1:18">
       <c r="A75">
         <v>2000</v>
       </c>
@@ -5708,8 +6745,17 @@
       <c r="O75" s="1">
         <v>0.058827813659585</v>
       </c>
-    </row>
-    <row r="76" spans="1:15">
+      <c r="P75" s="1">
+        <v>0.06947236664925005</v>
+      </c>
+      <c r="Q75" s="1">
+        <v>0.1268673918897096</v>
+      </c>
+      <c r="R75" s="1">
+        <v>0.1720561204383739</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18">
       <c r="A76">
         <v>2001</v>
       </c>
@@ -5755,8 +6801,17 @@
       <c r="O76" s="1">
         <v>0.0382480086493604</v>
       </c>
-    </row>
-    <row r="77" spans="1:15">
+      <c r="P76" s="1">
+        <v>0.06616419441026</v>
+      </c>
+      <c r="Q76" s="1">
+        <v>0.07416337965434461</v>
+      </c>
+      <c r="R76" s="1">
+        <v>0.05400870055352702</v>
+      </c>
+    </row>
+    <row r="77" spans="1:18">
       <c r="A77">
         <v>2002</v>
       </c>
@@ -5802,8 +6857,17 @@
       <c r="O77" s="1">
         <v>0.01632075190748306</v>
       </c>
-    </row>
-    <row r="78" spans="1:15">
+      <c r="P77" s="1">
+        <v>0.02826017875228959</v>
+      </c>
+      <c r="Q77" s="1">
+        <v>0.115320345901061</v>
+      </c>
+      <c r="R77" s="1">
+        <v>0.1537573799214909</v>
+      </c>
+    </row>
+    <row r="78" spans="1:18">
       <c r="A78">
         <v>2003</v>
       </c>
@@ -5849,8 +6913,17 @@
       <c r="O78" s="1">
         <v>0.01024772455565182</v>
       </c>
-    </row>
-    <row r="79" spans="1:15">
+      <c r="P78" s="1">
+        <v>0.0131044294611673</v>
+      </c>
+      <c r="Q78" s="1">
+        <v>0.007176581357773104</v>
+      </c>
+      <c r="R78" s="1">
+        <v>0.001802742887746067</v>
+      </c>
+    </row>
+    <row r="79" spans="1:18">
       <c r="A79">
         <v>2004</v>
       </c>
@@ -5896,8 +6969,17 @@
       <c r="O79" s="1">
         <v>0.01186345410952283</v>
       </c>
-    </row>
-    <row r="80" spans="1:15">
+      <c r="P79" s="1">
+        <v>0.004595313946105906</v>
+      </c>
+      <c r="Q79" s="1">
+        <v>0.01667004821020113</v>
+      </c>
+      <c r="R79" s="1">
+        <v>0.04495887807601018</v>
+      </c>
+    </row>
+    <row r="80" spans="1:18">
       <c r="A80">
         <v>2005</v>
       </c>
@@ -5943,8 +7025,17 @@
       <c r="O80" s="1">
         <v>0.02979774263277912</v>
       </c>
-    </row>
-    <row r="81" spans="1:15">
+      <c r="P80" s="1">
+        <v>0.02112337484194349</v>
+      </c>
+      <c r="Q80" s="1">
+        <v>0.007899658751238325</v>
+      </c>
+      <c r="R80" s="1">
+        <v>0.03024006626692799</v>
+      </c>
+    </row>
+    <row r="81" spans="1:18">
       <c r="A81">
         <v>2006</v>
       </c>
@@ -5990,8 +7081,17 @@
       <c r="O81" s="1">
         <v>0.04812968129714923</v>
       </c>
-    </row>
-    <row r="82" spans="1:15">
+      <c r="P81" s="1">
+        <v>0.04424575183298551</v>
+      </c>
+      <c r="Q81" s="1">
+        <v>0.03219517757581603</v>
+      </c>
+      <c r="R81" s="1">
+        <v>0.02208834601897269</v>
+      </c>
+    </row>
+    <row r="82" spans="1:18">
       <c r="A82">
         <v>2007</v>
       </c>
@@ -6037,8 +7137,17 @@
       <c r="O82" s="1">
         <v>0.04666772011205489</v>
       </c>
-    </row>
-    <row r="83" spans="1:15">
+      <c r="P82" s="1">
+        <v>0.06240340709126069</v>
+      </c>
+      <c r="Q82" s="1">
+        <v>0.1041722875618969</v>
+      </c>
+      <c r="R82" s="1">
+        <v>0.1038548518626017</v>
+      </c>
+    </row>
+    <row r="83" spans="1:18">
       <c r="A83">
         <v>2008</v>
       </c>
@@ -6084,8 +7193,17 @@
       <c r="O83" s="1">
         <v>0.015912653124452</v>
       </c>
-    </row>
-    <row r="84" spans="1:15">
+      <c r="P83" s="1">
+        <v>0.04759256874224183</v>
+      </c>
+      <c r="Q83" s="1">
+        <v>0.1224460045419693</v>
+      </c>
+      <c r="R83" s="1">
+        <v>0.204080667005339</v>
+      </c>
+    </row>
+    <row r="84" spans="1:18">
       <c r="A84">
         <v>2009</v>
       </c>
@@ -6131,8 +7249,17 @@
       <c r="O84" s="1">
         <v>0.0009003500770103923</v>
       </c>
-    </row>
-    <row r="85" spans="1:15">
+      <c r="P84" s="1">
+        <v>0.003790423532506804</v>
+      </c>
+      <c r="Q84" s="1">
+        <v>-0.03163333855445394</v>
+      </c>
+      <c r="R84" s="1">
+        <v>-0.1008181941956301</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18">
       <c r="A85">
         <v>2010</v>
       </c>
@@ -6178,8 +7305,17 @@
       <c r="O85" s="1">
         <v>0.001000450120020702</v>
       </c>
-    </row>
-    <row r="86" spans="1:15">
+      <c r="P85" s="1">
+        <v>0.004880790188244166</v>
+      </c>
+      <c r="Q85" s="1">
+        <v>0.05135132516523844</v>
+      </c>
+      <c r="R85" s="1">
+        <v>0.07888906402230811</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18">
       <c r="A86">
         <v>2011</v>
       </c>
@@ -6225,8 +7361,17 @@
       <c r="O86" s="1">
         <v>0.0004000600039999469</v>
       </c>
-    </row>
-    <row r="87" spans="1:15">
+      <c r="P86" s="1">
+        <v>0.003528202413766612</v>
+      </c>
+      <c r="Q86" s="1">
+        <v>0.07390112555592965</v>
+      </c>
+      <c r="R86" s="1">
+        <v>0.1614210300898378</v>
+      </c>
+    </row>
+    <row r="87" spans="1:18">
       <c r="A87">
         <v>2012</v>
       </c>
@@ -6272,8 +7417,17 @@
       <c r="O87" s="1">
         <v>0.0006001500200012444</v>
       </c>
-    </row>
-    <row r="88" spans="1:15">
+      <c r="P87" s="1">
+        <v>0.001351096590052281</v>
+      </c>
+      <c r="Q87" s="1">
+        <v>0.0126010382654218</v>
+      </c>
+      <c r="R87" s="1">
+        <v>0.02725188547113544</v>
+      </c>
+    </row>
+    <row r="88" spans="1:18">
       <c r="A88">
         <v>2013</v>
       </c>
@@ -6319,8 +7473,17 @@
       <c r="O88" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:15">
+      <c r="P88" s="1">
+        <v>0.001600794618772827</v>
+      </c>
+      <c r="Q88" s="1">
+        <v>-0.03740251669898598</v>
+      </c>
+      <c r="R88" s="1">
+        <v>-0.08492203504839635</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18">
       <c r="A89">
         <v>2014</v>
       </c>
@@ -6366,8 +7529,17 @@
       <c r="O89" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:15">
+      <c r="P89" s="1">
+        <v>5.133403511070611E-05</v>
+      </c>
+      <c r="Q89" s="1">
+        <v>0.02110419199381353</v>
+      </c>
+      <c r="R89" s="1">
+        <v>0.105742139151922</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18">
       <c r="A90">
         <v>2015</v>
       </c>
@@ -6413,8 +7585,17 @@
       <c r="O90" s="1">
         <v>9.999999999998899E-05</v>
       </c>
-    </row>
-    <row r="91" spans="1:15">
+      <c r="P90" s="1">
+        <v>-0.0006630578187433178</v>
+      </c>
+      <c r="Q90" s="1">
+        <v>0.009537520381164954</v>
+      </c>
+      <c r="R90" s="1">
+        <v>0.01130586094328456</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18">
       <c r="A91">
         <v>2016</v>
       </c>
@@ -6460,8 +7641,17 @@
       <c r="O91" s="1">
         <v>0.002102001142435306</v>
       </c>
-    </row>
-    <row r="92" spans="1:15">
+      <c r="P91" s="1">
+        <v>0.004165763558126701</v>
+      </c>
+      <c r="Q91" s="1">
+        <v>0.004783803516075436</v>
+      </c>
+      <c r="R91" s="1">
+        <v>0.001143850749403486</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18">
       <c r="A92">
         <v>2017</v>
       </c>
@@ -6507,8 +7697,17 @@
       <c r="O92" s="1">
         <v>0.007928391042689276</v>
       </c>
-    </row>
-    <row r="93" spans="1:15">
+      <c r="P92" s="1">
+        <v>0.003325270496266519</v>
+      </c>
+      <c r="Q92" s="1">
+        <v>0.006321009399657962</v>
+      </c>
+      <c r="R92" s="1">
+        <v>0.02787618565202199</v>
+      </c>
+    </row>
+    <row r="93" spans="1:18">
       <c r="A93">
         <v>2018</v>
       </c>
@@ -6554,8 +7753,17 @@
       <c r="O93" s="1">
         <v>0.01804714613104363</v>
       </c>
-    </row>
-    <row r="94" spans="1:15">
+      <c r="P93" s="1">
+        <v>0.01516833272729823</v>
+      </c>
+      <c r="Q93" s="1">
+        <v>0.01264784785415607</v>
+      </c>
+      <c r="R93" s="1">
+        <v>0.002774149127293901</v>
+      </c>
+    </row>
+    <row r="94" spans="1:18">
       <c r="A94">
         <v>2019</v>
       </c>
@@ -6601,8 +7809,17 @@
       <c r="O94" s="1">
         <v>0.02140673960956208</v>
       </c>
-    </row>
-    <row r="95" spans="1:15">
+      <c r="P94" s="1">
+        <v>0.03088799246541929</v>
+      </c>
+      <c r="Q94" s="1">
+        <v>0.05910933384103845</v>
+      </c>
+      <c r="R94" s="1">
+        <v>0.09217201732368774</v>
+      </c>
+    </row>
+    <row r="95" spans="1:18">
       <c r="A95">
         <v>2020</v>
       </c>
@@ -6648,8 +7865,17 @@
       <c r="O95" s="1">
         <v>0.004507806614990173</v>
       </c>
-    </row>
-    <row r="96" spans="1:15">
+      <c r="P95" s="1">
+        <v>0.01809902777672412</v>
+      </c>
+      <c r="Q95" s="1">
+        <v>0.07127287260409809</v>
+      </c>
+      <c r="R95" s="1">
+        <v>0.1041313820851044</v>
+      </c>
+    </row>
+    <row r="96" spans="1:18">
       <c r="A96">
         <v>2021</v>
       </c>
@@ -6695,8 +7921,17 @@
       <c r="O96" s="1">
         <v>9.999999999998899E-05</v>
       </c>
-    </row>
-    <row r="97" spans="1:15">
+      <c r="P96" s="1">
+        <v>-0.001702262084092077</v>
+      </c>
+      <c r="Q96" s="1">
+        <v>-0.03467104499973528</v>
+      </c>
+      <c r="R96" s="1">
+        <v>-0.04067539912126494</v>
+      </c>
+    </row>
+    <row r="97" spans="1:18">
       <c r="A97">
         <v>2022</v>
       </c>
@@ -6742,8 +7977,17 @@
       <c r="O97" s="1">
         <v>0.0140818064912358</v>
       </c>
-    </row>
-    <row r="98" spans="1:15">
+      <c r="P97" s="1">
+        <v>-0.01336836643987316</v>
+      </c>
+      <c r="Q97" s="1">
+        <v>-0.09312159939086873</v>
+      </c>
+      <c r="R97" s="1">
+        <v>-0.1635891239682772</v>
+      </c>
+    </row>
+    <row r="98" spans="1:18">
       <c r="A98">
         <v>2023</v>
       </c>
@@ -6789,8 +8033,17 @@
       <c r="O98" s="1">
         <v>0.04938241510313612</v>
       </c>
-    </row>
-    <row r="99" spans="1:15">
+      <c r="P98" s="1">
+        <v>0.05168596287459359</v>
+      </c>
+      <c r="Q98" s="1">
+        <v>0.0477372003232106</v>
+      </c>
+      <c r="R98" s="1">
+        <v>0.03838764405368678</v>
+      </c>
+    </row>
+    <row r="99" spans="1:18">
       <c r="A99">
         <v>2024</v>
       </c>
@@ -6836,8 +8089,17 @@
       <c r="O99" s="1">
         <v>0.05252283500850252</v>
       </c>
-    </row>
-    <row r="100" spans="1:15">
+      <c r="P99" s="1">
+        <v>0.0541744461586795</v>
+      </c>
+      <c r="Q99" s="1">
+        <v>0.01690210925782254</v>
+      </c>
+      <c r="R99" s="1">
+        <v>-0.01536790197705307</v>
+      </c>
+    </row>
+    <row r="100" spans="1:18">
       <c r="A100">
         <v>2025</v>
       </c>
@@ -6882,6 +8144,15 @@
       </c>
       <c r="O100" s="1">
         <v>0.0425059734032367</v>
+      </c>
+      <c r="P100" s="1">
+        <v>0.04642685162146187</v>
+      </c>
+      <c r="Q100" s="1">
+        <v>0.06977434210917988</v>
+      </c>
+      <c r="R100" s="1">
+        <v>0.07693351206000054</v>
       </c>
     </row>
   </sheetData>
@@ -6902,16 +8173,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>

<commit_message>
Continue Trend with AQMIX after AQR's factor data ends
Trend = AQR TSMOM + RF through AQR's last month (2026-05), then AQMIX's
monthly total return (Yahoo, distributions reinvested) to 2026-09.
Overlap 2010-02..2026-05: correlation 0.76, tracking error 8.5%/yr; the
fund returned 4.8%/yr vs the factor's 6.9%, a direct read on fees and
costs. Saved to trend_splice.csv and the Trend_Splice sheet.

Trend now runs as far as the other sleeves, so it starts ticked again
(default_on stays available for future sleeves). The Yahoo reader is
renamed read_yahoo_monthly and splice_check takes any two columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtyJ36mjEj9LzVccKuq7PT
</commit_message>
<xml_diff>
--- a/data/processed/stats.xlsx
+++ b/data/processed/stats.xlsx
@@ -19,13 +19,14 @@
     <sheet name="Annual_Check" sheetId="10" r:id="rId10"/>
     <sheet name="Size_Lag_Check" sheetId="11" r:id="rId11"/>
     <sheet name="Commodities_Splice" sheetId="12" r:id="rId12"/>
+    <sheet name="Trend_Splice" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="158">
   <si>
     <t>note</t>
   </si>
@@ -48,7 +49,7 @@
     <t>A window's stats are blank (see note) if the sleeve does not cover the whole window.</t>
   </si>
   <si>
-    <t>Correlation window: 1990-07 to 2026-05 (all sleeves present).</t>
+    <t>Correlation window: 1990-07 to 2026-09 (all sleeves present).</t>
   </si>
   <si>
     <t>DevExUS_Market/EM_Market: six portfolios weighted by avg firm size x number of firms, lagged 0 month(s) (lag chosen by tracking the US market; see Size_Lag_Check).</t>
@@ -105,6 +106,9 @@
     <t>AQR Time Series Momentum: Factors, Monthly</t>
   </si>
   <si>
+    <t>AQMIX (Yahoo Finance)</t>
+  </si>
+  <si>
     <t>F-F_Research_Data_Factors.csv</t>
   </si>
   <si>
@@ -138,6 +142,9 @@
     <t>Time-Series-Momentum-Factors-Monthly.xlsx</t>
   </si>
   <si>
+    <t>AQMIX_yahoo_daily.json</t>
+  </si>
+  <si>
     <t>This file was created using the 202609 CRSP database.</t>
   </si>
   <si>
@@ -159,6 +166,9 @@
     <t>data through 2026-05</t>
   </si>
   <si>
+    <t>2010-02 to 2026-09</t>
+  </si>
+  <si>
     <t>202609</t>
   </si>
   <si>
@@ -171,16 +181,16 @@
     <t>202605</t>
   </si>
   <si>
-    <t>2026-10-30T02:02:27</t>
+    <t>2026-10-30T02:07:52</t>
   </si>
   <si>
-    <t>2026-10-30T02:02:29</t>
+    <t>2026-10-30T02:07:53</t>
   </si>
   <si>
-    <t>2026-10-30T02:02:30</t>
+    <t>2026-10-30T02:07:55</t>
   </si>
   <si>
-    <t>2026-10-30T02:02:31</t>
+    <t>2026-10-30T02:07:56</t>
   </si>
   <si>
     <t>start</t>
@@ -294,9 +304,6 @@
     <t>2026-09</t>
   </si>
   <si>
-    <t>2026-05</t>
-  </si>
-  <si>
     <t>1990-01</t>
   </si>
   <si>
@@ -312,7 +319,7 @@
     <t>2025-12</t>
   </si>
   <si>
-    <t>1990-07 to 2026-05</t>
+    <t>1990-07 to 2026-09</t>
   </si>
   <si>
     <t>year</t>
@@ -388,6 +395,111 @@
   </si>
   <si>
     <t>0.4% / 6.6%</t>
+  </si>
+  <si>
+    <t>2010 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2011 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2012 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2013 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2014 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2015 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2016 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2017 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2018 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2019 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2020 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2021 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2022 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2023 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2024 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2025 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2026 factor / AQMIX</t>
+  </si>
+  <si>
+    <t>2010-02 to 2026-05</t>
+  </si>
+  <si>
+    <t>18.2% / 9.3%</t>
+  </si>
+  <si>
+    <t>-0.1% / -6.4%</t>
+  </si>
+  <si>
+    <t>-0.1% / 3.0%</t>
+  </si>
+  <si>
+    <t>18.2% / 9.4%</t>
+  </si>
+  <si>
+    <t>19.1% / 9.7%</t>
+  </si>
+  <si>
+    <t>18.1% / 2.0%</t>
+  </si>
+  <si>
+    <t>-10.9% / -8.4%</t>
+  </si>
+  <si>
+    <t>7.5% / -1.0%</t>
+  </si>
+  <si>
+    <t>-7.4% / -8.9%</t>
+  </si>
+  <si>
+    <t>5.4% / 1.9%</t>
+  </si>
+  <si>
+    <t>-6.3% / -0.4%</t>
+  </si>
+  <si>
+    <t>-4.6% / -1.0%</t>
+  </si>
+  <si>
+    <t>26.5% / 35.5%</t>
+  </si>
+  <si>
+    <t>-3.6% / 2.1%</t>
+  </si>
+  <si>
+    <t>8.9% / 8.1%</t>
+  </si>
+  <si>
+    <t>6.1% / 14.6%</t>
+  </si>
+  <si>
+    <t>17.0% / 11.0%</t>
   </si>
 </sst>
 </file>
@@ -824,21 +936,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B2">
         <v>99</v>
@@ -852,7 +964,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B3">
         <v>99</v>
@@ -866,7 +978,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>99</v>
@@ -880,7 +992,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B5">
         <v>99</v>
@@ -894,7 +1006,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B6">
         <v>62</v>
@@ -908,7 +1020,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B7">
         <v>62</v>
@@ -922,7 +1034,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B8">
         <v>35</v>
@@ -936,7 +1048,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B9">
         <v>35</v>
@@ -950,7 +1062,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B10">
         <v>36</v>
@@ -964,7 +1076,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -995,19 +1107,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1060,23 +1172,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B3">
         <v>39</v>
@@ -1084,58 +1196,256 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B4">
-        <v>0.8593973096503562</v>
+        <v>0.8593971379562713</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B5">
-        <v>0.06226036072395819</v>
+        <v>0.06226038908748011</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6">
-        <v>0.0342781852026973</v>
+        <v>0.03427818111792311</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4">
+        <v>0.7555474316099458</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5">
+        <v>0.08525353661429502</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B6">
+        <v>-0.02097658754190014</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>124</v>
+      </c>
+      <c r="B8" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B14" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B15" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B19" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>136</v>
+      </c>
+      <c r="B20" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1145,7 +1455,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
@@ -1175,16 +1485,16 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1192,16 +1502,16 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1209,16 +1519,16 @@
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1226,16 +1536,16 @@
         <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1243,16 +1553,16 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1260,16 +1570,16 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1277,16 +1587,16 @@
         <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1294,16 +1604,16 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1311,16 +1621,16 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1328,16 +1638,16 @@
         <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1345,16 +1655,33 @@
         <v>25</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
         <v>47</v>
       </c>
-      <c r="E12" t="s">
-        <v>51</v>
+      <c r="E13" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1378,31 +1705,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1410,13 +1737,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>1203</v>
@@ -1439,13 +1766,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>1203</v>
@@ -1468,13 +1795,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>1203</v>
@@ -1497,13 +1824,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>1203</v>
@@ -1526,13 +1853,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>1203</v>
@@ -1555,13 +1882,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>759</v>
@@ -1584,13 +1911,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D8">
         <v>759</v>
@@ -1613,13 +1940,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D9">
         <v>435</v>
@@ -1642,13 +1969,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D10">
         <v>435</v>
@@ -1671,13 +1998,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>435</v>
@@ -1700,13 +2027,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>447</v>
@@ -1729,13 +2056,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>447</v>
@@ -1758,13 +2085,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D14">
         <v>447</v>
@@ -1787,13 +2114,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>1203</v>
@@ -1813,13 +2140,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D16">
         <v>776</v>
@@ -1842,13 +2169,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>776</v>
@@ -1871,13 +2198,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D18">
         <v>776</v>
@@ -1900,13 +2227,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D19">
         <v>1203</v>
@@ -1929,25 +2256,25 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D20">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1565255407267883</v>
+        <v>0.157097573770842</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1256326523597845</v>
+        <v>0.1253688111581719</v>
       </c>
       <c r="G20" s="2">
-        <v>0.9809092639522505</v>
+        <v>0.9864060355664387</v>
       </c>
       <c r="H20" s="1">
         <v>-0.24751379044844</v>
@@ -1958,13 +2285,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D21">
         <v>1197</v>
@@ -2006,31 +2333,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -2038,13 +2365,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>441</v>
@@ -2067,13 +2394,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>441</v>
@@ -2096,13 +2423,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>441</v>
@@ -2125,13 +2452,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>441</v>
@@ -2154,13 +2481,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>441</v>
@@ -2183,13 +2510,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>441</v>
@@ -2212,13 +2539,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D8">
         <v>441</v>
@@ -2241,37 +2568,37 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="J9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="J11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>441</v>
@@ -2294,13 +2621,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>441</v>
@@ -2323,13 +2650,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D14">
         <v>441</v>
@@ -2352,13 +2679,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>441</v>
@@ -2378,13 +2705,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D16">
         <v>441</v>
@@ -2407,13 +2734,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>441</v>
@@ -2436,13 +2763,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D18">
         <v>441</v>
@@ -2465,13 +2792,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D19">
         <v>441</v>
@@ -2494,25 +2821,25 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D20">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1389978913304704</v>
+        <v>0.1397957942992942</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1255980836198725</v>
+        <v>0.1253045861553731</v>
       </c>
       <c r="G20" s="2">
-        <v>0.8934608328993161</v>
+        <v>0.9002521875071546</v>
       </c>
       <c r="H20" s="1">
         <v>-0.2475137904484402</v>
@@ -2523,13 +2850,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D21">
         <v>441</v>
@@ -2571,31 +2898,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -2603,13 +2930,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>321</v>
@@ -2632,13 +2959,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>321</v>
@@ -2661,13 +2988,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>321</v>
@@ -2690,13 +3017,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>321</v>
@@ -2719,13 +3046,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>321</v>
@@ -2748,13 +3075,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>321</v>
@@ -2777,13 +3104,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D8">
         <v>321</v>
@@ -2806,13 +3133,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D9">
         <v>321</v>
@@ -2835,13 +3162,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D10">
         <v>321</v>
@@ -2864,13 +3191,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>321</v>
@@ -2893,13 +3220,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>321</v>
@@ -2922,13 +3249,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>321</v>
@@ -2951,13 +3278,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D14">
         <v>321</v>
@@ -2980,13 +3307,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>321</v>
@@ -3006,13 +3333,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D16">
         <v>321</v>
@@ -3035,13 +3362,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>321</v>
@@ -3064,13 +3391,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D18">
         <v>321</v>
@@ -3093,13 +3420,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D19">
         <v>321</v>
@@ -3122,25 +3449,25 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D20">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1026235485420854</v>
+        <v>0.1041313313420678</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1302084249426989</v>
+        <v>0.1297851530001127</v>
       </c>
       <c r="G20" s="2">
-        <v>0.6736995970390685</v>
+        <v>0.6844767542346577</v>
       </c>
       <c r="H20" s="1">
         <v>-0.2475137904484401</v>
@@ -3151,13 +3478,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D21">
         <v>321</v>
@@ -3199,31 +3526,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -3231,13 +3558,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D2">
         <v>120</v>
@@ -3260,13 +3587,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D3">
         <v>120</v>
@@ -3289,13 +3616,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D4">
         <v>120</v>
@@ -3318,13 +3645,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5">
         <v>120</v>
@@ -3347,13 +3674,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6">
         <v>120</v>
@@ -3376,13 +3703,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D7">
         <v>120</v>
@@ -3405,13 +3732,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D8">
         <v>120</v>
@@ -3434,13 +3761,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D9">
         <v>120</v>
@@ -3463,13 +3790,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D10">
         <v>120</v>
@@ -3492,13 +3819,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D11">
         <v>120</v>
@@ -3521,13 +3848,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D12">
         <v>120</v>
@@ -3550,13 +3877,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D13">
         <v>120</v>
@@ -3579,13 +3906,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D14">
         <v>120</v>
@@ -3608,13 +3935,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C15" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D15">
         <v>120</v>
@@ -3634,13 +3961,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D16">
         <v>120</v>
@@ -3663,13 +3990,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D17">
         <v>120</v>
@@ -3692,13 +4019,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D18">
         <v>120</v>
@@ -3721,13 +4048,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D19">
         <v>120</v>
@@ -3750,13 +4077,13 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D20">
         <v>120</v>
@@ -3779,13 +4106,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D21">
         <v>120</v>
@@ -3833,1364 +4160,1364 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>0.8096433991813985</v>
+        <v>0.8084723245525287</v>
       </c>
       <c r="D2" s="2">
-        <v>0.846777718021643</v>
+        <v>0.8453565887860622</v>
       </c>
       <c r="E2" s="2">
-        <v>0.8453796249393708</v>
+        <v>0.8427478229847296</v>
       </c>
       <c r="F2" s="2">
-        <v>0.9726435036446569</v>
+        <v>0.9722190415305743</v>
       </c>
       <c r="G2" s="2">
-        <v>0.8560192076452968</v>
+        <v>0.853257488679916</v>
       </c>
       <c r="H2" s="2">
-        <v>0.8389198393695788</v>
+        <v>0.8369340000236228</v>
       </c>
       <c r="I2" s="2">
-        <v>0.6233767571877212</v>
+        <v>0.6226168068197092</v>
       </c>
       <c r="J2" s="2">
-        <v>0.7142828096505718</v>
+        <v>0.7124647204721374</v>
       </c>
       <c r="K2" s="2">
-        <v>0.7661183176682003</v>
+        <v>0.7658313815373569</v>
       </c>
       <c r="L2" s="2">
-        <v>0.6012799065004881</v>
+        <v>0.6018775544729295</v>
       </c>
       <c r="M2" s="2">
-        <v>0.6773848837824795</v>
+        <v>0.6774842229672553</v>
       </c>
       <c r="N2" s="2">
-        <v>0.7105012741986562</v>
+        <v>0.7107951348280582</v>
       </c>
       <c r="O2" s="2">
-        <v>0.009584646447675359</v>
+        <v>0.008720575418330557</v>
       </c>
       <c r="P2" s="2">
-        <v>-0.04636172981650317</v>
+        <v>-0.04506667671579052</v>
       </c>
       <c r="Q2" s="2">
-        <v>-0.09614128262587439</v>
+        <v>-0.09296776454437576</v>
       </c>
       <c r="R2" s="2">
-        <v>-0.07146393462854077</v>
+        <v>-0.06844342659119444</v>
       </c>
       <c r="S2" s="2">
-        <v>0.3378905257949931</v>
+        <v>0.3345626558024875</v>
       </c>
       <c r="T2" s="2">
-        <v>-0.1689177870014295</v>
+        <v>-0.1684954070223643</v>
       </c>
       <c r="U2" s="2">
-        <v>-0.32037206049654</v>
+        <v>-0.3189467570670729</v>
       </c>
     </row>
     <row r="3" spans="1:21">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B3" s="2">
-        <v>0.8096433991813985</v>
+        <v>0.8084723245525287</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2">
-        <v>0.8444904352509209</v>
+        <v>0.8442345773162365</v>
       </c>
       <c r="E3" s="2">
-        <v>0.8511767193053412</v>
+        <v>0.8508605159127607</v>
       </c>
       <c r="F3" s="2">
-        <v>0.6883274999494429</v>
+        <v>0.6857038262534598</v>
       </c>
       <c r="G3" s="2">
-        <v>0.9432701207377049</v>
+        <v>0.9424307523014479</v>
       </c>
       <c r="H3" s="2">
-        <v>0.8888881086631615</v>
+        <v>0.887638654114019</v>
       </c>
       <c r="I3" s="2">
-        <v>0.6204810907457552</v>
+        <v>0.616939304854914</v>
       </c>
       <c r="J3" s="2">
-        <v>0.6729017709675852</v>
+        <v>0.6707882856220584</v>
       </c>
       <c r="K3" s="2">
-        <v>0.6484196492772125</v>
+        <v>0.6479546343410681</v>
       </c>
       <c r="L3" s="2">
-        <v>0.5667203974854238</v>
+        <v>0.56490422972805</v>
       </c>
       <c r="M3" s="2">
-        <v>0.6193496593213892</v>
+        <v>0.6179141607712995</v>
       </c>
       <c r="N3" s="2">
-        <v>0.6196324027250396</v>
+        <v>0.6183865103958412</v>
       </c>
       <c r="O3" s="2">
-        <v>-0.02685617461986891</v>
+        <v>-0.02824889606400737</v>
       </c>
       <c r="P3" s="2">
-        <v>-0.08539910297957878</v>
+        <v>-0.08341305607916655</v>
       </c>
       <c r="Q3" s="2">
-        <v>-0.1736003111989576</v>
+        <v>-0.1669728157126054</v>
       </c>
       <c r="R3" s="2">
-        <v>-0.1597453856879754</v>
+        <v>-0.1530995276764361</v>
       </c>
       <c r="S3" s="2">
-        <v>0.3514232350344638</v>
+        <v>0.341024462184917</v>
       </c>
       <c r="T3" s="2">
-        <v>-0.1981611543076019</v>
+        <v>-0.2008957269764446</v>
       </c>
       <c r="U3" s="2">
-        <v>-0.1248352240258522</v>
+        <v>-0.1220064155989652</v>
       </c>
     </row>
     <row r="4" spans="1:21">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B4" s="2">
-        <v>0.846777718021643</v>
+        <v>0.8453565887860622</v>
       </c>
       <c r="C4" s="2">
-        <v>0.8444904352509209</v>
+        <v>0.8442345773162365</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
       </c>
       <c r="E4" s="2">
-        <v>0.6778518447442872</v>
+        <v>0.6784637482750013</v>
       </c>
       <c r="F4" s="2">
-        <v>0.7903926703768496</v>
+        <v>0.787093796941043</v>
       </c>
       <c r="G4" s="2">
-        <v>0.8744387742831448</v>
+        <v>0.8737886646264377</v>
       </c>
       <c r="H4" s="2">
-        <v>0.9796268873267917</v>
+        <v>0.9791311355923366</v>
       </c>
       <c r="I4" s="2">
-        <v>0.5543834926709202</v>
+        <v>0.5513730451567017</v>
       </c>
       <c r="J4" s="2">
-        <v>0.5785866749828059</v>
+        <v>0.5765671231031085</v>
       </c>
       <c r="K4" s="2">
-        <v>0.6449996198974118</v>
+        <v>0.6444648115467011</v>
       </c>
       <c r="L4" s="2">
-        <v>0.5517311495825314</v>
+        <v>0.5506400965176783</v>
       </c>
       <c r="M4" s="2">
-        <v>0.5977806327849094</v>
+        <v>0.5966444871624802</v>
       </c>
       <c r="N4" s="2">
-        <v>0.6531983783416054</v>
+        <v>0.652160674333882</v>
       </c>
       <c r="O4" s="2">
-        <v>-0.03686496465253911</v>
+        <v>-0.03719089081106493</v>
       </c>
       <c r="P4" s="2">
-        <v>-0.1001351572198626</v>
+        <v>-0.09814503936050406</v>
       </c>
       <c r="Q4" s="2">
-        <v>-0.1683106841155229</v>
+        <v>-0.1618658671180353</v>
       </c>
       <c r="R4" s="2">
-        <v>-0.1353218322228005</v>
+        <v>-0.1286849343882467</v>
       </c>
       <c r="S4" s="2">
-        <v>0.2679064134892237</v>
+        <v>0.2620500041526474</v>
       </c>
       <c r="T4" s="2">
-        <v>-0.1626674642662103</v>
+        <v>-0.165540027193309</v>
       </c>
       <c r="U4" s="2">
-        <v>-0.3648494781702741</v>
+        <v>-0.3609812152018139</v>
       </c>
     </row>
     <row r="5" spans="1:21">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B5" s="2">
-        <v>0.8453796249393708</v>
+        <v>0.8427478229847296</v>
       </c>
       <c r="C5" s="2">
-        <v>0.8511767193053412</v>
+        <v>0.8508605159127607</v>
       </c>
       <c r="D5" s="2">
-        <v>0.6778518447442872</v>
+        <v>0.6784637482750013</v>
       </c>
       <c r="E5" s="2">
         <v>1</v>
       </c>
       <c r="F5" s="2">
-        <v>0.7437531966309258</v>
+        <v>0.738754141063812</v>
       </c>
       <c r="G5" s="2">
-        <v>0.8308276422876273</v>
+        <v>0.8311419653760164</v>
       </c>
       <c r="H5" s="2">
-        <v>0.7110816436313072</v>
+        <v>0.7104386565659305</v>
       </c>
       <c r="I5" s="2">
-        <v>0.5888885343085898</v>
+        <v>0.5847784521158335</v>
       </c>
       <c r="J5" s="2">
-        <v>0.7229548269779759</v>
+        <v>0.7211187227494855</v>
       </c>
       <c r="K5" s="2">
-        <v>0.6753562183268415</v>
+        <v>0.6743214242036054</v>
       </c>
       <c r="L5" s="2">
-        <v>0.5393219082861939</v>
+        <v>0.5361976512742476</v>
       </c>
       <c r="M5" s="2">
-        <v>0.6152297655380377</v>
+        <v>0.6133184543655397</v>
       </c>
       <c r="N5" s="2">
-        <v>0.5990751299349901</v>
+        <v>0.5960924318780843</v>
       </c>
       <c r="O5" s="2">
-        <v>0.03399140212411957</v>
+        <v>0.03408876177247213</v>
       </c>
       <c r="P5" s="2">
-        <v>-0.04383561262469876</v>
+        <v>-0.04266035602041702</v>
       </c>
       <c r="Q5" s="2">
-        <v>-0.1376246887187236</v>
+        <v>-0.1331638473484328</v>
       </c>
       <c r="R5" s="2">
-        <v>-0.1328746699994343</v>
+        <v>-0.1282930343377397</v>
       </c>
       <c r="S5" s="2">
-        <v>0.3666724964036682</v>
+        <v>0.3572246201059924</v>
       </c>
       <c r="T5" s="2">
-        <v>-0.2092861314366406</v>
+        <v>-0.2124948053634381</v>
       </c>
       <c r="U5" s="2">
-        <v>-0.09148888749273987</v>
+        <v>-0.09041687676338699</v>
       </c>
     </row>
     <row r="6" spans="1:21">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B6" s="2">
-        <v>0.9726435036446569</v>
+        <v>0.9722190415305743</v>
       </c>
       <c r="C6" s="2">
-        <v>0.6883274999494429</v>
+        <v>0.6857038262534598</v>
       </c>
       <c r="D6" s="2">
-        <v>0.7903926703768496</v>
+        <v>0.787093796941043</v>
       </c>
       <c r="E6" s="2">
-        <v>0.7437531966309258</v>
+        <v>0.738754141063812</v>
       </c>
       <c r="F6" s="2">
         <v>1</v>
       </c>
       <c r="G6" s="2">
-        <v>0.7657979322849678</v>
+        <v>0.7607708316913162</v>
       </c>
       <c r="H6" s="2">
-        <v>0.7622933464652624</v>
+        <v>0.7588004995706208</v>
       </c>
       <c r="I6" s="2">
-        <v>0.5456236850082158</v>
+        <v>0.5455653619900337</v>
       </c>
       <c r="J6" s="2">
-        <v>0.6330013344656648</v>
+        <v>0.6303556794779929</v>
       </c>
       <c r="K6" s="2">
-        <v>0.7127159823198855</v>
+        <v>0.7116541350181254</v>
       </c>
       <c r="L6" s="2">
-        <v>0.5485906492778998</v>
+        <v>0.5497917868990337</v>
       </c>
       <c r="M6" s="2">
-        <v>0.6145555049673492</v>
+        <v>0.6145155097428121</v>
       </c>
       <c r="N6" s="2">
-        <v>0.6622117543843254</v>
+        <v>0.6628003878568192</v>
       </c>
       <c r="O6" s="2">
-        <v>0.0197771985145627</v>
+        <v>0.01855625776085682</v>
       </c>
       <c r="P6" s="2">
-        <v>-0.02575807527443629</v>
+        <v>-0.02456960704491969</v>
       </c>
       <c r="Q6" s="2">
-        <v>-0.05243182518594684</v>
+        <v>-0.05024814655886989</v>
       </c>
       <c r="R6" s="2">
-        <v>-0.02353782628363642</v>
+        <v>-0.02164763978431109</v>
       </c>
       <c r="S6" s="2">
-        <v>0.2766323047085008</v>
+        <v>0.2760077792474183</v>
       </c>
       <c r="T6" s="2">
-        <v>-0.146445277653909</v>
+        <v>-0.1441775053990973</v>
       </c>
       <c r="U6" s="2">
-        <v>-0.3771733162097329</v>
+        <v>-0.3754013538160224</v>
       </c>
     </row>
     <row r="7" spans="1:21">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B7" s="2">
-        <v>0.8560192076452968</v>
+        <v>0.853257488679916</v>
       </c>
       <c r="C7" s="2">
-        <v>0.9432701207377049</v>
+        <v>0.9424307523014479</v>
       </c>
       <c r="D7" s="2">
-        <v>0.8744387742831448</v>
+        <v>0.8737886646264377</v>
       </c>
       <c r="E7" s="2">
-        <v>0.8308276422876273</v>
+        <v>0.8311419653760164</v>
       </c>
       <c r="F7" s="2">
-        <v>0.7657979322849678</v>
+        <v>0.7607708316913162</v>
       </c>
       <c r="G7" s="2">
         <v>1</v>
       </c>
       <c r="H7" s="2">
-        <v>0.8664350243446503</v>
+        <v>0.8636991464038809</v>
       </c>
       <c r="I7" s="2">
-        <v>0.6299375548408933</v>
+        <v>0.6274339727052324</v>
       </c>
       <c r="J7" s="2">
-        <v>0.6826271710899674</v>
+        <v>0.6823128207506383</v>
       </c>
       <c r="K7" s="2">
-        <v>0.6848949644551299</v>
+        <v>0.6847755401222625</v>
       </c>
       <c r="L7" s="2">
-        <v>0.5986630610171139</v>
+        <v>0.5955790154563038</v>
       </c>
       <c r="M7" s="2">
-        <v>0.6483593086926021</v>
+        <v>0.6466960454123722</v>
       </c>
       <c r="N7" s="2">
-        <v>0.6558294329448272</v>
+        <v>0.6523683811807718</v>
       </c>
       <c r="O7" s="2">
-        <v>-0.03348573201749485</v>
+        <v>-0.03372260379160047</v>
       </c>
       <c r="P7" s="2">
-        <v>-0.1015550428804258</v>
+        <v>-0.0987636496596019</v>
       </c>
       <c r="Q7" s="2">
-        <v>-0.16373171378621</v>
+        <v>-0.1569293347194135</v>
       </c>
       <c r="R7" s="2">
-        <v>-0.1482563302733315</v>
+        <v>-0.1419150028229105</v>
       </c>
       <c r="S7" s="2">
-        <v>0.3450360379753788</v>
+        <v>0.3393877351057602</v>
       </c>
       <c r="T7" s="2">
-        <v>-0.2079441875225685</v>
+        <v>-0.211484808454069</v>
       </c>
       <c r="U7" s="2">
-        <v>-0.2393903818647102</v>
+        <v>-0.2397542147734855</v>
       </c>
     </row>
     <row r="8" spans="1:21">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B8" s="2">
-        <v>0.8389198393695788</v>
+        <v>0.8369340000236228</v>
       </c>
       <c r="C8" s="2">
-        <v>0.8888881086631615</v>
+        <v>0.887638654114019</v>
       </c>
       <c r="D8" s="2">
-        <v>0.9796268873267917</v>
+        <v>0.9791311355923366</v>
       </c>
       <c r="E8" s="2">
-        <v>0.7110816436313072</v>
+        <v>0.7104386565659305</v>
       </c>
       <c r="F8" s="2">
-        <v>0.7622933464652624</v>
+        <v>0.7588004995706208</v>
       </c>
       <c r="G8" s="2">
-        <v>0.8664350243446503</v>
+        <v>0.8636991464038809</v>
       </c>
       <c r="H8" s="2">
         <v>1</v>
       </c>
       <c r="I8" s="2">
-        <v>0.5827834654600033</v>
+        <v>0.5771672119289666</v>
       </c>
       <c r="J8" s="2">
-        <v>0.6043847731877485</v>
+        <v>0.5994339955388748</v>
       </c>
       <c r="K8" s="2">
-        <v>0.6528459191684159</v>
+        <v>0.6506133252461415</v>
       </c>
       <c r="L8" s="2">
-        <v>0.5649804331517488</v>
+        <v>0.5635961507293357</v>
       </c>
       <c r="M8" s="2">
-        <v>0.6161196328919373</v>
+        <v>0.6138102415392311</v>
       </c>
       <c r="N8" s="2">
-        <v>0.6633916545412428</v>
+        <v>0.6626772183491964</v>
       </c>
       <c r="O8" s="2">
-        <v>-0.03337555719644102</v>
+        <v>-0.03399474920195936</v>
       </c>
       <c r="P8" s="2">
-        <v>-0.09330109406670307</v>
+        <v>-0.09187391203733189</v>
       </c>
       <c r="Q8" s="2">
-        <v>-0.1755445867819954</v>
+        <v>-0.1688919112178923</v>
       </c>
       <c r="R8" s="2">
-        <v>-0.1457213353633865</v>
+        <v>-0.1382991339059669</v>
       </c>
       <c r="S8" s="2">
-        <v>0.2972792739820233</v>
+        <v>0.2867071752857003</v>
       </c>
       <c r="T8" s="2">
-        <v>-0.1617932016412099</v>
+        <v>-0.1642219365556789</v>
       </c>
       <c r="U8" s="2">
-        <v>-0.3054183134562681</v>
+        <v>-0.2984254417000554</v>
       </c>
     </row>
     <row r="9" spans="1:21">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2">
-        <v>0.6233767571877212</v>
+        <v>0.6226168068197092</v>
       </c>
       <c r="C9" s="2">
-        <v>0.6204810907457552</v>
+        <v>0.616939304854914</v>
       </c>
       <c r="D9" s="2">
-        <v>0.5543834926709202</v>
+        <v>0.5513730451567017</v>
       </c>
       <c r="E9" s="2">
-        <v>0.5888885343085898</v>
+        <v>0.5847784521158335</v>
       </c>
       <c r="F9" s="2">
-        <v>0.5456236850082158</v>
+        <v>0.5455653619900337</v>
       </c>
       <c r="G9" s="2">
-        <v>0.6299375548408933</v>
+        <v>0.6274339727052324</v>
       </c>
       <c r="H9" s="2">
-        <v>0.5827834654600033</v>
+        <v>0.5771672119289666</v>
       </c>
       <c r="I9" s="2">
         <v>1</v>
       </c>
       <c r="J9" s="2">
-        <v>0.8918043208913244</v>
+        <v>0.8911441158386861</v>
       </c>
       <c r="K9" s="2">
-        <v>0.8946489159016753</v>
+        <v>0.8938340968307302</v>
       </c>
       <c r="L9" s="2">
-        <v>0.6990758568531096</v>
+        <v>0.6986219926977082</v>
       </c>
       <c r="M9" s="2">
-        <v>0.7453873198548674</v>
+        <v>0.7452463294527234</v>
       </c>
       <c r="N9" s="2">
-        <v>0.7310765525783196</v>
+        <v>0.7286571574824861</v>
       </c>
       <c r="O9" s="2">
-        <v>-0.05985552146339091</v>
+        <v>-0.05951069382568925</v>
       </c>
       <c r="P9" s="2">
-        <v>-0.09475373588990976</v>
+        <v>-0.0920500071833109</v>
       </c>
       <c r="Q9" s="2">
-        <v>-0.065227516494911</v>
+        <v>-0.0631135836438298</v>
       </c>
       <c r="R9" s="2">
-        <v>-0.06957690766914951</v>
+        <v>-0.06846292883645531</v>
       </c>
       <c r="S9" s="2">
-        <v>0.4954537940781372</v>
+        <v>0.4994654824723255</v>
       </c>
       <c r="T9" s="2">
-        <v>-0.1736059617525851</v>
+        <v>-0.1715162899394772</v>
       </c>
       <c r="U9" s="2">
-        <v>-0.1774641860773877</v>
+        <v>-0.1871526740657589</v>
       </c>
     </row>
     <row r="10" spans="1:21">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B10" s="2">
-        <v>0.7142828096505718</v>
+        <v>0.7124647204721374</v>
       </c>
       <c r="C10" s="2">
-        <v>0.6729017709675852</v>
+        <v>0.6707882856220584</v>
       </c>
       <c r="D10" s="2">
-        <v>0.5785866749828059</v>
+        <v>0.5765671231031085</v>
       </c>
       <c r="E10" s="2">
-        <v>0.7229548269779759</v>
+        <v>0.7211187227494855</v>
       </c>
       <c r="F10" s="2">
-        <v>0.6330013344656648</v>
+        <v>0.6303556794779929</v>
       </c>
       <c r="G10" s="2">
-        <v>0.6826271710899674</v>
+        <v>0.6823128207506383</v>
       </c>
       <c r="H10" s="2">
-        <v>0.6043847731877485</v>
+        <v>0.5994339955388748</v>
       </c>
       <c r="I10" s="2">
-        <v>0.8918043208913244</v>
+        <v>0.8911441158386861</v>
       </c>
       <c r="J10" s="2">
         <v>1</v>
       </c>
       <c r="K10" s="2">
-        <v>0.9513827897847406</v>
+        <v>0.9507353729757182</v>
       </c>
       <c r="L10" s="2">
-        <v>0.6562805992684925</v>
+        <v>0.6541222537623749</v>
       </c>
       <c r="M10" s="2">
-        <v>0.747606729939191</v>
+        <v>0.7470311263495777</v>
       </c>
       <c r="N10" s="2">
-        <v>0.7285426364883216</v>
+        <v>0.7247025803243138</v>
       </c>
       <c r="O10" s="2">
-        <v>-0.004364604780607586</v>
+        <v>-0.003678721405237023</v>
       </c>
       <c r="P10" s="2">
-        <v>-0.07836931226757186</v>
+        <v>-0.07642551925864281</v>
       </c>
       <c r="Q10" s="2">
-        <v>-0.1258387040793985</v>
+        <v>-0.1238126821986896</v>
       </c>
       <c r="R10" s="2">
-        <v>-0.1435313280683901</v>
+        <v>-0.1423558442270655</v>
       </c>
       <c r="S10" s="2">
-        <v>0.4578966518656354</v>
+        <v>0.4583092063084198</v>
       </c>
       <c r="T10" s="2">
-        <v>-0.1855801250491936</v>
+        <v>-0.1856748158515933</v>
       </c>
       <c r="U10" s="2">
-        <v>-0.1878604972332749</v>
+        <v>-0.1943101739563054</v>
       </c>
     </row>
     <row r="11" spans="1:21">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B11" s="2">
-        <v>0.7661183176682003</v>
+        <v>0.7658313815373569</v>
       </c>
       <c r="C11" s="2">
-        <v>0.6484196492772125</v>
+        <v>0.6479546343410681</v>
       </c>
       <c r="D11" s="2">
-        <v>0.6449996198974118</v>
+        <v>0.6444648115467011</v>
       </c>
       <c r="E11" s="2">
-        <v>0.6753562183268415</v>
+        <v>0.6743214242036054</v>
       </c>
       <c r="F11" s="2">
-        <v>0.7127159823198855</v>
+        <v>0.7116541350181254</v>
       </c>
       <c r="G11" s="2">
-        <v>0.6848949644551299</v>
+        <v>0.6847755401222625</v>
       </c>
       <c r="H11" s="2">
-        <v>0.6528459191684159</v>
+        <v>0.6506133252461415</v>
       </c>
       <c r="I11" s="2">
-        <v>0.8946489159016753</v>
+        <v>0.8938340968307302</v>
       </c>
       <c r="J11" s="2">
-        <v>0.9513827897847406</v>
+        <v>0.9507353729757182</v>
       </c>
       <c r="K11" s="2">
         <v>1</v>
       </c>
       <c r="L11" s="2">
-        <v>0.6613533469054891</v>
+        <v>0.6609652840851206</v>
       </c>
       <c r="M11" s="2">
-        <v>0.7502552250104447</v>
+        <v>0.7503419338609657</v>
       </c>
       <c r="N11" s="2">
-        <v>0.7649959182315403</v>
+        <v>0.763697473242746</v>
       </c>
       <c r="O11" s="2">
-        <v>-0.01976407610881415</v>
+        <v>-0.02020794712335095</v>
       </c>
       <c r="P11" s="2">
-        <v>-0.06090999096451501</v>
+        <v>-0.05876270085485161</v>
       </c>
       <c r="Q11" s="2">
-        <v>-0.05272349172566651</v>
+        <v>-0.04906326386447808</v>
       </c>
       <c r="R11" s="2">
-        <v>-0.05599951351804124</v>
+        <v>-0.05280389386797559</v>
       </c>
       <c r="S11" s="2">
-        <v>0.4370170967980802</v>
+        <v>0.4347102962326969</v>
       </c>
       <c r="T11" s="2">
-        <v>-0.1601272046384987</v>
+        <v>-0.1608806417179749</v>
       </c>
       <c r="U11" s="2">
-        <v>-0.2438946616192481</v>
+        <v>-0.2468058826896434</v>
       </c>
     </row>
     <row r="12" spans="1:21">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B12" s="2">
-        <v>0.6012799065004881</v>
+        <v>0.6018775544729295</v>
       </c>
       <c r="C12" s="2">
-        <v>0.5667203974854238</v>
+        <v>0.56490422972805</v>
       </c>
       <c r="D12" s="2">
-        <v>0.5517311495825314</v>
+        <v>0.5506400965176783</v>
       </c>
       <c r="E12" s="2">
-        <v>0.5393219082861939</v>
+        <v>0.5361976512742476</v>
       </c>
       <c r="F12" s="2">
-        <v>0.5485906492778998</v>
+        <v>0.5497917868990337</v>
       </c>
       <c r="G12" s="2">
-        <v>0.5986630610171139</v>
+        <v>0.5955790154563038</v>
       </c>
       <c r="H12" s="2">
-        <v>0.5649804331517488</v>
+        <v>0.5635961507293357</v>
       </c>
       <c r="I12" s="2">
-        <v>0.6990758568531096</v>
+        <v>0.6986219926977082</v>
       </c>
       <c r="J12" s="2">
-        <v>0.6562805992684925</v>
+        <v>0.6541222537623749</v>
       </c>
       <c r="K12" s="2">
-        <v>0.6613533469054891</v>
+        <v>0.6609652840851206</v>
       </c>
       <c r="L12" s="2">
         <v>1</v>
       </c>
       <c r="M12" s="2">
-        <v>0.8956590981390005</v>
+        <v>0.8953083527111102</v>
       </c>
       <c r="N12" s="2">
-        <v>0.9104783024120462</v>
+        <v>0.9104056441867644</v>
       </c>
       <c r="O12" s="2">
-        <v>-0.04682185619165259</v>
+        <v>-0.04736336177182777</v>
       </c>
       <c r="P12" s="2">
-        <v>-0.1498223095093448</v>
+        <v>-0.1480923084546124</v>
       </c>
       <c r="Q12" s="2">
-        <v>-0.1788703147083445</v>
+        <v>-0.1752914157207034</v>
       </c>
       <c r="R12" s="2">
-        <v>-0.1603338311723812</v>
+        <v>-0.1568476382277995</v>
       </c>
       <c r="S12" s="2">
-        <v>0.4534461334711919</v>
+        <v>0.4509364578920367</v>
       </c>
       <c r="T12" s="2">
-        <v>-0.1278049496399567</v>
+        <v>-0.1263581861766898</v>
       </c>
       <c r="U12" s="2">
-        <v>-0.2446089130537028</v>
+        <v>-0.2462754075621131</v>
       </c>
     </row>
     <row r="13" spans="1:21">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B13" s="2">
-        <v>0.6773848837824795</v>
+        <v>0.6774842229672553</v>
       </c>
       <c r="C13" s="2">
-        <v>0.6193496593213892</v>
+        <v>0.6179141607712995</v>
       </c>
       <c r="D13" s="2">
-        <v>0.5977806327849094</v>
+        <v>0.5966444871624802</v>
       </c>
       <c r="E13" s="2">
-        <v>0.6152297655380377</v>
+        <v>0.6133184543655397</v>
       </c>
       <c r="F13" s="2">
-        <v>0.6145555049673492</v>
+        <v>0.6145155097428121</v>
       </c>
       <c r="G13" s="2">
-        <v>0.6483593086926021</v>
+        <v>0.6466960454123722</v>
       </c>
       <c r="H13" s="2">
-        <v>0.6161196328919373</v>
+        <v>0.6138102415392311</v>
       </c>
       <c r="I13" s="2">
-        <v>0.7453873198548674</v>
+        <v>0.7452463294527234</v>
       </c>
       <c r="J13" s="2">
-        <v>0.747606729939191</v>
+        <v>0.7470311263495777</v>
       </c>
       <c r="K13" s="2">
-        <v>0.7502552250104447</v>
+        <v>0.7503419338609657</v>
       </c>
       <c r="L13" s="2">
-        <v>0.8956590981390005</v>
+        <v>0.8953083527111102</v>
       </c>
       <c r="M13" s="2">
         <v>1</v>
       </c>
       <c r="N13" s="2">
-        <v>0.9562256128633357</v>
+        <v>0.9550848786347628</v>
       </c>
       <c r="O13" s="2">
-        <v>-0.03593945832635657</v>
+        <v>-0.03577601559653747</v>
       </c>
       <c r="P13" s="2">
-        <v>-0.09976166813954949</v>
+        <v>-0.09856543192274309</v>
       </c>
       <c r="Q13" s="2">
-        <v>-0.1348354759399666</v>
+        <v>-0.132987825107985</v>
       </c>
       <c r="R13" s="2">
-        <v>-0.1364211933548994</v>
+        <v>-0.1348365253180284</v>
       </c>
       <c r="S13" s="2">
-        <v>0.4721410661116966</v>
+        <v>0.4699504830762667</v>
       </c>
       <c r="T13" s="2">
-        <v>-0.127974512981622</v>
+        <v>-0.1272492165258428</v>
       </c>
       <c r="U13" s="2">
-        <v>-0.2550757132832688</v>
+        <v>-0.2573729833527058</v>
       </c>
     </row>
     <row r="14" spans="1:21">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B14" s="2">
-        <v>0.7105012741986562</v>
+        <v>0.7107951348280582</v>
       </c>
       <c r="C14" s="2">
-        <v>0.6196324027250396</v>
+        <v>0.6183865103958412</v>
       </c>
       <c r="D14" s="2">
-        <v>0.6531983783416054</v>
+        <v>0.652160674333882</v>
       </c>
       <c r="E14" s="2">
-        <v>0.5990751299349901</v>
+        <v>0.5960924318780843</v>
       </c>
       <c r="F14" s="2">
-        <v>0.6622117543843254</v>
+        <v>0.6628003878568192</v>
       </c>
       <c r="G14" s="2">
-        <v>0.6558294329448272</v>
+        <v>0.6523683811807718</v>
       </c>
       <c r="H14" s="2">
-        <v>0.6633916545412428</v>
+        <v>0.6626772183491964</v>
       </c>
       <c r="I14" s="2">
-        <v>0.7310765525783196</v>
+        <v>0.7286571574824861</v>
       </c>
       <c r="J14" s="2">
-        <v>0.7285426364883216</v>
+        <v>0.7247025803243138</v>
       </c>
       <c r="K14" s="2">
-        <v>0.7649959182315403</v>
+        <v>0.763697473242746</v>
       </c>
       <c r="L14" s="2">
-        <v>0.9104783024120462</v>
+        <v>0.9104056441867644</v>
       </c>
       <c r="M14" s="2">
-        <v>0.9562256128633357</v>
+        <v>0.9550848786347628</v>
       </c>
       <c r="N14" s="2">
         <v>1</v>
       </c>
       <c r="O14" s="2">
-        <v>-0.03081308414888551</v>
+        <v>-0.03205137004009748</v>
       </c>
       <c r="P14" s="2">
-        <v>-0.09716423714058922</v>
+        <v>-0.09573142285310315</v>
       </c>
       <c r="Q14" s="2">
-        <v>-0.1271854316610628</v>
+        <v>-0.1230057814950013</v>
       </c>
       <c r="R14" s="2">
-        <v>-0.1173630730764658</v>
+        <v>-0.1128898733858209</v>
       </c>
       <c r="S14" s="2">
-        <v>0.4437889072981735</v>
+        <v>0.4367398812841394</v>
       </c>
       <c r="T14" s="2">
-        <v>-0.135415431646576</v>
+        <v>-0.1346471757517568</v>
       </c>
       <c r="U14" s="2">
-        <v>-0.2922288077703387</v>
+        <v>-0.289452800892835</v>
       </c>
     </row>
     <row r="15" spans="1:21">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B15" s="2">
-        <v>0.009584646447675359</v>
+        <v>0.008720575418330557</v>
       </c>
       <c r="C15" s="2">
-        <v>-0.02685617461986891</v>
+        <v>-0.02824889606400737</v>
       </c>
       <c r="D15" s="2">
-        <v>-0.03686496465253911</v>
+        <v>-0.03719089081106493</v>
       </c>
       <c r="E15" s="2">
-        <v>0.03399140212411957</v>
+        <v>0.03408876177247213</v>
       </c>
       <c r="F15" s="2">
-        <v>0.0197771985145627</v>
+        <v>0.01855625776085682</v>
       </c>
       <c r="G15" s="2">
-        <v>-0.03348573201749485</v>
+        <v>-0.03372260379160047</v>
       </c>
       <c r="H15" s="2">
-        <v>-0.03337555719644102</v>
+        <v>-0.03399474920195936</v>
       </c>
       <c r="I15" s="2">
-        <v>-0.05985552146339091</v>
+        <v>-0.05951069382568925</v>
       </c>
       <c r="J15" s="2">
-        <v>-0.004364604780607586</v>
+        <v>-0.003678721405237023</v>
       </c>
       <c r="K15" s="2">
-        <v>-0.01976407610881415</v>
+        <v>-0.02020794712335095</v>
       </c>
       <c r="L15" s="2">
-        <v>-0.04682185619165259</v>
+        <v>-0.04736336177182777</v>
       </c>
       <c r="M15" s="2">
-        <v>-0.03593945832635657</v>
+        <v>-0.03577601559653747</v>
       </c>
       <c r="N15" s="2">
-        <v>-0.03081308414888551</v>
+        <v>-0.03205137004009748</v>
       </c>
       <c r="O15" s="2">
         <v>1</v>
       </c>
       <c r="P15" s="2">
-        <v>0.7424715126143425</v>
+        <v>0.7395611554326234</v>
       </c>
       <c r="Q15" s="2">
-        <v>0.207619419681204</v>
+        <v>0.2022336728240978</v>
       </c>
       <c r="R15" s="2">
-        <v>0.1132686137363011</v>
+        <v>0.1085441373330153</v>
       </c>
       <c r="S15" s="2">
-        <v>0.02451464751199372</v>
+        <v>0.02748929588193674</v>
       </c>
       <c r="T15" s="2">
-        <v>0.120520316877116</v>
+        <v>0.1210233072578733</v>
       </c>
       <c r="U15" s="2">
-        <v>0.172096873654907</v>
+        <v>0.1676753538624426</v>
       </c>
     </row>
     <row r="16" spans="1:21">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B16" s="2">
-        <v>-0.04636172981650317</v>
+        <v>-0.04506667671579052</v>
       </c>
       <c r="C16" s="2">
-        <v>-0.08539910297957878</v>
+        <v>-0.08341305607916655</v>
       </c>
       <c r="D16" s="2">
-        <v>-0.1001351572198626</v>
+        <v>-0.09814503936050406</v>
       </c>
       <c r="E16" s="2">
-        <v>-0.04383561262469876</v>
+        <v>-0.04266035602041702</v>
       </c>
       <c r="F16" s="2">
-        <v>-0.02575807527443629</v>
+        <v>-0.02456960704491969</v>
       </c>
       <c r="G16" s="2">
-        <v>-0.1015550428804258</v>
+        <v>-0.0987636496596019</v>
       </c>
       <c r="H16" s="2">
-        <v>-0.09330109406670307</v>
+        <v>-0.09187391203733189</v>
       </c>
       <c r="I16" s="2">
-        <v>-0.09475373588990976</v>
+        <v>-0.0920500071833109</v>
       </c>
       <c r="J16" s="2">
-        <v>-0.07836931226757186</v>
+        <v>-0.07642551925864281</v>
       </c>
       <c r="K16" s="2">
-        <v>-0.06090999096451501</v>
+        <v>-0.05876270085485161</v>
       </c>
       <c r="L16" s="2">
-        <v>-0.1498223095093448</v>
+        <v>-0.1480923084546124</v>
       </c>
       <c r="M16" s="2">
-        <v>-0.09976166813954949</v>
+        <v>-0.09856543192274309</v>
       </c>
       <c r="N16" s="2">
-        <v>-0.09716423714058922</v>
+        <v>-0.09573142285310315</v>
       </c>
       <c r="O16" s="2">
-        <v>0.7424715126143425</v>
+        <v>0.7395611554326234</v>
       </c>
       <c r="P16" s="2">
         <v>1</v>
       </c>
       <c r="Q16" s="2">
-        <v>0.6512417756146097</v>
+        <v>0.6510818536523723</v>
       </c>
       <c r="R16" s="2">
-        <v>0.5100493405091145</v>
+        <v>0.5104391547759107</v>
       </c>
       <c r="S16" s="2">
-        <v>-0.08284421304510328</v>
+        <v>-0.07907903964650614</v>
       </c>
       <c r="T16" s="2">
-        <v>0.1457178241640426</v>
+        <v>0.1436952554002458</v>
       </c>
       <c r="U16" s="2">
-        <v>0.1206242108250695</v>
+        <v>0.1159300913489198</v>
       </c>
     </row>
     <row r="17" spans="1:21">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B17" s="2">
-        <v>-0.09614128262587439</v>
+        <v>-0.09296776454437576</v>
       </c>
       <c r="C17" s="2">
-        <v>-0.1736003111989576</v>
+        <v>-0.1669728157126054</v>
       </c>
       <c r="D17" s="2">
-        <v>-0.1683106841155229</v>
+        <v>-0.1618658671180353</v>
       </c>
       <c r="E17" s="2">
-        <v>-0.1376246887187236</v>
+        <v>-0.1331638473484328</v>
       </c>
       <c r="F17" s="2">
-        <v>-0.05243182518594684</v>
+        <v>-0.05024814655886989</v>
       </c>
       <c r="G17" s="2">
-        <v>-0.16373171378621</v>
+        <v>-0.1569293347194135</v>
       </c>
       <c r="H17" s="2">
-        <v>-0.1755445867819954</v>
+        <v>-0.1688919112178923</v>
       </c>
       <c r="I17" s="2">
-        <v>-0.065227516494911</v>
+        <v>-0.0631135836438298</v>
       </c>
       <c r="J17" s="2">
-        <v>-0.1258387040793985</v>
+        <v>-0.1238126821986896</v>
       </c>
       <c r="K17" s="2">
-        <v>-0.05272349172566651</v>
+        <v>-0.04906326386447808</v>
       </c>
       <c r="L17" s="2">
-        <v>-0.1788703147083445</v>
+        <v>-0.1752914157207034</v>
       </c>
       <c r="M17" s="2">
-        <v>-0.1348354759399666</v>
+        <v>-0.132987825107985</v>
       </c>
       <c r="N17" s="2">
-        <v>-0.1271854316610628</v>
+        <v>-0.1230057814950013</v>
       </c>
       <c r="O17" s="2">
-        <v>0.207619419681204</v>
+        <v>0.2022336728240978</v>
       </c>
       <c r="P17" s="2">
-        <v>0.6512417756146097</v>
+        <v>0.6510818536523723</v>
       </c>
       <c r="Q17" s="2">
         <v>1</v>
       </c>
       <c r="R17" s="2">
-        <v>0.9395145283042745</v>
+        <v>0.9400664376200487</v>
       </c>
       <c r="S17" s="2">
-        <v>-0.1362471558555408</v>
+        <v>-0.1366429986766272</v>
       </c>
       <c r="T17" s="2">
-        <v>0.2117246607922079</v>
+        <v>0.2049573165761073</v>
       </c>
       <c r="U17" s="2">
-        <v>0.1119780280857743</v>
+        <v>0.1097506514905035</v>
       </c>
     </row>
     <row r="18" spans="1:21">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B18" s="2">
-        <v>-0.07146393462854077</v>
+        <v>-0.06844342659119444</v>
       </c>
       <c r="C18" s="2">
-        <v>-0.1597453856879754</v>
+        <v>-0.1530995276764361</v>
       </c>
       <c r="D18" s="2">
-        <v>-0.1353218322228005</v>
+        <v>-0.1286849343882467</v>
       </c>
       <c r="E18" s="2">
-        <v>-0.1328746699994343</v>
+        <v>-0.1282930343377397</v>
       </c>
       <c r="F18" s="2">
-        <v>-0.02353782628363642</v>
+        <v>-0.02164763978431109</v>
       </c>
       <c r="G18" s="2">
-        <v>-0.1482563302733315</v>
+        <v>-0.1419150028229105</v>
       </c>
       <c r="H18" s="2">
-        <v>-0.1457213353633865</v>
+        <v>-0.1382991339059669</v>
       </c>
       <c r="I18" s="2">
-        <v>-0.06957690766914951</v>
+        <v>-0.06846292883645531</v>
       </c>
       <c r="J18" s="2">
-        <v>-0.1435313280683901</v>
+        <v>-0.1423558442270655</v>
       </c>
       <c r="K18" s="2">
-        <v>-0.05599951351804124</v>
+        <v>-0.05280389386797559</v>
       </c>
       <c r="L18" s="2">
-        <v>-0.1603338311723812</v>
+        <v>-0.1568476382277995</v>
       </c>
       <c r="M18" s="2">
-        <v>-0.1364211933548994</v>
+        <v>-0.1348365253180284</v>
       </c>
       <c r="N18" s="2">
-        <v>-0.1173630730764658</v>
+        <v>-0.1128898733858209</v>
       </c>
       <c r="O18" s="2">
-        <v>0.1132686137363011</v>
+        <v>0.1085441373330153</v>
       </c>
       <c r="P18" s="2">
-        <v>0.5100493405091145</v>
+        <v>0.5104391547759107</v>
       </c>
       <c r="Q18" s="2">
-        <v>0.9395145283042745</v>
+        <v>0.9400664376200487</v>
       </c>
       <c r="R18" s="2">
         <v>1</v>
       </c>
       <c r="S18" s="2">
-        <v>-0.1717180651242541</v>
+        <v>-0.1731324640194044</v>
       </c>
       <c r="T18" s="2">
-        <v>0.2343069536878847</v>
+        <v>0.2271900752316423</v>
       </c>
       <c r="U18" s="2">
-        <v>0.09845462045055045</v>
+        <v>0.09815132479134112</v>
       </c>
     </row>
     <row r="19" spans="1:21">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B19" s="2">
-        <v>0.3378905257949931</v>
+        <v>0.3345626558024875</v>
       </c>
       <c r="C19" s="2">
-        <v>0.3514232350344638</v>
+        <v>0.341024462184917</v>
       </c>
       <c r="D19" s="2">
-        <v>0.2679064134892237</v>
+        <v>0.2620500041526474</v>
       </c>
       <c r="E19" s="2">
-        <v>0.3666724964036682</v>
+        <v>0.3572246201059924</v>
       </c>
       <c r="F19" s="2">
-        <v>0.2766323047085008</v>
+        <v>0.2760077792474183</v>
       </c>
       <c r="G19" s="2">
-        <v>0.3450360379753788</v>
+        <v>0.3393877351057602</v>
       </c>
       <c r="H19" s="2">
-        <v>0.2972792739820233</v>
+        <v>0.2867071752857003</v>
       </c>
       <c r="I19" s="2">
-        <v>0.4954537940781372</v>
+        <v>0.4994654824723255</v>
       </c>
       <c r="J19" s="2">
-        <v>0.4578966518656354</v>
+        <v>0.4583092063084198</v>
       </c>
       <c r="K19" s="2">
-        <v>0.4370170967980802</v>
+        <v>0.4347102962326969</v>
       </c>
       <c r="L19" s="2">
-        <v>0.4534461334711919</v>
+        <v>0.4509364578920367</v>
       </c>
       <c r="M19" s="2">
-        <v>0.4721410661116966</v>
+        <v>0.4699504830762667</v>
       </c>
       <c r="N19" s="2">
-        <v>0.4437889072981735</v>
+        <v>0.4367398812841394</v>
       </c>
       <c r="O19" s="2">
-        <v>0.02451464751199372</v>
+        <v>0.02748929588193674</v>
       </c>
       <c r="P19" s="2">
-        <v>-0.08284421304510328</v>
+        <v>-0.07907903964650614</v>
       </c>
       <c r="Q19" s="2">
-        <v>-0.1362471558555408</v>
+        <v>-0.1366429986766272</v>
       </c>
       <c r="R19" s="2">
-        <v>-0.1717180651242541</v>
+        <v>-0.1731324640194044</v>
       </c>
       <c r="S19" s="2">
         <v>1</v>
       </c>
       <c r="T19" s="2">
-        <v>-0.0438591718977256</v>
+        <v>-0.03836690585684775</v>
       </c>
       <c r="U19" s="2">
-        <v>-9.969907324492184E-05</v>
+        <v>-0.02834016125905013</v>
       </c>
     </row>
     <row r="20" spans="1:21">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B20" s="2">
-        <v>-0.1689177870014295</v>
+        <v>-0.1684954070223643</v>
       </c>
       <c r="C20" s="2">
-        <v>-0.1981611543076019</v>
+        <v>-0.2008957269764446</v>
       </c>
       <c r="D20" s="2">
-        <v>-0.1626674642662103</v>
+        <v>-0.165540027193309</v>
       </c>
       <c r="E20" s="2">
-        <v>-0.2092861314366406</v>
+        <v>-0.2124948053634381</v>
       </c>
       <c r="F20" s="2">
-        <v>-0.146445277653909</v>
+        <v>-0.1441775053990973</v>
       </c>
       <c r="G20" s="2">
-        <v>-0.2079441875225685</v>
+        <v>-0.211484808454069</v>
       </c>
       <c r="H20" s="2">
-        <v>-0.1617932016412099</v>
+        <v>-0.1642219365556789</v>
       </c>
       <c r="I20" s="2">
-        <v>-0.1736059617525851</v>
+        <v>-0.1715162899394772</v>
       </c>
       <c r="J20" s="2">
-        <v>-0.1855801250491936</v>
+        <v>-0.1856748158515933</v>
       </c>
       <c r="K20" s="2">
-        <v>-0.1601272046384987</v>
+        <v>-0.1608806417179749</v>
       </c>
       <c r="L20" s="2">
-        <v>-0.1278049496399567</v>
+        <v>-0.1263581861766898</v>
       </c>
       <c r="M20" s="2">
-        <v>-0.127974512981622</v>
+        <v>-0.1272492165258428</v>
       </c>
       <c r="N20" s="2">
-        <v>-0.135415431646576</v>
+        <v>-0.1346471757517568</v>
       </c>
       <c r="O20" s="2">
-        <v>0.120520316877116</v>
+        <v>0.1210233072578733</v>
       </c>
       <c r="P20" s="2">
-        <v>0.1457178241640426</v>
+        <v>0.1436952554002458</v>
       </c>
       <c r="Q20" s="2">
-        <v>0.2117246607922079</v>
+        <v>0.2049573165761073</v>
       </c>
       <c r="R20" s="2">
-        <v>0.2343069536878847</v>
+        <v>0.2271900752316423</v>
       </c>
       <c r="S20" s="2">
-        <v>-0.0438591718977256</v>
+        <v>-0.03836690585684775</v>
       </c>
       <c r="T20" s="2">
         <v>1</v>
       </c>
       <c r="U20" s="2">
-        <v>0.3360628322257901</v>
+        <v>0.3297098513205868</v>
       </c>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B21" s="2">
-        <v>-0.32037206049654</v>
+        <v>-0.3189467570670729</v>
       </c>
       <c r="C21" s="2">
-        <v>-0.1248352240258522</v>
+        <v>-0.1220064155989652</v>
       </c>
       <c r="D21" s="2">
-        <v>-0.3648494781702741</v>
+        <v>-0.3609812152018139</v>
       </c>
       <c r="E21" s="2">
-        <v>-0.09148888749273987</v>
+        <v>-0.09041687676338699</v>
       </c>
       <c r="F21" s="2">
-        <v>-0.3771733162097329</v>
+        <v>-0.3754013538160224</v>
       </c>
       <c r="G21" s="2">
-        <v>-0.2393903818647102</v>
+        <v>-0.2397542147734855</v>
       </c>
       <c r="H21" s="2">
-        <v>-0.3054183134562681</v>
+        <v>-0.2984254417000554</v>
       </c>
       <c r="I21" s="2">
-        <v>-0.1774641860773877</v>
+        <v>-0.1871526740657589</v>
       </c>
       <c r="J21" s="2">
-        <v>-0.1878604972332749</v>
+        <v>-0.1943101739563054</v>
       </c>
       <c r="K21" s="2">
-        <v>-0.2438946616192481</v>
+        <v>-0.2468058826896434</v>
       </c>
       <c r="L21" s="2">
-        <v>-0.2446089130537028</v>
+        <v>-0.2462754075621131</v>
       </c>
       <c r="M21" s="2">
-        <v>-0.2550757132832688</v>
+        <v>-0.2573729833527058</v>
       </c>
       <c r="N21" s="2">
-        <v>-0.2922288077703387</v>
+        <v>-0.289452800892835</v>
       </c>
       <c r="O21" s="2">
-        <v>0.172096873654907</v>
+        <v>0.1676753538624426</v>
       </c>
       <c r="P21" s="2">
-        <v>0.1206242108250695</v>
+        <v>0.1159300913489198</v>
       </c>
       <c r="Q21" s="2">
-        <v>0.1119780280857743</v>
+        <v>0.1097506514905035</v>
       </c>
       <c r="R21" s="2">
-        <v>0.09845462045055045</v>
+        <v>0.09815132479134112</v>
       </c>
       <c r="S21" s="2">
-        <v>-9.969907324492184E-05</v>
+        <v>-0.02834016125905013</v>
       </c>
       <c r="T21" s="2">
-        <v>0.3360628322257901</v>
+        <v>0.3297098513205868</v>
       </c>
       <c r="U21" s="2">
         <v>1</v>
@@ -5223,67 +5550,67 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -9876,13 +10203,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>

<commit_message>
Add comparison benchmarks: stock/bond blends and all-world equity
Seven benchmarks built from the existing sleeves (comparison only):
- FI 100 / 20/80 / 40/60 / 60/40 / 80/20: US market + 5-year Treasury,
  rebalanced monthly, from 1962-02; US 100 = US market from 1926-07.
- World: US, developed ex-US and EM markets weighted by each region's
  total market value from French's files (US share 33% in 1990 -> 56%
  in 2026), from 1990-07.
- Checked against real funds: 60/40 vs VBINX corr 0.996 (8.3% vs 8.4%
  /yr, 1992-2026); World vs VT corr 0.993 (8.7% vs 8.8%, 2008-2026).

App: Benchmark menu grouped into Benchmarks and Sleeves; all benchmarks
marked on the frontier; new Benchmarks panel comparing the portfolio with
each over the same months, plus a calendar-year table. Benchmarks that
start after the window say so rather than showing partial numbers.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtyJ36mjEj9LzVccKuq7PT
</commit_message>
<xml_diff>
--- a/data/processed/stats.xlsx
+++ b/data/processed/stats.xlsx
@@ -19,14 +19,17 @@
     <sheet name="Annual_Check" sheetId="10" r:id="rId10"/>
     <sheet name="Size_Lag_Check" sheetId="11" r:id="rId11"/>
     <sheet name="Commodities_Splice" sheetId="12" r:id="rId12"/>
-    <sheet name="Trend_Splice" sheetId="13" r:id="rId13"/>
+    <sheet name="Benchmarks_Full" sheetId="13" r:id="rId13"/>
+    <sheet name="Benchmarks_Calendar" sheetId="14" r:id="rId14"/>
+    <sheet name="Benchmark_Checks" sheetId="15" r:id="rId15"/>
+    <sheet name="Trend_Splice" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="177">
   <si>
     <t>note</t>
   </si>
@@ -181,10 +184,16 @@
     <t>202605</t>
   </si>
   <si>
-    <t>2026-10-30T02:15:19</t>
+    <t>2026-10-30T02:30:35</t>
   </si>
   <si>
-    <t>2026-10-30T02:15:20</t>
+    <t>2026-10-30T02:30:36</t>
+  </si>
+  <si>
+    <t>2026-10-30T02:30:37</t>
+  </si>
+  <si>
+    <t>2026-10-30T02:30:38</t>
   </si>
   <si>
     <t>start</t>
@@ -389,6 +398,63 @@
   </si>
   <si>
     <t>0.4% / 6.6%</t>
+  </si>
+  <si>
+    <t>BM_FI100</t>
+  </si>
+  <si>
+    <t>BM_20_80</t>
+  </si>
+  <si>
+    <t>BM_40_60</t>
+  </si>
+  <si>
+    <t>BM_60_40</t>
+  </si>
+  <si>
+    <t>BM_80_20</t>
+  </si>
+  <si>
+    <t>BM_EQ100</t>
+  </si>
+  <si>
+    <t>BM_World</t>
+  </si>
+  <si>
+    <t>fund</t>
+  </si>
+  <si>
+    <t>from</t>
+  </si>
+  <si>
+    <t>to</t>
+  </si>
+  <si>
+    <t>CAGR_built</t>
+  </si>
+  <si>
+    <t>CAGR_fund</t>
+  </si>
+  <si>
+    <t>vol_built</t>
+  </si>
+  <si>
+    <t>vol_fund</t>
+  </si>
+  <si>
+    <t>benchmark</t>
+  </si>
+  <si>
+    <t>VBINX</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>1992-10</t>
+  </si>
+  <si>
+    <t>2008-07</t>
   </si>
   <si>
     <t>2010 factor / AQMIX</t>
@@ -930,21 +996,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B2">
         <v>99</v>
@@ -958,7 +1024,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B3">
         <v>99</v>
@@ -972,7 +1038,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>99</v>
@@ -986,7 +1052,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B5">
         <v>99</v>
@@ -1000,7 +1066,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B6">
         <v>62</v>
@@ -1014,7 +1080,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B7">
         <v>62</v>
@@ -1028,7 +1094,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B8">
         <v>35</v>
@@ -1042,7 +1108,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B9">
         <v>35</v>
@@ -1056,7 +1122,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B10">
         <v>36</v>
@@ -1070,7 +1136,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -1101,19 +1167,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="E1" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1166,23 +1232,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B3">
         <v>39</v>
@@ -1190,58 +1256,58 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B4">
-        <v>0.8593971379562713</v>
+        <v>0.8593974426563644</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B5">
-        <v>0.06226038908748011</v>
+        <v>0.06226033065836247</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6">
-        <v>0.03427818111792311</v>
+        <v>0.03427818511853675</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1250,6 +1316,2264 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="6" width="12.7109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2">
+        <v>776</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.05482375892730773</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.05310849875295689</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0.2251862498175984</v>
+      </c>
+      <c r="H2" s="1">
+        <v>-0.1461807592457053</v>
+      </c>
+      <c r="I2" s="1">
+        <v>-0.1143645431823892</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3">
+        <v>776</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.06718874556416066</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.05481264589181195</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0.4336760600882943</v>
+      </c>
+      <c r="H3" s="1">
+        <v>-0.1408634303897456</v>
+      </c>
+      <c r="I3" s="1">
+        <v>-0.1265993975406244</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4">
+        <v>776</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.07860960793836869</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.07212246320110707</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0.4903585705936396</v>
+      </c>
+      <c r="H4" s="1">
+        <v>-0.1888128809785479</v>
+      </c>
+      <c r="I4" s="1">
+        <v>-0.1753400252209177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5">
+        <v>776</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.08904354069227938</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.09701640729997395</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0.4847732509370196</v>
+      </c>
+      <c r="H5" s="1">
+        <v>-0.2965848785813319</v>
+      </c>
+      <c r="I5" s="1">
+        <v>-0.2614408759453398</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6">
+        <v>776</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.09844677483520337</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.1250440998658448</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.4699317919662618</v>
+      </c>
+      <c r="H6" s="1">
+        <v>-0.4073526740236613</v>
+      </c>
+      <c r="I6" s="1">
+        <v>-0.3467859496799597</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7">
+        <v>1203</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.1035912957550589</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.1832365805253884</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.4537367752389381</v>
+      </c>
+      <c r="H7" s="1">
+        <v>-0.8365224657023862</v>
+      </c>
+      <c r="I7" s="1">
+        <v>-0.6573974517625623</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8">
+        <v>435</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.08411669585931425</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.1515488583112376</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.4372517717288407</v>
+      </c>
+      <c r="H8" s="1">
+        <v>-0.5452239152850423</v>
+      </c>
+      <c r="I8" s="1">
+        <v>-0.4800238871239021</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H100"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="8" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2">
+        <v>1927</v>
+      </c>
+      <c r="G2">
+        <v>0.3258372260927358</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3">
+        <v>1928</v>
+      </c>
+      <c r="G3">
+        <v>0.3907859670535343</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4">
+        <v>1929</v>
+      </c>
+      <c r="G4">
+        <v>-0.1485230019924366</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5">
+        <v>1930</v>
+      </c>
+      <c r="G5">
+        <v>-0.2872601404747539</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6">
+        <v>1931</v>
+      </c>
+      <c r="G6">
+        <v>-0.4376338865587707</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7">
+        <v>1932</v>
+      </c>
+      <c r="G7">
+        <v>-0.08658574309335187</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8">
+        <v>1933</v>
+      </c>
+      <c r="G8">
+        <v>0.5679565173050356</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9">
+        <v>1934</v>
+      </c>
+      <c r="G9">
+        <v>0.03263777211935426</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10">
+        <v>1935</v>
+      </c>
+      <c r="G10">
+        <v>0.4500465652631138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11">
+        <v>1936</v>
+      </c>
+      <c r="G11">
+        <v>0.3215330595896722</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12">
+        <v>1937</v>
+      </c>
+      <c r="G12">
+        <v>-0.3472891622823772</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13">
+        <v>1938</v>
+      </c>
+      <c r="G13">
+        <v>0.2816784749277403</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14">
+        <v>1939</v>
+      </c>
+      <c r="G14">
+        <v>0.02505468821084089</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15">
+        <v>1940</v>
+      </c>
+      <c r="G15">
+        <v>-0.07206559093168263</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16">
+        <v>1941</v>
+      </c>
+      <c r="G16">
+        <v>-0.1055018394556686</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17">
+        <v>1942</v>
+      </c>
+      <c r="G17">
+        <v>0.1649378017045231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18">
+        <v>1943</v>
+      </c>
+      <c r="G18">
+        <v>0.2831996487499311</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19">
+        <v>1944</v>
+      </c>
+      <c r="G19">
+        <v>0.2134477108795263</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20">
+        <v>1945</v>
+      </c>
+      <c r="G20">
+        <v>0.3873569957118941</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21">
+        <v>1946</v>
+      </c>
+      <c r="G21">
+        <v>-0.06396093599835906</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>1947</v>
+      </c>
+      <c r="G22">
+        <v>0.03433766682547623</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23">
+        <v>1948</v>
+      </c>
+      <c r="G23">
+        <v>0.01855188283887887</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24">
+        <v>1949</v>
+      </c>
+      <c r="G24">
+        <v>0.2019866413495468</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25">
+        <v>1950</v>
+      </c>
+      <c r="G25">
+        <v>0.3006678408427548</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26">
+        <v>1951</v>
+      </c>
+      <c r="G26">
+        <v>0.2069446316447421</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27">
+        <v>1952</v>
+      </c>
+      <c r="G27">
+        <v>0.1347490574608889</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28">
+        <v>1953</v>
+      </c>
+      <c r="G28">
+        <v>0.007186150650095646</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29">
+        <v>1954</v>
+      </c>
+      <c r="G29">
+        <v>0.503056319732156</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30">
+        <v>1955</v>
+      </c>
+      <c r="G30">
+        <v>0.2535560147425555</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31">
+        <v>1956</v>
+      </c>
+      <c r="G31">
+        <v>0.08337524461505508</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32">
+        <v>1957</v>
+      </c>
+      <c r="G32">
+        <v>-0.1000407578408515</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33">
+        <v>1958</v>
+      </c>
+      <c r="G33">
+        <v>0.4498099989508733</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34">
+        <v>1959</v>
+      </c>
+      <c r="G34">
+        <v>0.1276065549467555</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35">
+        <v>1960</v>
+      </c>
+      <c r="G35">
+        <v>0.0120096817509785</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36">
+        <v>1961</v>
+      </c>
+      <c r="G36">
+        <v>0.2693875395017462</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37">
+        <v>1962</v>
+      </c>
+      <c r="G37">
+        <v>-0.1018704309519154</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38">
+        <v>1963</v>
+      </c>
+      <c r="B38">
+        <v>0.01596314470176896</v>
+      </c>
+      <c r="C38">
+        <v>0.05296842081998476</v>
+      </c>
+      <c r="D38">
+        <v>0.09083021606443742</v>
+      </c>
+      <c r="E38">
+        <v>0.1295520257202833</v>
+      </c>
+      <c r="F38">
+        <v>0.1691368422338544</v>
+      </c>
+      <c r="G38">
+        <v>0.2095871431453795</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39">
+        <v>1964</v>
+      </c>
+      <c r="B39">
+        <v>0.03872754652216259</v>
+      </c>
+      <c r="C39">
+        <v>0.06226000277548605</v>
+      </c>
+      <c r="D39">
+        <v>0.08622109444618165</v>
+      </c>
+      <c r="E39">
+        <v>0.1106165431678208</v>
+      </c>
+      <c r="F39">
+        <v>0.1354521107732587</v>
+      </c>
+      <c r="G39">
+        <v>0.1607335989631846</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40">
+        <v>1965</v>
+      </c>
+      <c r="B40">
+        <v>0.008969981844349606</v>
+      </c>
+      <c r="C40">
+        <v>0.03547046753458383</v>
+      </c>
+      <c r="D40">
+        <v>0.06227190835961172</v>
+      </c>
+      <c r="E40">
+        <v>0.08936180817301342</v>
+      </c>
+      <c r="F40">
+        <v>0.1167268495791589</v>
+      </c>
+      <c r="G40">
+        <v>0.144352872447127</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41">
+        <v>1966</v>
+      </c>
+      <c r="B41">
+        <v>0.05579973864792831</v>
+      </c>
+      <c r="C41">
+        <v>0.02623440452793813</v>
+      </c>
+      <c r="D41">
+        <v>-0.002941994767466594</v>
+      </c>
+      <c r="E41">
+        <v>-0.03172155666839527</v>
+      </c>
+      <c r="F41">
+        <v>-0.06009681438016279</v>
+      </c>
+      <c r="G41">
+        <v>-0.08806073452750751</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42">
+        <v>1967</v>
+      </c>
+      <c r="B42">
+        <v>0.008483485773714827</v>
+      </c>
+      <c r="C42">
+        <v>0.06027128717515651</v>
+      </c>
+      <c r="D42">
+        <v>0.1139764816769273</v>
+      </c>
+      <c r="E42">
+        <v>0.1696355759919608</v>
+      </c>
+      <c r="F42">
+        <v>0.2272842268344679</v>
+      </c>
+      <c r="G42">
+        <v>0.2869571477452084</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43">
+        <v>1968</v>
+      </c>
+      <c r="B43">
+        <v>0.03399151180147597</v>
+      </c>
+      <c r="C43">
+        <v>0.05636376081423333</v>
+      </c>
+      <c r="D43">
+        <v>0.07831552061741132</v>
+      </c>
+      <c r="E43">
+        <v>0.09981692185872015</v>
+      </c>
+      <c r="F43">
+        <v>0.1208384229742236</v>
+      </c>
+      <c r="G43">
+        <v>0.1413508533397874</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44">
+        <v>1969</v>
+      </c>
+      <c r="B44">
+        <v>-0.008535237276688701</v>
+      </c>
+      <c r="C44">
+        <v>-0.02829241057654774</v>
+      </c>
+      <c r="D44">
+        <v>-0.04829386377671419</v>
+      </c>
+      <c r="E44">
+        <v>-0.06851742455856624</v>
+      </c>
+      <c r="F44">
+        <v>-0.08894085274784724</v>
+      </c>
+      <c r="G44">
+        <v>-0.1095418650330425</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45">
+        <v>1970</v>
+      </c>
+      <c r="B45">
+        <v>0.1791787278820318</v>
+      </c>
+      <c r="C45">
+        <v>0.1442499619402062</v>
+      </c>
+      <c r="D45">
+        <v>0.1088761598523835</v>
+      </c>
+      <c r="E45">
+        <v>0.07313905820437272</v>
+      </c>
+      <c r="F45">
+        <v>0.03711993383199563</v>
+      </c>
+      <c r="G45">
+        <v>0.0008993764352729361</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46">
+        <v>1971</v>
+      </c>
+      <c r="B46">
+        <v>0.08232169351177943</v>
+      </c>
+      <c r="C46">
+        <v>0.0994377411681604</v>
+      </c>
+      <c r="D46">
+        <v>0.1159520042373707</v>
+      </c>
+      <c r="E46">
+        <v>0.131838493330501</v>
+      </c>
+      <c r="F46">
+        <v>0.147071925938639</v>
+      </c>
+      <c r="G46">
+        <v>0.1616277679367735</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47">
+        <v>1972</v>
+      </c>
+      <c r="B47">
+        <v>0.02768211514310681</v>
+      </c>
+      <c r="C47">
+        <v>0.05506003643351476</v>
+      </c>
+      <c r="D47">
+        <v>0.08289576245925412</v>
+      </c>
+      <c r="E47">
+        <v>0.1111904504276859</v>
+      </c>
+      <c r="F47">
+        <v>0.1399451124788722</v>
+      </c>
+      <c r="G47">
+        <v>0.1691606132961412</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48">
+        <v>1973</v>
+      </c>
+      <c r="B48">
+        <v>0.0451092556470496</v>
+      </c>
+      <c r="C48">
+        <v>-0.004580313316982054</v>
+      </c>
+      <c r="D48">
+        <v>-0.05330687065100259</v>
+      </c>
+      <c r="E48">
+        <v>-0.1010084951139595</v>
+      </c>
+      <c r="F48">
+        <v>-0.1476295032303292</v>
+      </c>
+      <c r="G48">
+        <v>-0.1931202152998392</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49">
+        <v>1974</v>
+      </c>
+      <c r="B49">
+        <v>0.05731689230463521</v>
+      </c>
+      <c r="C49">
+        <v>-0.01519413439155071</v>
+      </c>
+      <c r="D49">
+        <v>-0.0851175381392224</v>
+      </c>
+      <c r="E49">
+        <v>-0.1523051080255586</v>
+      </c>
+      <c r="F49">
+        <v>-0.2166431993009053</v>
+      </c>
+      <c r="G49">
+        <v>-0.2780494915166808</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50">
+        <v>1975</v>
+      </c>
+      <c r="B50">
+        <v>0.07369038246157067</v>
+      </c>
+      <c r="C50">
+        <v>0.1327360823963948</v>
+      </c>
+      <c r="D50">
+        <v>0.1932738150613982</v>
+      </c>
+      <c r="E50">
+        <v>0.255251258847079</v>
+      </c>
+      <c r="F50">
+        <v>0.3186105789406626</v>
+      </c>
+      <c r="G50">
+        <v>0.3832883780080145</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51">
+        <v>1976</v>
+      </c>
+      <c r="B51">
+        <v>0.1366127078135049</v>
+      </c>
+      <c r="C51">
+        <v>0.1639637440710386</v>
+      </c>
+      <c r="D51">
+        <v>0.1909812064949425</v>
+      </c>
+      <c r="E51">
+        <v>0.2176420125311094</v>
+      </c>
+      <c r="F51">
+        <v>0.2439234571811364</v>
+      </c>
+      <c r="G51">
+        <v>0.2698032315995844</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52">
+        <v>1977</v>
+      </c>
+      <c r="B52">
+        <v>0.01120144432326642</v>
+      </c>
+      <c r="C52">
+        <v>0.003006249096123348</v>
+      </c>
+      <c r="D52">
+        <v>-0.005334269266996872</v>
+      </c>
+      <c r="E52">
+        <v>-0.01381482781832555</v>
+      </c>
+      <c r="F52">
+        <v>-0.0224301603209236</v>
+      </c>
+      <c r="G52">
+        <v>-0.03117501976681369</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53">
+        <v>1978</v>
+      </c>
+      <c r="B53">
+        <v>0.01244082494516974</v>
+      </c>
+      <c r="C53">
+        <v>0.02815292806285119</v>
+      </c>
+      <c r="D53">
+        <v>0.04305938573619517</v>
+      </c>
+      <c r="E53">
+        <v>0.05711160494139089</v>
+      </c>
+      <c r="F53">
+        <v>0.07026106229996376</v>
+      </c>
+      <c r="G53">
+        <v>0.08245940100341231</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54">
+        <v>1979</v>
+      </c>
+      <c r="B54">
+        <v>0.05411383013561677</v>
+      </c>
+      <c r="C54">
+        <v>0.0890120159273422</v>
+      </c>
+      <c r="D54">
+        <v>0.1245226693766792</v>
+      </c>
+      <c r="E54">
+        <v>0.1606397105744335</v>
+      </c>
+      <c r="F54">
+        <v>0.1973564411053426</v>
+      </c>
+      <c r="G54">
+        <v>0.2346655354587941</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55">
+        <v>1980</v>
+      </c>
+      <c r="B55">
+        <v>0.02999612832269682</v>
+      </c>
+      <c r="C55">
+        <v>0.08999578635824745</v>
+      </c>
+      <c r="D55">
+        <v>0.1505418335842068</v>
+      </c>
+      <c r="E55">
+        <v>0.2113529550301039</v>
+      </c>
+      <c r="F55">
+        <v>0.272123286785988</v>
+      </c>
+      <c r="G55">
+        <v>0.3325223708647589</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56">
+        <v>1981</v>
+      </c>
+      <c r="B56">
+        <v>0.09479057826594861</v>
+      </c>
+      <c r="C56">
+        <v>0.06914212525826136</v>
+      </c>
+      <c r="D56">
+        <v>0.04356268109484063</v>
+      </c>
+      <c r="E56">
+        <v>0.01806907788315826</v>
+      </c>
+      <c r="F56">
+        <v>-0.007322178875985186</v>
+      </c>
+      <c r="G56">
+        <v>-0.0325949211030877</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57">
+        <v>1982</v>
+      </c>
+      <c r="B57">
+        <v>0.3090957058801094</v>
+      </c>
+      <c r="C57">
+        <v>0.2918622788987151</v>
+      </c>
+      <c r="D57">
+        <v>0.2737496548178446</v>
+      </c>
+      <c r="E57">
+        <v>0.2547992391124561</v>
+      </c>
+      <c r="F57">
+        <v>0.2350531971457903</v>
+      </c>
+      <c r="G57">
+        <v>0.2145543582405749</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58">
+        <v>1983</v>
+      </c>
+      <c r="B58">
+        <v>0.05298500745996915</v>
+      </c>
+      <c r="C58">
+        <v>0.08627308329690364</v>
+      </c>
+      <c r="D58">
+        <v>0.1201719243855652</v>
+      </c>
+      <c r="E58">
+        <v>0.1546792217215125</v>
+      </c>
+      <c r="F58">
+        <v>0.189792221553339</v>
+      </c>
+      <c r="G58">
+        <v>0.2255077190856862</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59">
+        <v>1984</v>
+      </c>
+      <c r="B59">
+        <v>0.149908050800257</v>
+      </c>
+      <c r="C59">
+        <v>0.128402839544467</v>
+      </c>
+      <c r="D59">
+        <v>0.1064619557357633</v>
+      </c>
+      <c r="E59">
+        <v>0.08413415316272199</v>
+      </c>
+      <c r="F59">
+        <v>0.0614666779048394</v>
+      </c>
+      <c r="G59">
+        <v>0.0385052691028358</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60">
+        <v>1985</v>
+      </c>
+      <c r="B60">
+        <v>0.2208820094991095</v>
+      </c>
+      <c r="C60">
+        <v>0.2424875152421322</v>
+      </c>
+      <c r="D60">
+        <v>0.2638459593919038</v>
+      </c>
+      <c r="E60">
+        <v>0.2849373154141686</v>
+      </c>
+      <c r="F60">
+        <v>0.3057415443059965</v>
+      </c>
+      <c r="G60">
+        <v>0.3262386133802919</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61">
+        <v>1986</v>
+      </c>
+      <c r="B61">
+        <v>0.149991521385427</v>
+      </c>
+      <c r="C61">
+        <v>0.1547128000434506</v>
+      </c>
+      <c r="D61">
+        <v>0.1585039638102932</v>
+      </c>
+      <c r="E61">
+        <v>0.1613521642417632</v>
+      </c>
+      <c r="F61">
+        <v>0.1632459012860048</v>
+      </c>
+      <c r="G61">
+        <v>0.1641750614524851</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62">
+        <v>1987</v>
+      </c>
+      <c r="B62">
+        <v>0.01643336726600375</v>
+      </c>
+      <c r="C62">
+        <v>0.02565564475944915</v>
+      </c>
+      <c r="D62">
+        <v>0.0306664473184064</v>
+      </c>
+      <c r="E62">
+        <v>0.03107257164068433</v>
+      </c>
+      <c r="F62">
+        <v>0.02647050983576937</v>
+      </c>
+      <c r="G62">
+        <v>0.0164476560239466</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63">
+        <v>1988</v>
+      </c>
+      <c r="B63">
+        <v>0.05302374893568063</v>
+      </c>
+      <c r="C63">
+        <v>0.07767662432634692</v>
+      </c>
+      <c r="D63">
+        <v>0.1026930167660352</v>
+      </c>
+      <c r="E63">
+        <v>0.1280733912147021</v>
+      </c>
+      <c r="F63">
+        <v>0.1538180849247046</v>
+      </c>
+      <c r="G63">
+        <v>0.1799273043809233</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64">
+        <v>1989</v>
+      </c>
+      <c r="B64">
+        <v>0.1444321340535573</v>
+      </c>
+      <c r="C64">
+        <v>0.1731892616936461</v>
+      </c>
+      <c r="D64">
+        <v>0.2020093860508332</v>
+      </c>
+      <c r="E64">
+        <v>0.230865576892378</v>
+      </c>
+      <c r="F64">
+        <v>0.2597300555278541</v>
+      </c>
+      <c r="G64">
+        <v>0.2885742032222949</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65">
+        <v>1990</v>
+      </c>
+      <c r="B65">
+        <v>0.09450938294858524</v>
+      </c>
+      <c r="C65">
+        <v>0.06381881860927163</v>
+      </c>
+      <c r="D65">
+        <v>0.03294713001653382</v>
+      </c>
+      <c r="E65">
+        <v>0.001946267322256334</v>
+      </c>
+      <c r="F65">
+        <v>-0.02913275383753888</v>
+      </c>
+      <c r="G65">
+        <v>-0.06023993422837426</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66">
+        <v>1991</v>
+      </c>
+      <c r="B66">
+        <v>0.1565975541786297</v>
+      </c>
+      <c r="C66">
+        <v>0.194732337930543</v>
+      </c>
+      <c r="D66">
+        <v>0.233007805347283</v>
+      </c>
+      <c r="E66">
+        <v>0.2713732983893644</v>
+      </c>
+      <c r="F66">
+        <v>0.3097766627876237</v>
+      </c>
+      <c r="G66">
+        <v>0.3481643112451338</v>
+      </c>
+      <c r="H66">
+        <v>0.1842989677204454</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67">
+        <v>1992</v>
+      </c>
+      <c r="B67">
+        <v>0.058538284073544</v>
+      </c>
+      <c r="C67">
+        <v>0.06692657794929646</v>
+      </c>
+      <c r="D67">
+        <v>0.07505168939199924</v>
+      </c>
+      <c r="E67">
+        <v>0.08290794822107106</v>
+      </c>
+      <c r="F67">
+        <v>0.09048978706893407</v>
+      </c>
+      <c r="G67">
+        <v>0.09779174543548419</v>
+      </c>
+      <c r="H67">
+        <v>-0.05602518161594505</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68">
+        <v>1993</v>
+      </c>
+      <c r="B68">
+        <v>0.09047464372571379</v>
+      </c>
+      <c r="C68">
+        <v>0.09507911634107202</v>
+      </c>
+      <c r="D68">
+        <v>0.09949618887866407</v>
+      </c>
+      <c r="E68">
+        <v>0.103723713789954</v>
+      </c>
+      <c r="F68">
+        <v>0.107759600111893</v>
+      </c>
+      <c r="G68">
+        <v>0.1116018143265147</v>
+      </c>
+      <c r="H68">
+        <v>0.2351511355326681</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69">
+        <v>1994</v>
+      </c>
+      <c r="B69">
+        <v>-0.04248263935540941</v>
+      </c>
+      <c r="C69">
+        <v>-0.03400156202489413</v>
+      </c>
+      <c r="D69">
+        <v>-0.02565674862770717</v>
+      </c>
+      <c r="E69">
+        <v>-0.01745242844774852</v>
+      </c>
+      <c r="F69">
+        <v>-0.009392807567437877</v>
+      </c>
+      <c r="G69">
+        <v>-0.001482066493663892</v>
+      </c>
+      <c r="H69">
+        <v>0.05366036868856217</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70">
+        <v>1995</v>
+      </c>
+      <c r="B70">
+        <v>0.1798037366119227</v>
+      </c>
+      <c r="C70">
+        <v>0.21586063844626</v>
+      </c>
+      <c r="D70">
+        <v>0.2527485898068851</v>
+      </c>
+      <c r="E70">
+        <v>0.2904794947164266</v>
+      </c>
+      <c r="F70">
+        <v>0.3290652494315727</v>
+      </c>
+      <c r="G70">
+        <v>0.3685177368764043</v>
+      </c>
+      <c r="H70">
+        <v>0.1780988733524507</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71">
+        <v>1996</v>
+      </c>
+      <c r="B71">
+        <v>0.0263013390062603</v>
+      </c>
+      <c r="C71">
+        <v>0.06208483928094721</v>
+      </c>
+      <c r="D71">
+        <v>0.09856495662650588</v>
+      </c>
+      <c r="E71">
+        <v>0.1357307084303099</v>
+      </c>
+      <c r="F71">
+        <v>0.1735696565856519</v>
+      </c>
+      <c r="G71">
+        <v>0.2120678553794846</v>
+      </c>
+      <c r="H71">
+        <v>0.1179281751994707</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72">
+        <v>1997</v>
+      </c>
+      <c r="B72">
+        <v>0.08635774012010766</v>
+      </c>
+      <c r="C72">
+        <v>0.1298938682556685</v>
+      </c>
+      <c r="D72">
+        <v>0.1742986757719704</v>
+      </c>
+      <c r="E72">
+        <v>0.2195478788921952</v>
+      </c>
+      <c r="F72">
+        <v>0.2656148489526029</v>
+      </c>
+      <c r="G72">
+        <v>0.3124705754048294</v>
+      </c>
+      <c r="H72">
+        <v>0.119320304738425</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73">
+        <v>1998</v>
+      </c>
+      <c r="B73">
+        <v>0.105931558725012</v>
+      </c>
+      <c r="C73">
+        <v>0.1377952570121421</v>
+      </c>
+      <c r="D73">
+        <v>0.1677100613723497</v>
+      </c>
+      <c r="E73">
+        <v>0.1953688553985671</v>
+      </c>
+      <c r="F73">
+        <v>0.2204479257647105</v>
+      </c>
+      <c r="G73">
+        <v>0.2426068290312333</v>
+      </c>
+      <c r="H73">
+        <v>0.1868581466985748</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74">
+        <v>1999</v>
+      </c>
+      <c r="B74">
+        <v>-0.02195072677628562</v>
+      </c>
+      <c r="C74">
+        <v>0.0294425393290827</v>
+      </c>
+      <c r="D74">
+        <v>0.08256459979498953</v>
+      </c>
+      <c r="E74">
+        <v>0.1374284528865075</v>
+      </c>
+      <c r="F74">
+        <v>0.1940452151641765</v>
+      </c>
+      <c r="G74">
+        <v>0.2524240515544416</v>
+      </c>
+      <c r="H74">
+        <v>0.3183676310450916</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75">
+        <v>2000</v>
+      </c>
+      <c r="B75">
+        <v>0.1268673918897096</v>
+      </c>
+      <c r="C75">
+        <v>0.07643527447429177</v>
+      </c>
+      <c r="D75">
+        <v>0.02688948829831528</v>
+      </c>
+      <c r="E75">
+        <v>-0.02171718001087641</v>
+      </c>
+      <c r="F75">
+        <v>-0.06933576768036798</v>
+      </c>
+      <c r="G75">
+        <v>-0.1159211246098051</v>
+      </c>
+      <c r="H75">
+        <v>-0.1465912393270606</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76">
+        <v>2001</v>
+      </c>
+      <c r="B76">
+        <v>0.07416337965434461</v>
+      </c>
+      <c r="C76">
+        <v>0.03883151472702395</v>
+      </c>
+      <c r="D76">
+        <v>0.002380487942543752</v>
+      </c>
+      <c r="E76">
+        <v>-0.03502190779994552</v>
+      </c>
+      <c r="F76">
+        <v>-0.07320860145226482</v>
+      </c>
+      <c r="G76">
+        <v>-0.1120139990433334</v>
+      </c>
+      <c r="H76">
+        <v>-0.1521191713645424</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77">
+        <v>2002</v>
+      </c>
+      <c r="B77">
+        <v>0.115320345901061</v>
+      </c>
+      <c r="C77">
+        <v>0.04646084697162811</v>
+      </c>
+      <c r="D77">
+        <v>-0.02082644958346402</v>
+      </c>
+      <c r="E77">
+        <v>-0.08634421583581164</v>
+      </c>
+      <c r="F77">
+        <v>-0.1499163223929004</v>
+      </c>
+      <c r="G77">
+        <v>-0.2113877500485872</v>
+      </c>
+      <c r="H77">
+        <v>-0.1648645765030684</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78">
+        <v>2003</v>
+      </c>
+      <c r="B78">
+        <v>0.007176581357773104</v>
+      </c>
+      <c r="C78">
+        <v>0.0646727309819326</v>
+      </c>
+      <c r="D78">
+        <v>0.124367998550829</v>
+      </c>
+      <c r="E78">
+        <v>0.1862916058742787</v>
+      </c>
+      <c r="F78">
+        <v>0.2504704870427417</v>
+      </c>
+      <c r="G78">
+        <v>0.3169291440246134</v>
+      </c>
+      <c r="H78">
+        <v>0.3815135221464241</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79">
+        <v>2004</v>
+      </c>
+      <c r="B79">
+        <v>0.01667004821020113</v>
+      </c>
+      <c r="C79">
+        <v>0.03719162972332701</v>
+      </c>
+      <c r="D79">
+        <v>0.05772945644694882</v>
+      </c>
+      <c r="E79">
+        <v>0.07827110469357534</v>
+      </c>
+      <c r="F79">
+        <v>0.09880384002066123</v>
+      </c>
+      <c r="G79">
+        <v>0.1193146188637602</v>
+      </c>
+      <c r="H79">
+        <v>0.1785002831868965</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80">
+        <v>2005</v>
+      </c>
+      <c r="B80">
+        <v>0.007899658751238325</v>
+      </c>
+      <c r="C80">
+        <v>0.01906964395380539</v>
+      </c>
+      <c r="D80">
+        <v>0.02997358498977953</v>
+      </c>
+      <c r="E80">
+        <v>0.04060327230821126</v>
+      </c>
+      <c r="F80">
+        <v>0.05095065255345688</v>
+      </c>
+      <c r="G80">
+        <v>0.0610078353075616</v>
+      </c>
+      <c r="H80">
+        <v>0.1298805161235121</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81">
+        <v>2006</v>
+      </c>
+      <c r="B81">
+        <v>0.03219517757581603</v>
+      </c>
+      <c r="C81">
+        <v>0.05589339765267276</v>
+      </c>
+      <c r="D81">
+        <v>0.07992237724236162</v>
+      </c>
+      <c r="E81">
+        <v>0.1042812580358636</v>
+      </c>
+      <c r="F81">
+        <v>0.1289690039282221</v>
+      </c>
+      <c r="G81">
+        <v>0.1539843968000569</v>
+      </c>
+      <c r="H81">
+        <v>0.2192940289128165</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82">
+        <v>2007</v>
+      </c>
+      <c r="B82">
+        <v>0.1041722875618969</v>
+      </c>
+      <c r="C82">
+        <v>0.09602440515239263</v>
+      </c>
+      <c r="D82">
+        <v>0.08726396839514217</v>
+      </c>
+      <c r="E82">
+        <v>0.07789778975628803</v>
+      </c>
+      <c r="F82">
+        <v>0.06793337159329682</v>
+      </c>
+      <c r="G82">
+        <v>0.05737890319654992</v>
+      </c>
+      <c r="H82">
+        <v>0.1252492200328073</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83">
+        <v>2008</v>
+      </c>
+      <c r="B83">
+        <v>0.1224460045419693</v>
+      </c>
+      <c r="C83">
+        <v>0.008245797654735876</v>
+      </c>
+      <c r="D83">
+        <v>-0.09738895921550517</v>
+      </c>
+      <c r="E83">
+        <v>-0.1948209535887682</v>
+      </c>
+      <c r="F83">
+        <v>-0.2844199852695848</v>
+      </c>
+      <c r="G83">
+        <v>-0.3665607845119463</v>
+      </c>
+      <c r="H83">
+        <v>-0.4181832135899017</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84">
+        <v>2009</v>
+      </c>
+      <c r="B84">
+        <v>-0.03163333855445394</v>
+      </c>
+      <c r="C84">
+        <v>0.0290446746637576</v>
+      </c>
+      <c r="D84">
+        <v>0.09131851167015781</v>
+      </c>
+      <c r="E84">
+        <v>0.155053040731979</v>
+      </c>
+      <c r="F84">
+        <v>0.220096250203889</v>
+      </c>
+      <c r="G84">
+        <v>0.2862788266190115</v>
+      </c>
+      <c r="H84">
+        <v>0.3618470176983573</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85">
+        <v>2010</v>
+      </c>
+      <c r="B85">
+        <v>0.05135132516523844</v>
+      </c>
+      <c r="C85">
+        <v>0.07900426919007608</v>
+      </c>
+      <c r="D85">
+        <v>0.1052356954291385</v>
+      </c>
+      <c r="E85">
+        <v>0.1299157236250041</v>
+      </c>
+      <c r="F85">
+        <v>0.1529176267232821</v>
+      </c>
+      <c r="G85">
+        <v>0.1741185592177583</v>
+      </c>
+      <c r="H85">
+        <v>0.1527105135475917</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86">
+        <v>2011</v>
+      </c>
+      <c r="B86">
+        <v>0.07390112555592965</v>
+      </c>
+      <c r="C86">
+        <v>0.06228352575522189</v>
+      </c>
+      <c r="D86">
+        <v>0.04953610122044827</v>
+      </c>
+      <c r="E86">
+        <v>0.0357080233828504</v>
+      </c>
+      <c r="F86">
+        <v>0.02084922429129854</v>
+      </c>
+      <c r="G86">
+        <v>0.005010313959058044</v>
+      </c>
+      <c r="H86">
+        <v>-0.08654616887477418</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87">
+        <v>2012</v>
+      </c>
+      <c r="B87">
+        <v>0.0126010382654218</v>
+      </c>
+      <c r="C87">
+        <v>0.04235339796530568</v>
+      </c>
+      <c r="D87">
+        <v>0.07234658087099133</v>
+      </c>
+      <c r="E87">
+        <v>0.1025518833220469</v>
+      </c>
+      <c r="F87">
+        <v>0.1329389782243442</v>
+      </c>
+      <c r="G87">
+        <v>0.1634758825967311</v>
+      </c>
+      <c r="H87">
+        <v>0.1719822496192716</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88">
+        <v>2013</v>
+      </c>
+      <c r="B88">
+        <v>-0.03740251669898598</v>
+      </c>
+      <c r="C88">
+        <v>0.03148375289506045</v>
+      </c>
+      <c r="D88">
+        <v>0.1045982573658413</v>
+      </c>
+      <c r="E88">
+        <v>0.1821583305893979</v>
+      </c>
+      <c r="F88">
+        <v>0.2643903158454619</v>
+      </c>
+      <c r="G88">
+        <v>0.3515298465112644</v>
+      </c>
+      <c r="H88">
+        <v>0.2466840524112641</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89">
+        <v>2014</v>
+      </c>
+      <c r="B89">
+        <v>0.02110419199381353</v>
+      </c>
+      <c r="C89">
+        <v>0.04031426035030594</v>
+      </c>
+      <c r="D89">
+        <v>0.05956120601030013</v>
+      </c>
+      <c r="E89">
+        <v>0.07883488383802129</v>
+      </c>
+      <c r="F89">
+        <v>0.09812487415371307</v>
+      </c>
+      <c r="G89">
+        <v>0.1174204822031344</v>
+      </c>
+      <c r="H89">
+        <v>0.02766159905719601</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90">
+        <v>2015</v>
+      </c>
+      <c r="B90">
+        <v>0.009537520381164954</v>
+      </c>
+      <c r="C90">
+        <v>0.009822023548612613</v>
+      </c>
+      <c r="D90">
+        <v>0.009212735089158652</v>
+      </c>
+      <c r="E90">
+        <v>0.007719191077378618</v>
+      </c>
+      <c r="F90">
+        <v>0.005352238705074397</v>
+      </c>
+      <c r="G90">
+        <v>0.00212399634782523</v>
+      </c>
+      <c r="H90">
+        <v>-0.01529600966646494</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91">
+        <v>2016</v>
+      </c>
+      <c r="B91">
+        <v>0.004783803516075436</v>
+      </c>
+      <c r="C91">
+        <v>0.03130600850579057</v>
+      </c>
+      <c r="D91">
+        <v>0.05771316191412557</v>
+      </c>
+      <c r="E91">
+        <v>0.08396541286571502</v>
+      </c>
+      <c r="F91">
+        <v>0.1100216298614582</v>
+      </c>
+      <c r="G91">
+        <v>0.1358393997271168</v>
+      </c>
+      <c r="H91">
+        <v>0.08591330858293267</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92">
+        <v>2017</v>
+      </c>
+      <c r="B92">
+        <v>0.006321009399657962</v>
+      </c>
+      <c r="C92">
+        <v>0.04681209642524298</v>
+      </c>
+      <c r="D92">
+        <v>0.08870240621021486</v>
+      </c>
+      <c r="E92">
+        <v>0.1320327156122365</v>
+      </c>
+      <c r="F92">
+        <v>0.1768447794740906</v>
+      </c>
+      <c r="G92">
+        <v>0.2231813492439731</v>
+      </c>
+      <c r="H92">
+        <v>0.2587995974302768</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8">
+      <c r="A93">
+        <v>2018</v>
+      </c>
+      <c r="B93">
+        <v>0.01264784785415607</v>
+      </c>
+      <c r="C93">
+        <v>0.00201542367300811</v>
+      </c>
+      <c r="D93">
+        <v>-0.009612222836275275</v>
+      </c>
+      <c r="E93">
+        <v>-0.02222178047126144</v>
+      </c>
+      <c r="F93">
+        <v>-0.03579803134417558</v>
+      </c>
+      <c r="G93">
+        <v>-0.05032383811285335</v>
+      </c>
+      <c r="H93">
+        <v>-0.1002542548777808</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94">
+        <v>2019</v>
+      </c>
+      <c r="B94">
+        <v>0.05910933384103845</v>
+      </c>
+      <c r="C94">
+        <v>0.1067058542800259</v>
+      </c>
+      <c r="D94">
+        <v>0.1552204486966333</v>
+      </c>
+      <c r="E94">
+        <v>0.2045928133264405</v>
+      </c>
+      <c r="F94">
+        <v>0.2547563433952991</v>
+      </c>
+      <c r="G94">
+        <v>0.305637914454973</v>
+      </c>
+      <c r="H94">
+        <v>0.2524451410094963</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95">
+        <v>2020</v>
+      </c>
+      <c r="B95">
+        <v>0.07127287260409809</v>
+      </c>
+      <c r="C95">
+        <v>0.1106603429282058</v>
+      </c>
+      <c r="D95">
+        <v>0.1476376491512099</v>
+      </c>
+      <c r="E95">
+        <v>0.1818597925868803</v>
+      </c>
+      <c r="F95">
+        <v>0.2129819421429819</v>
+      </c>
+      <c r="G95">
+        <v>0.240661929523305</v>
+      </c>
+      <c r="H95">
+        <v>0.1786432468428296</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96">
+        <v>2021</v>
+      </c>
+      <c r="B96">
+        <v>-0.03467104499973528</v>
+      </c>
+      <c r="C96">
+        <v>0.01594983260153326</v>
+      </c>
+      <c r="D96">
+        <v>0.06854446134418413</v>
+      </c>
+      <c r="E96">
+        <v>0.1231587848089555</v>
+      </c>
+      <c r="F96">
+        <v>0.1798385538171232</v>
+      </c>
+      <c r="G96">
+        <v>0.238629263612596</v>
+      </c>
+      <c r="H96">
+        <v>0.1677975747130003</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97">
+        <v>2022</v>
+      </c>
+      <c r="B97">
+        <v>-0.09312159939086873</v>
+      </c>
+      <c r="C97">
+        <v>-0.1125568962929426</v>
+      </c>
+      <c r="D97">
+        <v>-0.1329639214410837</v>
+      </c>
+      <c r="E97">
+        <v>-0.1542582607707412</v>
+      </c>
+      <c r="F97">
+        <v>-0.176354769174605</v>
+      </c>
+      <c r="G97">
+        <v>-0.1991679402165283</v>
+      </c>
+      <c r="H97">
+        <v>-0.1785360445541773</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98">
+        <v>2023</v>
+      </c>
+      <c r="B98">
+        <v>0.0477372003232106</v>
+      </c>
+      <c r="C98">
+        <v>0.08981610186135947</v>
+      </c>
+      <c r="D98">
+        <v>0.1327832053294453</v>
+      </c>
+      <c r="E98">
+        <v>0.1766289161713988</v>
+      </c>
+      <c r="F98">
+        <v>0.2213425505725926</v>
+      </c>
+      <c r="G98">
+        <v>0.2669123246958292</v>
+      </c>
+      <c r="H98">
+        <v>0.2112398302694116</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
+      <c r="A99">
+        <v>2024</v>
+      </c>
+      <c r="B99">
+        <v>0.01690210925782254</v>
+      </c>
+      <c r="C99">
+        <v>0.06076609467165484</v>
+      </c>
+      <c r="D99">
+        <v>0.1060003171092398</v>
+      </c>
+      <c r="E99">
+        <v>0.1526299670563722</v>
+      </c>
+      <c r="F99">
+        <v>0.2006801972016281</v>
+      </c>
+      <c r="G99">
+        <v>0.250176105461307</v>
+      </c>
+      <c r="H99">
+        <v>0.1545105919177152</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
+      <c r="A100">
+        <v>2025</v>
+      </c>
+      <c r="B100">
+        <v>0.06977434210917988</v>
+      </c>
+      <c r="C100">
+        <v>0.0915401309371815</v>
+      </c>
+      <c r="D100">
+        <v>0.1130182089358862</v>
+      </c>
+      <c r="E100">
+        <v>0.1341769567452189</v>
+      </c>
+      <c r="F100">
+        <v>0.1549843140267351</v>
+      </c>
+      <c r="G100">
+        <v>0.1754078096429585</v>
+      </c>
+      <c r="H100">
+        <v>0.2313488662180263</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="13.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" style="1" customWidth="1"/>
+    <col min="8" max="11" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H1" t="s">
+        <v>133</v>
+      </c>
+      <c r="I1" t="s">
+        <v>134</v>
+      </c>
+      <c r="J1" t="s">
+        <v>135</v>
+      </c>
+      <c r="K1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2">
+        <v>408</v>
+      </c>
+      <c r="D2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0.9956484528139071</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.009378186665058876</v>
+      </c>
+      <c r="H2">
+        <v>0.08343854699931041</v>
+      </c>
+      <c r="I2">
+        <v>0.08379761056351676</v>
+      </c>
+      <c r="J2">
+        <v>0.09050128895817289</v>
+      </c>
+      <c r="K2">
+        <v>0.09420904493697409</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3">
+        <v>219</v>
+      </c>
+      <c r="D3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" t="s">
+        <v>91</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.993430650596881</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0.01909815941748197</v>
+      </c>
+      <c r="H3">
+        <v>0.08728703203381971</v>
+      </c>
+      <c r="I3">
+        <v>0.08818700738392726</v>
+      </c>
+      <c r="J3">
+        <v>0.1626312957614541</v>
+      </c>
+      <c r="K3">
+        <v>0.165849695726203</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B23"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1260,23 +3584,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B3">
         <v>196</v>
@@ -1284,162 +3608,162 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B4">
-        <v>0.7555474316099458</v>
+        <v>0.7555477977676611</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B5">
-        <v>0.08525353661429502</v>
+        <v>0.08525348168327691</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6">
-        <v>-0.02097658754190014</v>
+        <v>-0.02097657704159607</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="B7" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="B9" t="s">
-        <v>141</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="B16" t="s">
-        <v>148</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B18" t="s">
-        <v>150</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="B22" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="B23" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -1624,7 +3948,7 @@
         <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1641,7 +3965,7 @@
         <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1658,7 +3982,7 @@
         <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1675,7 +3999,7 @@
         <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1699,31 +4023,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1731,13 +4055,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>1203</v>
@@ -1760,13 +4084,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>1203</v>
@@ -1789,13 +4113,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>1203</v>
@@ -1818,13 +4142,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>1203</v>
@@ -1847,13 +4171,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>1203</v>
@@ -1876,13 +4200,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>759</v>
@@ -1905,13 +4229,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D8">
         <v>759</v>
@@ -1934,13 +4258,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D9">
         <v>435</v>
@@ -1963,13 +4287,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D10">
         <v>435</v>
@@ -1992,13 +4316,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>435</v>
@@ -2021,13 +4345,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>447</v>
@@ -2050,13 +4374,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>447</v>
@@ -2079,13 +4403,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D14">
         <v>447</v>
@@ -2108,13 +4432,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>1203</v>
@@ -2134,13 +4458,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D16">
         <v>776</v>
@@ -2163,13 +4487,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>776</v>
@@ -2192,13 +4516,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D18">
         <v>776</v>
@@ -2221,13 +4545,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D19">
         <v>1203</v>
@@ -2250,13 +4574,13 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D20">
         <v>501</v>
@@ -2279,13 +4603,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D21">
         <v>1197</v>
@@ -2327,31 +4651,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -2359,13 +4683,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>441</v>
@@ -2388,13 +4712,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>441</v>
@@ -2417,13 +4741,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>441</v>
@@ -2446,13 +4770,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>441</v>
@@ -2475,13 +4799,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>441</v>
@@ -2504,13 +4828,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>441</v>
@@ -2533,13 +4857,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D8">
         <v>441</v>
@@ -2562,37 +4886,37 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J10" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J11" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>441</v>
@@ -2615,13 +4939,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>441</v>
@@ -2644,13 +4968,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D14">
         <v>441</v>
@@ -2673,13 +4997,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>441</v>
@@ -2699,13 +5023,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D16">
         <v>441</v>
@@ -2728,13 +5052,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>441</v>
@@ -2757,13 +5081,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D18">
         <v>441</v>
@@ -2786,13 +5110,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D19">
         <v>441</v>
@@ -2815,13 +5139,13 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D20">
         <v>441</v>
@@ -2844,13 +5168,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D21">
         <v>441</v>
@@ -2892,31 +5216,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -2924,13 +5248,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D2">
         <v>321</v>
@@ -2953,13 +5277,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D3">
         <v>321</v>
@@ -2982,13 +5306,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D4">
         <v>321</v>
@@ -3011,13 +5335,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D5">
         <v>321</v>
@@ -3040,13 +5364,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D6">
         <v>321</v>
@@ -3069,13 +5393,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D7">
         <v>321</v>
@@ -3098,13 +5422,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D8">
         <v>321</v>
@@ -3127,13 +5451,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D9">
         <v>321</v>
@@ -3156,13 +5480,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C10" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D10">
         <v>321</v>
@@ -3185,13 +5509,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D11">
         <v>321</v>
@@ -3214,13 +5538,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D12">
         <v>321</v>
@@ -3243,13 +5567,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>321</v>
@@ -3272,13 +5596,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D14">
         <v>321</v>
@@ -3301,13 +5625,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D15">
         <v>321</v>
@@ -3327,13 +5651,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D16">
         <v>321</v>
@@ -3356,13 +5680,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>321</v>
@@ -3385,13 +5709,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D18">
         <v>321</v>
@@ -3414,13 +5738,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D19">
         <v>321</v>
@@ -3443,13 +5767,13 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D20">
         <v>321</v>
@@ -3472,13 +5796,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D21">
         <v>321</v>
@@ -3520,31 +5844,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -3552,13 +5876,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D2">
         <v>120</v>
@@ -3581,13 +5905,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D3">
         <v>120</v>
@@ -3610,13 +5934,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D4">
         <v>120</v>
@@ -3639,13 +5963,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5">
         <v>120</v>
@@ -3668,13 +5992,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6">
         <v>120</v>
@@ -3697,13 +6021,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D7">
         <v>120</v>
@@ -3726,13 +6050,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D8">
         <v>120</v>
@@ -3755,13 +6079,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D9">
         <v>120</v>
@@ -3784,13 +6108,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D10">
         <v>120</v>
@@ -3813,13 +6137,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D11">
         <v>120</v>
@@ -3842,13 +6166,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D12">
         <v>120</v>
@@ -3871,13 +6195,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D13">
         <v>120</v>
@@ -3900,13 +6224,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C14" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D14">
         <v>120</v>
@@ -3929,13 +6253,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C15" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D15">
         <v>120</v>
@@ -3955,13 +6279,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D16">
         <v>120</v>
@@ -3984,13 +6308,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D17">
         <v>120</v>
@@ -4013,13 +6337,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D18">
         <v>120</v>
@@ -4042,13 +6366,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C19" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D19">
         <v>120</v>
@@ -4071,13 +6395,13 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B20" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C20" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D20">
         <v>120</v>
@@ -4100,13 +6424,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D21">
         <v>120</v>
@@ -4154,72 +6478,72 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -4284,7 +6608,7 @@
     </row>
     <row r="3" spans="1:21">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B3" s="2">
         <v>0.8084723245525287</v>
@@ -4349,7 +6673,7 @@
     </row>
     <row r="4" spans="1:21">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" s="2">
         <v>0.8453565887860622</v>
@@ -4414,7 +6738,7 @@
     </row>
     <row r="5" spans="1:21">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B5" s="2">
         <v>0.8427478229847296</v>
@@ -4479,7 +6803,7 @@
     </row>
     <row r="6" spans="1:21">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B6" s="2">
         <v>0.9722190415305743</v>
@@ -4544,7 +6868,7 @@
     </row>
     <row r="7" spans="1:21">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" s="2">
         <v>0.853257488679916</v>
@@ -4609,7 +6933,7 @@
     </row>
     <row r="8" spans="1:21">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B8" s="2">
         <v>0.8369340000236228</v>
@@ -4674,7 +6998,7 @@
     </row>
     <row r="9" spans="1:21">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2">
         <v>0.6226168068197092</v>
@@ -4739,7 +7063,7 @@
     </row>
     <row r="10" spans="1:21">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B10" s="2">
         <v>0.7124647204721374</v>
@@ -4804,7 +7128,7 @@
     </row>
     <row r="11" spans="1:21">
       <c r="A11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B11" s="2">
         <v>0.7658313815373569</v>
@@ -4869,7 +7193,7 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B12" s="2">
         <v>0.6018775544729295</v>
@@ -4934,7 +7258,7 @@
     </row>
     <row r="13" spans="1:21">
       <c r="A13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B13" s="2">
         <v>0.6774842229672553</v>
@@ -4999,7 +7323,7 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B14" s="2">
         <v>0.7107951348280582</v>
@@ -5064,7 +7388,7 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B15" s="2">
         <v>0.008720575418330557</v>
@@ -5129,7 +7453,7 @@
     </row>
     <row r="16" spans="1:21">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B16" s="2">
         <v>-0.04506667671579052</v>
@@ -5194,7 +7518,7 @@
     </row>
     <row r="17" spans="1:21">
       <c r="A17" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B17" s="2">
         <v>-0.09296776454437576</v>
@@ -5259,7 +7583,7 @@
     </row>
     <row r="18" spans="1:21">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B18" s="2">
         <v>-0.06844342659119444</v>
@@ -5324,7 +7648,7 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" s="2">
         <v>0.3345626558024875</v>
@@ -5389,7 +7713,7 @@
     </row>
     <row r="20" spans="1:21">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B20" s="2">
         <v>-0.1684954070223643</v>
@@ -5454,7 +7778,7 @@
     </row>
     <row r="21" spans="1:21">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B21" s="2">
         <v>-0.3189467570670729</v>
@@ -5544,67 +7868,67 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -10197,13 +12521,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>

<commit_message>
Use AQMIX for Trend from January 2026
Trend now takes AQMIX's actual monthly returns (after fees) from
2026-01 instead of only after AQR's factor data ends (2026-05), so the
current year matches the real fund: Jan-Sep 2026 = 18.91%, the same as
AQMIX. 1985-2025 stays on the AQR factor. The switch month is the
TREND_FUND_FROM setting; if AQR's data ends earlier, AQMIX fills from
there. Data rebuilt from the downloaded files (no new vintage).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtyJ36mjEj9LzVccKuq7PT
</commit_message>
<xml_diff>
--- a/data/processed/stats.xlsx
+++ b/data/processed/stats.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="174">
   <si>
     <t>note</t>
   </si>
@@ -184,16 +184,7 @@
     <t>202605</t>
   </si>
   <si>
-    <t>2026-10-30T02:30:35</t>
-  </si>
-  <si>
-    <t>2026-10-30T02:30:36</t>
-  </si>
-  <si>
-    <t>2026-10-30T02:30:37</t>
-  </si>
-  <si>
-    <t>2026-10-30T02:30:38</t>
+    <t>2026-10-30T03:19:49</t>
   </si>
   <si>
     <t>start</t>
@@ -996,21 +987,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B2">
         <v>99</v>
@@ -1024,7 +1015,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B3">
         <v>99</v>
@@ -1038,7 +1029,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B4">
         <v>99</v>
@@ -1052,7 +1043,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B5">
         <v>99</v>
@@ -1066,7 +1057,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B6">
         <v>62</v>
@@ -1080,7 +1071,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B7">
         <v>62</v>
@@ -1094,7 +1085,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B8">
         <v>35</v>
@@ -1108,7 +1099,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B9">
         <v>35</v>
@@ -1122,7 +1113,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B10">
         <v>36</v>
@@ -1136,7 +1127,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -1167,19 +1158,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1232,23 +1223,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B3">
         <v>39</v>
@@ -1256,7 +1247,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B4">
         <v>0.8593974426563644</v>
@@ -1264,7 +1255,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B5">
         <v>0.06226033065836247</v>
@@ -1272,7 +1263,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B6">
         <v>0.03427818511853675</v>
@@ -1280,34 +1271,34 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1331,31 +1322,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1363,13 +1354,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" t="s">
         <v>88</v>
-      </c>
-      <c r="C2" t="s">
-        <v>91</v>
       </c>
       <c r="D2">
         <v>776</v>
@@ -1392,13 +1383,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
         <v>88</v>
-      </c>
-      <c r="C3" t="s">
-        <v>91</v>
       </c>
       <c r="D3">
         <v>776</v>
@@ -1421,13 +1412,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" t="s">
         <v>88</v>
-      </c>
-      <c r="C4" t="s">
-        <v>91</v>
       </c>
       <c r="D4">
         <v>776</v>
@@ -1450,13 +1441,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" t="s">
         <v>88</v>
-      </c>
-      <c r="C5" t="s">
-        <v>91</v>
       </c>
       <c r="D5">
         <v>776</v>
@@ -1479,13 +1470,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" t="s">
         <v>88</v>
-      </c>
-      <c r="C6" t="s">
-        <v>91</v>
       </c>
       <c r="D6">
         <v>776</v>
@@ -1508,13 +1499,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D7">
         <v>1203</v>
@@ -1537,13 +1528,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D8">
         <v>435</v>
@@ -1580,28 +1571,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" t="s">
         <v>123</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>126</v>
-      </c>
-      <c r="F1" t="s">
-        <v>127</v>
-      </c>
-      <c r="G1" t="s">
-        <v>128</v>
-      </c>
-      <c r="H1" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3465,54 +3456,54 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H1" t="s">
         <v>130</v>
       </c>
-      <c r="C1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="I1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" t="s">
+      <c r="J1" t="s">
         <v>132</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>133</v>
-      </c>
-      <c r="I1" t="s">
-        <v>134</v>
-      </c>
-      <c r="J1" t="s">
-        <v>135</v>
-      </c>
-      <c r="K1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C2">
         <v>408</v>
       </c>
       <c r="D2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F2" s="2">
         <v>0.9956484528139071</v>
@@ -3535,19 +3526,19 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C3">
         <v>219</v>
       </c>
       <c r="D3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F3" s="2">
         <v>0.993430650596881</v>
@@ -3584,23 +3575,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B3">
         <v>196</v>
@@ -3608,7 +3599,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B4">
         <v>0.7555477977676611</v>
@@ -3616,7 +3607,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B5">
         <v>0.08525348168327691</v>
@@ -3624,7 +3615,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B6">
         <v>-0.02097657704159607</v>
@@ -3632,138 +3623,138 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B8" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B9" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B13" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B15" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B16" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B19" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B20" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B21" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B22" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B23" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -3931,7 +3922,7 @@
         <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -3948,7 +3939,7 @@
         <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -3965,7 +3956,7 @@
         <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3982,7 +3973,7 @@
         <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -3999,7 +3990,7 @@
         <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -4023,31 +4014,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -4055,13 +4046,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D2">
         <v>1203</v>
@@ -4084,13 +4075,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D3">
         <v>1203</v>
@@ -4113,13 +4104,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D4">
         <v>1203</v>
@@ -4142,13 +4133,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D5">
         <v>1203</v>
@@ -4171,13 +4162,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D6">
         <v>1203</v>
@@ -4200,13 +4191,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D7">
         <v>759</v>
@@ -4229,13 +4220,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D8">
         <v>759</v>
@@ -4258,13 +4249,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D9">
         <v>435</v>
@@ -4287,13 +4278,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D10">
         <v>435</v>
@@ -4316,13 +4307,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D11">
         <v>435</v>
@@ -4345,13 +4336,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D12">
         <v>447</v>
@@ -4374,13 +4365,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D13">
         <v>447</v>
@@ -4403,13 +4394,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D14">
         <v>447</v>
@@ -4432,13 +4423,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D15">
         <v>1203</v>
@@ -4458,13 +4449,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" t="s">
         <v>88</v>
-      </c>
-      <c r="C16" t="s">
-        <v>91</v>
       </c>
       <c r="D16">
         <v>776</v>
@@ -4487,13 +4478,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" t="s">
         <v>88</v>
-      </c>
-      <c r="C17" t="s">
-        <v>91</v>
       </c>
       <c r="D17">
         <v>776</v>
@@ -4516,13 +4507,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" t="s">
         <v>88</v>
-      </c>
-      <c r="C18" t="s">
-        <v>91</v>
       </c>
       <c r="D18">
         <v>776</v>
@@ -4545,13 +4536,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" t="s">
         <v>81</v>
       </c>
-      <c r="B19" t="s">
-        <v>84</v>
-      </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D19">
         <v>1203</v>
@@ -4574,25 +4565,25 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D20">
         <v>501</v>
       </c>
       <c r="E20" s="1">
-        <v>0.157097573770842</v>
+        <v>0.1556294157205564</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1253688111581719</v>
+        <v>0.1252023158505678</v>
       </c>
       <c r="G20" s="2">
-        <v>0.9864060355664387</v>
+        <v>0.9772161400699121</v>
       </c>
       <c r="H20" s="1">
         <v>-0.24751379044844</v>
@@ -4603,13 +4594,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D21">
         <v>1197</v>
@@ -4651,31 +4642,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -4683,13 +4674,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D2">
         <v>441</v>
@@ -4712,13 +4703,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D3">
         <v>441</v>
@@ -4741,13 +4732,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D4">
         <v>441</v>
@@ -4770,13 +4761,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D5">
         <v>441</v>
@@ -4799,13 +4790,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D6">
         <v>441</v>
@@ -4828,13 +4819,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D7">
         <v>441</v>
@@ -4857,13 +4848,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D8">
         <v>441</v>
@@ -4886,37 +4877,37 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="J9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J11" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D12">
         <v>441</v>
@@ -4939,13 +4930,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D13">
         <v>441</v>
@@ -4968,13 +4959,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D14">
         <v>441</v>
@@ -4997,13 +4988,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D15">
         <v>441</v>
@@ -5023,13 +5014,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D16">
         <v>441</v>
@@ -5052,13 +5043,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D17">
         <v>441</v>
@@ -5081,13 +5072,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D18">
         <v>441</v>
@@ -5110,13 +5101,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D19">
         <v>441</v>
@@ -5139,25 +5130,25 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D20">
         <v>441</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1397957942992942</v>
+        <v>0.1381529685055534</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1253045861553731</v>
+        <v>0.1251000736905589</v>
       </c>
       <c r="G20" s="2">
-        <v>0.9002521875071546</v>
+        <v>0.8897698278315144</v>
       </c>
       <c r="H20" s="1">
         <v>-0.2475137904484402</v>
@@ -5168,13 +5159,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D21">
         <v>441</v>
@@ -5216,31 +5207,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -5248,13 +5239,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D2">
         <v>321</v>
@@ -5277,13 +5268,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C3" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D3">
         <v>321</v>
@@ -5306,13 +5297,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D4">
         <v>321</v>
@@ -5335,13 +5326,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D5">
         <v>321</v>
@@ -5364,13 +5355,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D6">
         <v>321</v>
@@ -5393,13 +5384,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D7">
         <v>321</v>
@@ -5422,13 +5413,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D8">
         <v>321</v>
@@ -5451,13 +5442,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D9">
         <v>321</v>
@@ -5480,13 +5471,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D10">
         <v>321</v>
@@ -5509,13 +5500,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D11">
         <v>321</v>
@@ -5538,13 +5529,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D12">
         <v>321</v>
@@ -5567,13 +5558,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D13">
         <v>321</v>
@@ -5596,13 +5587,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D14">
         <v>321</v>
@@ -5625,13 +5616,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D15">
         <v>321</v>
@@ -5651,13 +5642,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D16">
         <v>321</v>
@@ -5680,13 +5671,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D17">
         <v>321</v>
@@ -5709,13 +5700,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C18" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D18">
         <v>321</v>
@@ -5738,13 +5729,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D19">
         <v>321</v>
@@ -5767,25 +5758,25 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D20">
         <v>321</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1041313313420678</v>
+        <v>0.1019455752360796</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1297851530001127</v>
+        <v>0.1294717532982563</v>
       </c>
       <c r="G20" s="2">
-        <v>0.6844767542346577</v>
+        <v>0.6702673451143426</v>
       </c>
       <c r="H20" s="1">
         <v>-0.2475137904484401</v>
@@ -5796,13 +5787,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C21" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D21">
         <v>321</v>
@@ -5844,31 +5835,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -5876,13 +5867,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D2">
         <v>120</v>
@@ -5905,13 +5896,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D3">
         <v>120</v>
@@ -5934,13 +5925,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D4">
         <v>120</v>
@@ -5963,13 +5954,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D5">
         <v>120</v>
@@ -5992,13 +5983,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D6">
         <v>120</v>
@@ -6021,13 +6012,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D7">
         <v>120</v>
@@ -6050,13 +6041,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D8">
         <v>120</v>
@@ -6079,13 +6070,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D9">
         <v>120</v>
@@ -6108,13 +6099,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D10">
         <v>120</v>
@@ -6137,13 +6128,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D11">
         <v>120</v>
@@ -6166,13 +6157,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C12" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D12">
         <v>120</v>
@@ -6195,13 +6186,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D13">
         <v>120</v>
@@ -6224,13 +6215,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D14">
         <v>120</v>
@@ -6253,13 +6244,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D15">
         <v>120</v>
@@ -6279,13 +6270,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C16" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D16">
         <v>120</v>
@@ -6308,13 +6299,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C17" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D17">
         <v>120</v>
@@ -6337,13 +6328,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D18">
         <v>120</v>
@@ -6366,13 +6357,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D19">
         <v>120</v>
@@ -6395,13 +6386,13 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D20">
         <v>120</v>
@@ -6424,13 +6415,13 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D21">
         <v>120</v>
@@ -6478,72 +6469,72 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -6600,7 +6591,7 @@
         <v>0.3345626558024875</v>
       </c>
       <c r="T2" s="2">
-        <v>-0.1684954070223643</v>
+        <v>-0.174051117222249</v>
       </c>
       <c r="U2" s="2">
         <v>-0.3189467570670729</v>
@@ -6608,7 +6599,7 @@
     </row>
     <row r="3" spans="1:21">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" s="2">
         <v>0.8084723245525287</v>
@@ -6665,7 +6656,7 @@
         <v>0.341024462184917</v>
       </c>
       <c r="T3" s="2">
-        <v>-0.2008957269764446</v>
+        <v>-0.2043652910733721</v>
       </c>
       <c r="U3" s="2">
         <v>-0.1220064155989652</v>
@@ -6673,7 +6664,7 @@
     </row>
     <row r="4" spans="1:21">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" s="2">
         <v>0.8453565887860622</v>
@@ -6730,7 +6721,7 @@
         <v>0.2620500041526474</v>
       </c>
       <c r="T4" s="2">
-        <v>-0.165540027193309</v>
+        <v>-0.1704806329162473</v>
       </c>
       <c r="U4" s="2">
         <v>-0.3609812152018139</v>
@@ -6738,7 +6729,7 @@
     </row>
     <row r="5" spans="1:21">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" s="2">
         <v>0.8427478229847296</v>
@@ -6795,7 +6786,7 @@
         <v>0.3572246201059924</v>
       </c>
       <c r="T5" s="2">
-        <v>-0.2124948053634381</v>
+        <v>-0.218902768171632</v>
       </c>
       <c r="U5" s="2">
         <v>-0.09041687676338699</v>
@@ -6803,7 +6794,7 @@
     </row>
     <row r="6" spans="1:21">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B6" s="2">
         <v>0.9722190415305743</v>
@@ -6860,7 +6851,7 @@
         <v>0.2760077792474183</v>
       </c>
       <c r="T6" s="2">
-        <v>-0.1441775053990973</v>
+        <v>-0.1501815314812725</v>
       </c>
       <c r="U6" s="2">
         <v>-0.3754013538160224</v>
@@ -6868,7 +6859,7 @@
     </row>
     <row r="7" spans="1:21">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B7" s="2">
         <v>0.853257488679916</v>
@@ -6925,7 +6916,7 @@
         <v>0.3393877351057602</v>
       </c>
       <c r="T7" s="2">
-        <v>-0.211484808454069</v>
+        <v>-0.2150169267444245</v>
       </c>
       <c r="U7" s="2">
         <v>-0.2397542147734855</v>
@@ -6933,7 +6924,7 @@
     </row>
     <row r="8" spans="1:21">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B8" s="2">
         <v>0.8369340000236228</v>
@@ -6990,7 +6981,7 @@
         <v>0.2867071752857003</v>
       </c>
       <c r="T8" s="2">
-        <v>-0.1642219365556789</v>
+        <v>-0.1688066755923048</v>
       </c>
       <c r="U8" s="2">
         <v>-0.2984254417000554</v>
@@ -6998,7 +6989,7 @@
     </row>
     <row r="9" spans="1:21">
       <c r="A9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B9" s="2">
         <v>0.6226168068197092</v>
@@ -7055,7 +7046,7 @@
         <v>0.4994654824723255</v>
       </c>
       <c r="T9" s="2">
-        <v>-0.1715162899394772</v>
+        <v>-0.1743342388622958</v>
       </c>
       <c r="U9" s="2">
         <v>-0.1871526740657589</v>
@@ -7063,7 +7054,7 @@
     </row>
     <row r="10" spans="1:21">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B10" s="2">
         <v>0.7124647204721374</v>
@@ -7120,7 +7111,7 @@
         <v>0.4583092063084198</v>
       </c>
       <c r="T10" s="2">
-        <v>-0.1856748158515933</v>
+        <v>-0.1883349938814105</v>
       </c>
       <c r="U10" s="2">
         <v>-0.1943101739563054</v>
@@ -7128,7 +7119,7 @@
     </row>
     <row r="11" spans="1:21">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B11" s="2">
         <v>0.7658313815373569</v>
@@ -7185,7 +7176,7 @@
         <v>0.4347102962326969</v>
       </c>
       <c r="T11" s="2">
-        <v>-0.1608806417179749</v>
+        <v>-0.1638422366177304</v>
       </c>
       <c r="U11" s="2">
         <v>-0.2468058826896434</v>
@@ -7193,7 +7184,7 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B12" s="2">
         <v>0.6018775544729295</v>
@@ -7250,7 +7241,7 @@
         <v>0.4509364578920367</v>
       </c>
       <c r="T12" s="2">
-        <v>-0.1263581861766898</v>
+        <v>-0.128997772606995</v>
       </c>
       <c r="U12" s="2">
         <v>-0.2462754075621131</v>
@@ -7258,7 +7249,7 @@
     </row>
     <row r="13" spans="1:21">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B13" s="2">
         <v>0.6774842229672553</v>
@@ -7315,7 +7306,7 @@
         <v>0.4699504830762667</v>
       </c>
       <c r="T13" s="2">
-        <v>-0.1272492165258428</v>
+        <v>-0.1301171097783223</v>
       </c>
       <c r="U13" s="2">
         <v>-0.2573729833527058</v>
@@ -7323,7 +7314,7 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" s="2">
         <v>0.7107951348280582</v>
@@ -7380,7 +7371,7 @@
         <v>0.4367398812841394</v>
       </c>
       <c r="T14" s="2">
-        <v>-0.1346471757517568</v>
+        <v>-0.1399960256845093</v>
       </c>
       <c r="U14" s="2">
         <v>-0.289452800892835</v>
@@ -7388,7 +7379,7 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B15" s="2">
         <v>0.008720575418330557</v>
@@ -7445,7 +7436,7 @@
         <v>0.02748929588193674</v>
       </c>
       <c r="T15" s="2">
-        <v>0.1210233072578733</v>
+        <v>0.1198458693796355</v>
       </c>
       <c r="U15" s="2">
         <v>0.1676753538624426</v>
@@ -7453,7 +7444,7 @@
     </row>
     <row r="16" spans="1:21">
       <c r="A16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B16" s="2">
         <v>-0.04506667671579052</v>
@@ -7510,7 +7501,7 @@
         <v>-0.07907903964650614</v>
       </c>
       <c r="T16" s="2">
-        <v>0.1436952554002458</v>
+        <v>0.1440231798102623</v>
       </c>
       <c r="U16" s="2">
         <v>0.1159300913489198</v>
@@ -7518,7 +7509,7 @@
     </row>
     <row r="17" spans="1:21">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B17" s="2">
         <v>-0.09296776454437576</v>
@@ -7575,7 +7566,7 @@
         <v>-0.1366429986766272</v>
       </c>
       <c r="T17" s="2">
-        <v>0.2049573165761073</v>
+        <v>0.2071043058025451</v>
       </c>
       <c r="U17" s="2">
         <v>0.1097506514905035</v>
@@ -7583,7 +7574,7 @@
     </row>
     <row r="18" spans="1:21">
       <c r="A18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B18" s="2">
         <v>-0.06844342659119444</v>
@@ -7640,7 +7631,7 @@
         <v>-0.1731324640194044</v>
       </c>
       <c r="T18" s="2">
-        <v>0.2271900752316423</v>
+        <v>0.229318943397713</v>
       </c>
       <c r="U18" s="2">
         <v>0.09815132479134112</v>
@@ -7648,7 +7639,7 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B19" s="2">
         <v>0.3345626558024875</v>
@@ -7705,7 +7696,7 @@
         <v>1</v>
       </c>
       <c r="T19" s="2">
-        <v>-0.03836690585684775</v>
+        <v>-0.04264386944636318</v>
       </c>
       <c r="U19" s="2">
         <v>-0.02834016125905013</v>
@@ -7713,72 +7704,72 @@
     </row>
     <row r="20" spans="1:21">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B20" s="2">
-        <v>-0.1684954070223643</v>
+        <v>-0.174051117222249</v>
       </c>
       <c r="C20" s="2">
-        <v>-0.2008957269764446</v>
+        <v>-0.2043652910733721</v>
       </c>
       <c r="D20" s="2">
-        <v>-0.165540027193309</v>
+        <v>-0.1704806329162473</v>
       </c>
       <c r="E20" s="2">
-        <v>-0.2124948053634381</v>
+        <v>-0.218902768171632</v>
       </c>
       <c r="F20" s="2">
-        <v>-0.1441775053990973</v>
+        <v>-0.1501815314812725</v>
       </c>
       <c r="G20" s="2">
-        <v>-0.211484808454069</v>
+        <v>-0.2150169267444245</v>
       </c>
       <c r="H20" s="2">
-        <v>-0.1642219365556789</v>
+        <v>-0.1688066755923048</v>
       </c>
       <c r="I20" s="2">
-        <v>-0.1715162899394772</v>
+        <v>-0.1743342388622958</v>
       </c>
       <c r="J20" s="2">
-        <v>-0.1856748158515933</v>
+        <v>-0.1883349938814105</v>
       </c>
       <c r="K20" s="2">
-        <v>-0.1608806417179749</v>
+        <v>-0.1638422366177304</v>
       </c>
       <c r="L20" s="2">
-        <v>-0.1263581861766898</v>
+        <v>-0.128997772606995</v>
       </c>
       <c r="M20" s="2">
-        <v>-0.1272492165258428</v>
+        <v>-0.1301171097783223</v>
       </c>
       <c r="N20" s="2">
-        <v>-0.1346471757517568</v>
+        <v>-0.1399960256845093</v>
       </c>
       <c r="O20" s="2">
-        <v>0.1210233072578733</v>
+        <v>0.1198458693796355</v>
       </c>
       <c r="P20" s="2">
-        <v>0.1436952554002458</v>
+        <v>0.1440231798102623</v>
       </c>
       <c r="Q20" s="2">
-        <v>0.2049573165761073</v>
+        <v>0.2071043058025451</v>
       </c>
       <c r="R20" s="2">
-        <v>0.2271900752316423</v>
+        <v>0.229318943397713</v>
       </c>
       <c r="S20" s="2">
-        <v>-0.03836690585684775</v>
+        <v>-0.04264386944636318</v>
       </c>
       <c r="T20" s="2">
         <v>1</v>
       </c>
       <c r="U20" s="2">
-        <v>0.3297098513205868</v>
+        <v>0.3258666629084061</v>
       </c>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B21" s="2">
         <v>-0.3189467570670729</v>
@@ -7835,7 +7826,7 @@
         <v>-0.02834016125905013</v>
       </c>
       <c r="T21" s="2">
-        <v>0.3297098513205868</v>
+        <v>0.3258666629084061</v>
       </c>
       <c r="U21" s="2">
         <v>1</v>
@@ -7868,67 +7859,67 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -12521,13 +12512,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>

<commit_message>
Subtract a 2%/yr fee from the Trend factor months
Trend's AQR factor months (1985-2025) now have 2%/12 subtracted each
month (TREND_FACTOR_FEE). AQMIX months from 2026 are unchanged since
they're already net of fees. Effect since 1985: CAGR 15.7% -> 13.3%,
Sharpe 0.98 -> 0.82. Against AQMIX (2010-2026 overlap) the average gap
falls from -2.1%/yr to -0.1%/yr. Data rebuilt from downloaded files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtyJ36mjEj9LzVccKuq7PT
</commit_message>
<xml_diff>
--- a/data/processed/stats.xlsx
+++ b/data/processed/stats.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="175">
   <si>
     <t>note</t>
   </si>
@@ -184,7 +184,10 @@
     <t>202605</t>
   </si>
   <si>
-    <t>2026-10-30T03:19:49</t>
+    <t>2026-10-30T03:24:46</t>
+  </si>
+  <si>
+    <t>2026-10-30T03:24:47</t>
   </si>
   <si>
     <t>start</t>
@@ -502,55 +505,55 @@
     <t>2010-02 to 2026-05</t>
   </si>
   <si>
-    <t>18.2% / 9.3%</t>
+    <t>16.1% / 9.3%</t>
   </si>
   <si>
-    <t>-0.1% / -6.4%</t>
+    <t>-2.0% / -6.4%</t>
   </si>
   <si>
-    <t>-0.1% / 3.0%</t>
+    <t>-2.1% / 3.0%</t>
   </si>
   <si>
-    <t>18.2% / 9.4%</t>
+    <t>15.9% / 9.4%</t>
   </si>
   <si>
-    <t>19.1% / 9.7%</t>
+    <t>16.8% / 9.7%</t>
   </si>
   <si>
-    <t>18.1% / 2.0%</t>
+    <t>15.8% / 2.0%</t>
   </si>
   <si>
-    <t>-10.9% / -8.4%</t>
+    <t>-12.7% / -8.4%</t>
   </si>
   <si>
-    <t>7.5% / -1.0%</t>
+    <t>5.3% / -1.0%</t>
   </si>
   <si>
-    <t>-7.4% / -8.9%</t>
+    <t>-9.2% / -8.9%</t>
   </si>
   <si>
-    <t>5.4% / 1.9%</t>
+    <t>3.3% / 1.9%</t>
   </si>
   <si>
-    <t>-6.3% / -0.4%</t>
+    <t>-8.2% / -0.4%</t>
   </si>
   <si>
-    <t>-4.6% / -1.0%</t>
+    <t>-6.5% / -1.0%</t>
   </si>
   <si>
-    <t>26.5% / 35.5%</t>
+    <t>24.0% / 35.5%</t>
   </si>
   <si>
-    <t>-3.6% / 2.1%</t>
+    <t>-5.5% / 2.1%</t>
   </si>
   <si>
-    <t>8.9% / 8.1%</t>
+    <t>6.8% / 8.1%</t>
   </si>
   <si>
-    <t>6.1% / 14.6%</t>
+    <t>4.0% / 14.6%</t>
   </si>
   <si>
-    <t>17.0% / 11.0%</t>
+    <t>16.1% / 11.0%</t>
   </si>
 </sst>
 </file>
@@ -987,21 +990,21 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B2">
         <v>99</v>
@@ -1015,7 +1018,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B3">
         <v>99</v>
@@ -1029,7 +1032,7 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4">
         <v>99</v>
@@ -1043,7 +1046,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B5">
         <v>99</v>
@@ -1057,7 +1060,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B6">
         <v>62</v>
@@ -1071,7 +1074,7 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B7">
         <v>62</v>
@@ -1085,7 +1088,7 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B8">
         <v>35</v>
@@ -1099,7 +1102,7 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B9">
         <v>35</v>
@@ -1113,7 +1116,7 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B10">
         <v>36</v>
@@ -1127,7 +1130,7 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B11">
         <v>36</v>
@@ -1158,19 +1161,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -1223,23 +1226,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
         <v>107</v>
-      </c>
-      <c r="B1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3">
         <v>39</v>
@@ -1247,7 +1250,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4">
         <v>0.8593974426563644</v>
@@ -1255,7 +1258,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B5">
         <v>0.06226033065836247</v>
@@ -1263,7 +1266,7 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B6">
         <v>0.03427818511853675</v>
@@ -1271,34 +1274,34 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1322,31 +1325,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -1354,13 +1357,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D2">
         <v>776</v>
@@ -1383,13 +1386,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D3">
         <v>776</v>
@@ -1412,13 +1415,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D4">
         <v>776</v>
@@ -1441,13 +1444,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5">
         <v>776</v>
@@ -1470,13 +1473,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6">
         <v>776</v>
@@ -1499,13 +1502,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D7">
         <v>1203</v>
@@ -1528,13 +1531,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D8">
         <v>435</v>
@@ -1571,28 +1574,28 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -3456,54 +3459,54 @@
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="H1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I1" t="s">
+        <v>132</v>
+      </c>
+      <c r="J1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K1" t="s">
         <v>134</v>
-      </c>
-      <c r="B1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" t="s">
-        <v>128</v>
-      </c>
-      <c r="E1" t="s">
-        <v>129</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="H1" t="s">
-        <v>130</v>
-      </c>
-      <c r="I1" t="s">
-        <v>131</v>
-      </c>
-      <c r="J1" t="s">
-        <v>132</v>
-      </c>
-      <c r="K1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C2">
         <v>408</v>
       </c>
       <c r="D2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F2" s="2">
         <v>0.9956484528139071</v>
@@ -3526,19 +3529,19 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C3">
         <v>219</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F3" s="2">
         <v>0.993430650596881</v>
@@ -3575,23 +3578,23 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" t="s">
         <v>107</v>
-      </c>
-      <c r="B1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B3">
         <v>196</v>
@@ -3599,7 +3602,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B4">
         <v>0.7555477977676611</v>
@@ -3607,154 +3610,154 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B5">
-        <v>0.08525348168327691</v>
+        <v>0.0852534816832769</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B6">
-        <v>-0.02097657704159607</v>
+        <v>-0.0009765770415960757</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B23" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -3939,7 +3942,7 @@
         <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -3956,7 +3959,7 @@
         <v>47</v>
       </c>
       <c r="E11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3973,7 +3976,7 @@
         <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -3990,7 +3993,7 @@
         <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -4014,31 +4017,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -4046,13 +4049,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D2">
         <v>1203</v>
@@ -4075,13 +4078,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D3">
         <v>1203</v>
@@ -4104,13 +4107,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D4">
         <v>1203</v>
@@ -4133,13 +4136,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5">
         <v>1203</v>
@@ -4162,13 +4165,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6">
         <v>1203</v>
@@ -4191,13 +4194,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D7">
         <v>759</v>
@@ -4220,13 +4223,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D8">
         <v>759</v>
@@ -4249,13 +4252,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D9">
         <v>435</v>
@@ -4278,13 +4281,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D10">
         <v>435</v>
@@ -4307,13 +4310,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D11">
         <v>435</v>
@@ -4336,13 +4339,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D12">
         <v>447</v>
@@ -4365,13 +4368,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D13">
         <v>447</v>
@@ -4394,13 +4397,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D14">
         <v>447</v>
@@ -4423,13 +4426,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D15">
         <v>1203</v>
@@ -4449,13 +4452,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D16">
         <v>776</v>
@@ -4478,13 +4481,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D17">
         <v>776</v>
@@ -4507,13 +4510,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D18">
         <v>776</v>
@@ -4536,13 +4539,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D19">
         <v>1203</v>
@@ -4565,42 +4568,42 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D20">
         <v>501</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1556294157205564</v>
+        <v>0.1333848451629769</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1252023158505678</v>
+        <v>0.1252244230925287</v>
       </c>
       <c r="G20" s="2">
-        <v>0.9772161400699121</v>
+        <v>0.819225592323488</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.24751379044844</v>
+        <v>-0.3227383379097589</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.2151279293765394</v>
+        <v>-0.2310023528471506</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D21">
         <v>1197</v>
@@ -4642,31 +4645,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -4674,13 +4677,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C2" t="s">
         <v>89</v>
-      </c>
-      <c r="C2" t="s">
-        <v>88</v>
       </c>
       <c r="D2">
         <v>441</v>
@@ -4703,13 +4706,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C3" t="s">
         <v>89</v>
-      </c>
-      <c r="C3" t="s">
-        <v>88</v>
       </c>
       <c r="D3">
         <v>441</v>
@@ -4732,13 +4735,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
         <v>89</v>
-      </c>
-      <c r="C4" t="s">
-        <v>88</v>
       </c>
       <c r="D4">
         <v>441</v>
@@ -4761,13 +4764,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" t="s">
         <v>89</v>
-      </c>
-      <c r="C5" t="s">
-        <v>88</v>
       </c>
       <c r="D5">
         <v>441</v>
@@ -4790,13 +4793,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" t="s">
         <v>89</v>
-      </c>
-      <c r="C6" t="s">
-        <v>88</v>
       </c>
       <c r="D6">
         <v>441</v>
@@ -4819,13 +4822,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" t="s">
         <v>89</v>
-      </c>
-      <c r="C7" t="s">
-        <v>88</v>
       </c>
       <c r="D7">
         <v>441</v>
@@ -4848,13 +4851,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C8" t="s">
         <v>89</v>
-      </c>
-      <c r="C8" t="s">
-        <v>88</v>
       </c>
       <c r="D8">
         <v>441</v>
@@ -4877,37 +4880,37 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J10" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" t="s">
         <v>89</v>
-      </c>
-      <c r="C12" t="s">
-        <v>88</v>
       </c>
       <c r="D12">
         <v>441</v>
@@ -4930,13 +4933,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" t="s">
         <v>89</v>
-      </c>
-      <c r="C13" t="s">
-        <v>88</v>
       </c>
       <c r="D13">
         <v>441</v>
@@ -4959,13 +4962,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" t="s">
         <v>89</v>
-      </c>
-      <c r="C14" t="s">
-        <v>88</v>
       </c>
       <c r="D14">
         <v>441</v>
@@ -4988,13 +4991,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" t="s">
         <v>89</v>
-      </c>
-      <c r="C15" t="s">
-        <v>88</v>
       </c>
       <c r="D15">
         <v>441</v>
@@ -5014,13 +5017,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" t="s">
         <v>89</v>
-      </c>
-      <c r="C16" t="s">
-        <v>88</v>
       </c>
       <c r="D16">
         <v>441</v>
@@ -5043,13 +5046,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" t="s">
         <v>89</v>
-      </c>
-      <c r="C17" t="s">
-        <v>88</v>
       </c>
       <c r="D17">
         <v>441</v>
@@ -5072,13 +5075,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" t="s">
         <v>89</v>
-      </c>
-      <c r="C18" t="s">
-        <v>88</v>
       </c>
       <c r="D18">
         <v>441</v>
@@ -5101,13 +5104,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" t="s">
         <v>89</v>
-      </c>
-      <c r="C19" t="s">
-        <v>88</v>
       </c>
       <c r="D19">
         <v>441</v>
@@ -5130,42 +5133,42 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
         <v>89</v>
-      </c>
-      <c r="C20" t="s">
-        <v>88</v>
       </c>
       <c r="D20">
         <v>441</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1381529685055534</v>
+        <v>0.1162703364215698</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1251000736905589</v>
+        <v>0.1251294141813558</v>
       </c>
       <c r="G20" s="2">
-        <v>0.8897698278315144</v>
+        <v>0.7323344250606967</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.2475137904484402</v>
+        <v>-0.3227383379097591</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.2151279293765394</v>
+        <v>-0.2310023528471506</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" t="s">
         <v>89</v>
-      </c>
-      <c r="C21" t="s">
-        <v>88</v>
       </c>
       <c r="D21">
         <v>441</v>
@@ -5207,31 +5210,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -5239,13 +5242,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D2">
         <v>321</v>
@@ -5268,13 +5271,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D3">
         <v>321</v>
@@ -5297,13 +5300,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D4">
         <v>321</v>
@@ -5326,13 +5329,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5">
         <v>321</v>
@@ -5355,13 +5358,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D6">
         <v>321</v>
@@ -5384,13 +5387,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D7">
         <v>321</v>
@@ -5413,13 +5416,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D8">
         <v>321</v>
@@ -5442,13 +5445,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D9">
         <v>321</v>
@@ -5471,13 +5474,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D10">
         <v>321</v>
@@ -5500,13 +5503,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D11">
         <v>321</v>
@@ -5529,13 +5532,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D12">
         <v>321</v>
@@ -5558,13 +5561,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D13">
         <v>321</v>
@@ -5587,13 +5590,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D14">
         <v>321</v>
@@ -5616,13 +5619,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D15">
         <v>321</v>
@@ -5642,13 +5645,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D16">
         <v>321</v>
@@ -5671,13 +5674,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D17">
         <v>321</v>
@@ -5700,13 +5703,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D18">
         <v>321</v>
@@ -5729,13 +5732,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D19">
         <v>321</v>
@@ -5758,42 +5761,42 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D20">
         <v>321</v>
       </c>
       <c r="E20" s="1">
-        <v>0.1019455752360796</v>
+        <v>0.08086217213248981</v>
       </c>
       <c r="F20" s="1">
-        <v>0.1294717532982563</v>
+        <v>0.1295223146925609</v>
       </c>
       <c r="G20" s="2">
-        <v>0.6702673451143426</v>
+        <v>0.5197821791038664</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.2475137904484401</v>
+        <v>-0.3227383379097597</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.2151279293765394</v>
+        <v>-0.2310023528471506</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D21">
         <v>321</v>
@@ -5835,31 +5838,31 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="J1" t="s">
         <v>0</v>
@@ -5867,13 +5870,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2">
         <v>120</v>
@@ -5896,13 +5899,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D3">
         <v>120</v>
@@ -5925,13 +5928,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D4">
         <v>120</v>
@@ -5954,13 +5957,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D5">
         <v>120</v>
@@ -5983,13 +5986,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D6">
         <v>120</v>
@@ -6012,13 +6015,13 @@
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D7">
         <v>120</v>
@@ -6041,13 +6044,13 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D8">
         <v>120</v>
@@ -6070,13 +6073,13 @@
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D9">
         <v>120</v>
@@ -6099,13 +6102,13 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D10">
         <v>120</v>
@@ -6128,13 +6131,13 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D11">
         <v>120</v>
@@ -6157,13 +6160,13 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D12">
         <v>120</v>
@@ -6186,13 +6189,13 @@
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D13">
         <v>120</v>
@@ -6215,13 +6218,13 @@
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D14">
         <v>120</v>
@@ -6244,13 +6247,13 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D15">
         <v>120</v>
@@ -6270,13 +6273,13 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D16">
         <v>120</v>
@@ -6299,13 +6302,13 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D17">
         <v>120</v>
@@ -6328,13 +6331,13 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D18">
         <v>120</v>
@@ -6357,13 +6360,13 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D19">
         <v>120</v>
@@ -6386,42 +6389,42 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C20" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D20">
         <v>120</v>
       </c>
       <c r="E20" s="1">
-        <v>0.01647964566294258</v>
+        <v>-0.003650964742586638</v>
       </c>
       <c r="F20" s="1">
         <v>0.1280616153759044</v>
       </c>
       <c r="G20" s="2">
-        <v>0.02792638743068743</v>
+        <v>-0.1283604120825013</v>
       </c>
       <c r="H20" s="1">
-        <v>-0.2475137904484402</v>
+        <v>-0.3227383379097597</v>
       </c>
       <c r="I20" s="1">
-        <v>-0.2151279293765394</v>
+        <v>-0.2310023528471506</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C21" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D21">
         <v>120</v>
@@ -6469,72 +6472,72 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U1" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:21">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -6591,7 +6594,7 @@
         <v>0.3345626558024875</v>
       </c>
       <c r="T2" s="2">
-        <v>-0.174051117222249</v>
+        <v>-0.1739314254767215</v>
       </c>
       <c r="U2" s="2">
         <v>-0.3189467570670729</v>
@@ -6599,7 +6602,7 @@
     </row>
     <row r="3" spans="1:21">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B3" s="2">
         <v>0.8084723245525287</v>
@@ -6656,7 +6659,7 @@
         <v>0.341024462184917</v>
       </c>
       <c r="T3" s="2">
-        <v>-0.2043652910733721</v>
+        <v>-0.2042294230916621</v>
       </c>
       <c r="U3" s="2">
         <v>-0.1220064155989652</v>
@@ -6664,7 +6667,7 @@
     </row>
     <row r="4" spans="1:21">
       <c r="A4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" s="2">
         <v>0.8453565887860622</v>
@@ -6721,7 +6724,7 @@
         <v>0.2620500041526474</v>
       </c>
       <c r="T4" s="2">
-        <v>-0.1704806329162473</v>
+        <v>-0.1703430425228417</v>
       </c>
       <c r="U4" s="2">
         <v>-0.3609812152018139</v>
@@ -6729,7 +6732,7 @@
     </row>
     <row r="5" spans="1:21">
       <c r="A5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B5" s="2">
         <v>0.8427478229847296</v>
@@ -6786,7 +6789,7 @@
         <v>0.3572246201059924</v>
       </c>
       <c r="T5" s="2">
-        <v>-0.218902768171632</v>
+        <v>-0.2186278527143195</v>
       </c>
       <c r="U5" s="2">
         <v>-0.09041687676338699</v>
@@ -6794,7 +6797,7 @@
     </row>
     <row r="6" spans="1:21">
       <c r="A6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B6" s="2">
         <v>0.9722190415305743</v>
@@ -6851,7 +6854,7 @@
         <v>0.2760077792474183</v>
       </c>
       <c r="T6" s="2">
-        <v>-0.1501815314812725</v>
+        <v>-0.1501580296443984</v>
       </c>
       <c r="U6" s="2">
         <v>-0.3754013538160224</v>
@@ -6859,7 +6862,7 @@
     </row>
     <row r="7" spans="1:21">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B7" s="2">
         <v>0.853257488679916</v>
@@ -6916,7 +6919,7 @@
         <v>0.3393877351057602</v>
       </c>
       <c r="T7" s="2">
-        <v>-0.2150169267444245</v>
+        <v>-0.2149361341923391</v>
       </c>
       <c r="U7" s="2">
         <v>-0.2397542147734855</v>
@@ -6924,7 +6927,7 @@
     </row>
     <row r="8" spans="1:21">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" s="2">
         <v>0.8369340000236228</v>
@@ -6981,7 +6984,7 @@
         <v>0.2867071752857003</v>
       </c>
       <c r="T8" s="2">
-        <v>-0.1688066755923048</v>
+        <v>-0.1685415940436771</v>
       </c>
       <c r="U8" s="2">
         <v>-0.2984254417000554</v>
@@ -6989,7 +6992,7 @@
     </row>
     <row r="9" spans="1:21">
       <c r="A9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="2">
         <v>0.6226168068197092</v>
@@ -7046,7 +7049,7 @@
         <v>0.4994654824723255</v>
       </c>
       <c r="T9" s="2">
-        <v>-0.1743342388622958</v>
+        <v>-0.174094512729544</v>
       </c>
       <c r="U9" s="2">
         <v>-0.1871526740657589</v>
@@ -7054,7 +7057,7 @@
     </row>
     <row r="10" spans="1:21">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10" s="2">
         <v>0.7124647204721374</v>
@@ -7111,7 +7114,7 @@
         <v>0.4583092063084198</v>
       </c>
       <c r="T10" s="2">
-        <v>-0.1883349938814105</v>
+        <v>-0.1880768705967719</v>
       </c>
       <c r="U10" s="2">
         <v>-0.1943101739563054</v>
@@ -7119,7 +7122,7 @@
     </row>
     <row r="11" spans="1:21">
       <c r="A11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B11" s="2">
         <v>0.7658313815373569</v>
@@ -7176,7 +7179,7 @@
         <v>0.4347102962326969</v>
       </c>
       <c r="T11" s="2">
-        <v>-0.1638422366177304</v>
+        <v>-0.1636985791053485</v>
       </c>
       <c r="U11" s="2">
         <v>-0.2468058826896434</v>
@@ -7184,7 +7187,7 @@
     </row>
     <row r="12" spans="1:21">
       <c r="A12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B12" s="2">
         <v>0.6018775544729295</v>
@@ -7241,7 +7244,7 @@
         <v>0.4509364578920367</v>
       </c>
       <c r="T12" s="2">
-        <v>-0.128997772606995</v>
+        <v>-0.1290250505123238</v>
       </c>
       <c r="U12" s="2">
         <v>-0.2462754075621131</v>
@@ -7249,7 +7252,7 @@
     </row>
     <row r="13" spans="1:21">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" s="2">
         <v>0.6774842229672553</v>
@@ -7306,7 +7309,7 @@
         <v>0.4699504830762667</v>
       </c>
       <c r="T13" s="2">
-        <v>-0.1301171097783223</v>
+        <v>-0.1299454058009104</v>
       </c>
       <c r="U13" s="2">
         <v>-0.2573729833527058</v>
@@ -7314,7 +7317,7 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B14" s="2">
         <v>0.7107951348280582</v>
@@ -7371,7 +7374,7 @@
         <v>0.4367398812841394</v>
       </c>
       <c r="T14" s="2">
-        <v>-0.1399960256845093</v>
+        <v>-0.1397330377540217</v>
       </c>
       <c r="U14" s="2">
         <v>-0.289452800892835</v>
@@ -7379,7 +7382,7 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B15" s="2">
         <v>0.008720575418330557</v>
@@ -7436,7 +7439,7 @@
         <v>0.02748929588193674</v>
       </c>
       <c r="T15" s="2">
-        <v>0.1198458693796355</v>
+        <v>0.1202382146812478</v>
       </c>
       <c r="U15" s="2">
         <v>0.1676753538624426</v>
@@ -7444,7 +7447,7 @@
     </row>
     <row r="16" spans="1:21">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" s="2">
         <v>-0.04506667671579052</v>
@@ -7501,7 +7504,7 @@
         <v>-0.07907903964650614</v>
       </c>
       <c r="T16" s="2">
-        <v>0.1440231798102623</v>
+        <v>0.1438391416985031</v>
       </c>
       <c r="U16" s="2">
         <v>0.1159300913489198</v>
@@ -7509,7 +7512,7 @@
     </row>
     <row r="17" spans="1:21">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B17" s="2">
         <v>-0.09296776454437576</v>
@@ -7566,7 +7569,7 @@
         <v>-0.1366429986766272</v>
       </c>
       <c r="T17" s="2">
-        <v>0.2071043058025451</v>
+        <v>0.2065493697799801</v>
       </c>
       <c r="U17" s="2">
         <v>0.1097506514905035</v>
@@ -7574,7 +7577,7 @@
     </row>
     <row r="18" spans="1:21">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B18" s="2">
         <v>-0.06844342659119444</v>
@@ -7631,7 +7634,7 @@
         <v>-0.1731324640194044</v>
       </c>
       <c r="T18" s="2">
-        <v>0.229318943397713</v>
+        <v>0.2288143655682168</v>
       </c>
       <c r="U18" s="2">
         <v>0.09815132479134112</v>
@@ -7639,7 +7642,7 @@
     </row>
     <row r="19" spans="1:21">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B19" s="2">
         <v>0.3345626558024875</v>
@@ -7696,7 +7699,7 @@
         <v>1</v>
       </c>
       <c r="T19" s="2">
-        <v>-0.04264386944636318</v>
+        <v>-0.04175554167041785</v>
       </c>
       <c r="U19" s="2">
         <v>-0.02834016125905013</v>
@@ -7704,72 +7707,72 @@
     </row>
     <row r="20" spans="1:21">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20" s="2">
-        <v>-0.174051117222249</v>
+        <v>-0.1739314254767215</v>
       </c>
       <c r="C20" s="2">
-        <v>-0.2043652910733721</v>
+        <v>-0.2042294230916621</v>
       </c>
       <c r="D20" s="2">
-        <v>-0.1704806329162473</v>
+        <v>-0.1703430425228417</v>
       </c>
       <c r="E20" s="2">
-        <v>-0.218902768171632</v>
+        <v>-0.2186278527143195</v>
       </c>
       <c r="F20" s="2">
-        <v>-0.1501815314812725</v>
+        <v>-0.1501580296443984</v>
       </c>
       <c r="G20" s="2">
-        <v>-0.2150169267444245</v>
+        <v>-0.2149361341923391</v>
       </c>
       <c r="H20" s="2">
-        <v>-0.1688066755923048</v>
+        <v>-0.1685415940436771</v>
       </c>
       <c r="I20" s="2">
-        <v>-0.1743342388622958</v>
+        <v>-0.174094512729544</v>
       </c>
       <c r="J20" s="2">
-        <v>-0.1883349938814105</v>
+        <v>-0.1880768705967719</v>
       </c>
       <c r="K20" s="2">
-        <v>-0.1638422366177304</v>
+        <v>-0.1636985791053485</v>
       </c>
       <c r="L20" s="2">
-        <v>-0.128997772606995</v>
+        <v>-0.1290250505123238</v>
       </c>
       <c r="M20" s="2">
-        <v>-0.1301171097783223</v>
+        <v>-0.1299454058009104</v>
       </c>
       <c r="N20" s="2">
-        <v>-0.1399960256845093</v>
+        <v>-0.1397330377540217</v>
       </c>
       <c r="O20" s="2">
-        <v>0.1198458693796355</v>
+        <v>0.1202382146812478</v>
       </c>
       <c r="P20" s="2">
-        <v>0.1440231798102623</v>
+        <v>0.1438391416985031</v>
       </c>
       <c r="Q20" s="2">
-        <v>0.2071043058025451</v>
+        <v>0.2065493697799801</v>
       </c>
       <c r="R20" s="2">
-        <v>0.229318943397713</v>
+        <v>0.2288143655682168</v>
       </c>
       <c r="S20" s="2">
-        <v>-0.04264386944636318</v>
+        <v>-0.04175554167041785</v>
       </c>
       <c r="T20" s="2">
         <v>1</v>
       </c>
       <c r="U20" s="2">
-        <v>0.3258666629084061</v>
+        <v>0.326092761371734</v>
       </c>
     </row>
     <row r="21" spans="1:21">
       <c r="A21" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B21" s="2">
         <v>-0.3189467570670729</v>
@@ -7826,7 +7829,7 @@
         <v>-0.02834016125905013</v>
       </c>
       <c r="T21" s="2">
-        <v>0.3258666629084061</v>
+        <v>0.326092761371734</v>
       </c>
       <c r="U21" s="2">
         <v>1</v>
@@ -7859,67 +7862,67 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -9969,7 +9972,7 @@
         <v>0.114441031439952</v>
       </c>
       <c r="T60" s="1">
-        <v>0.387343704164353</v>
+        <v>0.360568548928748</v>
       </c>
       <c r="U60" s="1">
         <v>0.1310376608210853</v>
@@ -10016,7 +10019,7 @@
         <v>-0.007012076902771613</v>
       </c>
       <c r="T61" s="1">
-        <v>0.270551158962796</v>
+        <v>0.2458442540980899</v>
       </c>
       <c r="U61" s="1">
         <v>0.161467777309896</v>
@@ -10063,7 +10066,7 @@
         <v>0.2167979084691873</v>
       </c>
       <c r="T62" s="1">
-        <v>0.2721620549849582</v>
+        <v>0.2474246149759063</v>
       </c>
       <c r="U62" s="1">
         <v>0.03638357221620847</v>
@@ -10110,7 +10113,7 @@
         <v>0.244290289144139</v>
       </c>
       <c r="T63" s="1">
-        <v>0.1676447285297988</v>
+        <v>0.1447958890516232</v>
       </c>
       <c r="U63" s="1">
         <v>0.09851495423013734</v>
@@ -10157,7 +10160,7 @@
         <v>0.09159538414072155</v>
       </c>
       <c r="T64" s="1">
-        <v>0.3780764467840105</v>
+        <v>0.3514658863535187</v>
       </c>
       <c r="U64" s="1">
         <v>0.1937111709771338</v>
@@ -10213,7 +10216,7 @@
         <v>0.08182536785920025</v>
       </c>
       <c r="T65" s="1">
-        <v>0.2588299653987005</v>
+        <v>0.2343302510651173</v>
       </c>
       <c r="U65" s="1">
         <v>0.1255559253081009</v>
@@ -10278,7 +10281,7 @@
         <v>-0.04096829428187165</v>
       </c>
       <c r="T66" s="1">
-        <v>0.1654034322636335</v>
+        <v>0.1425892911874969</v>
       </c>
       <c r="U66" s="1">
         <v>0.04638949678406745</v>
@@ -10343,7 +10346,7 @@
         <v>0.02776567334419311</v>
       </c>
       <c r="T67" s="1">
-        <v>0.2346916383378714</v>
+        <v>0.2106393875606847</v>
       </c>
       <c r="U67" s="1">
         <v>0.1623855637084952</v>
@@ -10408,7 +10411,7 @@
         <v>0.03848613775652554</v>
       </c>
       <c r="T68" s="1">
-        <v>0.3820647673977888</v>
+        <v>0.3553887917639569</v>
       </c>
       <c r="U68" s="1">
         <v>0.2237107309431685</v>
@@ -10473,7 +10476,7 @@
         <v>0.1276748696036625</v>
       </c>
       <c r="T69" s="1">
-        <v>0.004254001497079329</v>
+        <v>-0.01564863770526348</v>
       </c>
       <c r="U69" s="1">
         <v>0.05165178257412517</v>
@@ -10538,7 +10541,7 @@
         <v>0.148429225586286</v>
       </c>
       <c r="T70" s="1">
-        <v>0.2014488770847589</v>
+        <v>0.1779920161113211</v>
       </c>
       <c r="U70" s="1">
         <v>0.1546065829226049</v>
@@ -10603,7 +10606,7 @@
         <v>0.1676519709923268</v>
       </c>
       <c r="T71" s="1">
-        <v>0.3370405961595766</v>
+        <v>0.3111535854338559</v>
       </c>
       <c r="U71" s="1">
         <v>0.1141360620278205</v>
@@ -10668,7 +10671,7 @@
         <v>0.02783534871878568</v>
       </c>
       <c r="T72" s="1">
-        <v>0.3310926548904642</v>
+        <v>0.3053168826726125</v>
       </c>
       <c r="U72" s="1">
         <v>0.1769377219395731</v>
@@ -10733,7 +10736,7 @@
         <v>-0.2540204455798922</v>
       </c>
       <c r="T73" s="1">
-        <v>0.4757118929289581</v>
+        <v>0.4473860244258341</v>
       </c>
       <c r="U73" s="1">
         <v>0.1047056287822092</v>
@@ -10798,7 +10801,7 @@
         <v>0.1866230867432503</v>
       </c>
       <c r="T74" s="1">
-        <v>0.09183213197226991</v>
+        <v>0.07034124641177053</v>
       </c>
       <c r="U74" s="1">
         <v>0.05822630743064416</v>
@@ -10863,7 +10866,7 @@
         <v>0.1713618501012419</v>
       </c>
       <c r="T75" s="1">
-        <v>0.1784336327060614</v>
+        <v>0.1553882428188906</v>
       </c>
       <c r="U75" s="1">
         <v>0.4121585765933322</v>
@@ -10928,7 +10931,7 @@
         <v>-0.1229703963432026</v>
       </c>
       <c r="T76" s="1">
-        <v>0.2233807163083363</v>
+        <v>0.1995150727615422</v>
       </c>
       <c r="U76" s="1">
         <v>0.06966189995986682</v>
@@ -10993,7 +10996,7 @@
         <v>0.2469490988133209</v>
       </c>
       <c r="T77" s="1">
-        <v>0.3126907745054128</v>
+        <v>0.2872336313478705</v>
       </c>
       <c r="U77" s="1">
         <v>0.2180005329044024</v>
@@ -11058,7 +11061,7 @@
         <v>0.2583041205089083</v>
       </c>
       <c r="T78" s="1">
-        <v>0.2507563281135989</v>
+        <v>0.2264007568425903</v>
       </c>
       <c r="U78" s="1">
         <v>-0.06467542162413453</v>
@@ -11123,7 +11126,7 @@
         <v>0.1495893480776995</v>
       </c>
       <c r="T79" s="1">
-        <v>0.1426088650614679</v>
+        <v>0.1202028055395929</v>
       </c>
       <c r="U79" s="1">
         <v>0.04534130269148995</v>
@@ -11188,7 +11191,7 @@
         <v>0.2284582066899552</v>
       </c>
       <c r="T80" s="1">
-        <v>0.1899902817162331</v>
+        <v>0.1667367132302147</v>
       </c>
       <c r="U80" s="1">
         <v>0.1522427431081248</v>
@@ -11253,7 +11256,7 @@
         <v>0.1335395818680263</v>
       </c>
       <c r="T81" s="1">
-        <v>0.1717280286805771</v>
+        <v>0.1488039655039384</v>
       </c>
       <c r="U81" s="1">
         <v>0.06595336345353964</v>
@@ -11318,7 +11321,7 @@
         <v>0.2211813232949635</v>
       </c>
       <c r="T82" s="1">
-        <v>0.1892389178515672</v>
+        <v>0.1659925247753895</v>
       </c>
       <c r="U82" s="1">
         <v>0.07024792457026896</v>
@@ -11383,7 +11386,7 @@
         <v>-0.3379635137599797</v>
       </c>
       <c r="T83" s="1">
-        <v>0.2661437457652731</v>
+        <v>0.2415042677773638</v>
       </c>
       <c r="U83" s="1">
         <v>0.1329200456829667</v>
@@ -11448,7 +11451,7 @@
         <v>0.2530201431080041</v>
       </c>
       <c r="T84" s="1">
-        <v>-0.09830067300211665</v>
+        <v>-0.116333011440156</v>
       </c>
       <c r="U84" s="1">
         <v>-0.2955429528991608</v>
@@ -11513,7 +11516,7 @@
         <v>0.2314695344622091</v>
       </c>
       <c r="T85" s="1">
-        <v>0.1269471192238096</v>
+        <v>0.1048209760849741</v>
       </c>
       <c r="U85" s="1">
         <v>0.01317164508397006</v>
@@ -11578,7 +11581,7 @@
         <v>-0.1081347921032141</v>
       </c>
       <c r="T86" s="1">
-        <v>-0.0005285111951345289</v>
+        <v>-0.02035084892761807</v>
       </c>
       <c r="U86" s="1">
         <v>-0.001668320164379344</v>
@@ -11643,7 +11646,7 @@
         <v>0.022815637710347</v>
       </c>
       <c r="T87" s="1">
-        <v>-0.0009835159038299457</v>
+        <v>-0.02079892408104578</v>
       </c>
       <c r="U87" s="1">
         <v>0.03874179160380198</v>
@@ -11708,7 +11711,7 @@
         <v>-0.07728855544097302</v>
       </c>
       <c r="T88" s="1">
-        <v>0.1823515002486349</v>
+        <v>0.159236376125423</v>
       </c>
       <c r="U88" s="1">
         <v>0.03846318136329407</v>
@@ -11773,7 +11776,7 @@
         <v>-0.09376587234938971</v>
       </c>
       <c r="T89" s="1">
-        <v>0.1908611997513623</v>
+        <v>0.1675876851674991</v>
       </c>
       <c r="U89" s="1">
         <v>-0.005066299511012229</v>
@@ -11838,7 +11841,7 @@
         <v>-0.2189811536430536</v>
       </c>
       <c r="T90" s="1">
-        <v>0.1814864069735014</v>
+        <v>0.158359175959248</v>
       </c>
       <c r="U90" s="1">
         <v>0.05204189027672923</v>
@@ -11903,7 +11906,7 @@
         <v>0.09039645666772</v>
       </c>
       <c r="T91" s="1">
-        <v>-0.1093636611773106</v>
+        <v>-0.1271954030893555</v>
       </c>
       <c r="U91" s="1">
         <v>0.0006120008988992343</v>
@@ -11968,7 +11971,7 @@
         <v>0.04490108284118799</v>
       </c>
       <c r="T92" s="1">
-        <v>0.07465006210143521</v>
+        <v>0.05347461934754372</v>
       </c>
       <c r="U92" s="1">
         <v>-0.02868830433155678</v>
@@ -12033,7 +12036,7 @@
         <v>-0.09522329020521325</v>
       </c>
       <c r="T93" s="1">
-        <v>-0.0735076934117832</v>
+        <v>-0.09198868633710544</v>
       </c>
       <c r="U93" s="1">
         <v>0.01657854798739899</v>
@@ -12098,7 +12101,7 @@
         <v>0.08208573088549209</v>
       </c>
       <c r="T94" s="1">
-        <v>0.05380704579521001</v>
+        <v>0.03299094936267055</v>
       </c>
       <c r="U94" s="1">
         <v>-0.04075160708600234</v>
@@ -12163,7 +12166,7 @@
         <v>0.02827927901716287</v>
       </c>
       <c r="T95" s="1">
-        <v>-0.06326240955208084</v>
+        <v>-0.08194179404721402</v>
       </c>
       <c r="U95" s="1">
         <v>-0.1553573054907049</v>
@@ -12228,7 +12231,7 @@
         <v>0.2963038566467555</v>
       </c>
       <c r="T96" s="1">
-        <v>-0.04553757230162414</v>
+        <v>-0.0645488729011473</v>
       </c>
       <c r="U96" s="1">
         <v>0.09794179650006218</v>
@@ -12293,7 +12296,7 @@
         <v>0.187245961069445</v>
       </c>
       <c r="T97" s="1">
-        <v>0.2650325770318311</v>
+        <v>0.2404178230944836</v>
       </c>
       <c r="U97" s="1">
         <v>0.2817522988442891</v>
@@ -12358,7 +12361,7 @@
         <v>-0.03723080438281368</v>
       </c>
       <c r="T98" s="1">
-        <v>-0.0356983420549325</v>
+        <v>-0.05487567191830456</v>
       </c>
       <c r="U98" s="1">
         <v>-0.1113620948080671</v>
@@ -12423,7 +12426,7 @@
         <v>0.1170369896310031</v>
       </c>
       <c r="T99" s="1">
-        <v>0.08901709739058838</v>
+        <v>0.06757803868203216</v>
       </c>
       <c r="U99" s="1">
         <v>0.1086013426297989</v>
@@ -12488,7 +12491,7 @@
         <v>0.1307363410026265</v>
       </c>
       <c r="T100" s="1">
-        <v>0.0609388795451038</v>
+        <v>0.0400118250300916</v>
       </c>
       <c r="U100" s="1">
         <v>0.06850885311364108</v>
@@ -12512,13 +12515,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:4">

</xml_diff>